<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-21 16:42 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="296">
   <si>
     <t>50001415-ZITRON PERU METRO DE LIMA  E05</t>
   </si>
@@ -154,7 +154,7 @@
     <t>Ingenieria Servicios:</t>
   </si>
   <si>
-    <t>Ingenieria electrica,Revisión tableros pruebas</t>
+    <t>Ingenieria electrica,Revisiónx tableros pruebas</t>
   </si>
   <si>
     <t>1213425187968716</t>
@@ -175,7 +175,7 @@
     <t>1213425187968717</t>
   </si>
   <si>
-    <t>Revisión tableros pruebas</t>
+    <t>Revisiónx tableros pruebas</t>
   </si>
   <si>
     <t>sergio saavedra fernandez</t>
@@ -187,7 +187,7 @@
     <t xml:space="preserve">Recepcion Tableros OT 4115 - 4116 - 4117 - 4118 </t>
   </si>
   <si>
-    <t>Ingenieria Servicios:,Embalaje</t>
+    <t>Ingenieria Servicios:,Embalaje,Coordinacion Entrega con Cliente</t>
   </si>
   <si>
     <t>Tarea en curso</t>
@@ -673,7 +673,7 @@
     <t>1213425187981415</t>
   </si>
   <si>
-    <t>Bodega:,Revisión tableros pruebas</t>
+    <t>Bodega:,Revisiónx tableros pruebas</t>
   </si>
   <si>
     <t>1213425187981416</t>
@@ -805,6 +805,9 @@
     <t>kpinto@zitron.com</t>
   </si>
   <si>
+    <t>RE-PINTADO,Revisiónx tableros pruebas</t>
+  </si>
+  <si>
     <t>Logistica:,Embalaje</t>
   </si>
   <si>
@@ -814,7 +817,7 @@
     <t>Embalaje</t>
   </si>
   <si>
-    <t>Coordinacion Entrega con Cliente,Revisión tableros pruebas</t>
+    <t>Coordinacion Entrega con Cliente,Revisiónx tableros pruebas</t>
   </si>
   <si>
     <t>Logistica:,PACKING LIST</t>
@@ -2002,7 +2005,7 @@
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46182.711985104164</v>
+        <v>46194.68600292824</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -5797,7 +5800,7 @@
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46181.69962024306</v>
+        <v>46194.685942372686</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5828,10 +5831,10 @@
         <v>258</v>
       </c>
       <c r="O73" s="9" t="s">
-        <v>203</v>
+        <v>264</v>
       </c>
       <c r="P73" s="9" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q73" s="8">
         <v>46160</v>
@@ -5851,7 +5854,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B74" s="5">
         <v>46077.794069456024</v>
@@ -5861,7 +5864,7 @@
         <v>46161.2503321875</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
@@ -5889,10 +5892,10 @@
         <v>258</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="Q74" s="5">
         <v>46161</v>
@@ -5912,7 +5915,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B75" s="8">
         <v>46077.79406971065</v>
@@ -5922,16 +5925,16 @@
         <v>46162.25043027778</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I75" s="8">
         <v>46162</v>
@@ -5952,10 +5955,10 @@
         <v>258</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q75" s="8">
         <v>46162</v>
@@ -5975,7 +5978,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B76" s="5">
         <v>46077.79407002315</v>
@@ -5985,16 +5988,16 @@
         <v>46164.250411307876</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I76" s="6"/>
       <c r="J76" s="5">
@@ -6013,10 +6016,10 @@
         <v>258</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="Q76" s="5">
         <v>46164</v>
@@ -6036,7 +6039,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B77" s="8">
         <v>46077.794070289354</v>
@@ -6046,7 +6049,7 @@
         <v>46092.562138657406</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>25</v>
@@ -6070,7 +6073,7 @@
         <v>26</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="P77" s="9" t="s">
         <v>26</v>
@@ -6083,7 +6086,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B78" s="5">
         <v>46077.794070578704</v>
@@ -6093,16 +6096,16 @@
         <v>46175.16763520833</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I78" s="5">
         <v>46167</v>
@@ -6120,13 +6123,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="Q78" s="5">
         <v>46167</v>
@@ -6146,7 +6149,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B79" s="8">
         <v>46077.794070856486</v>
@@ -6156,16 +6159,16 @@
         <v>46175.167637245366</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="9" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H79" s="9" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I79" s="8">
         <v>46167</v>
@@ -6183,13 +6186,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="Q79" s="8">
         <v>46167</v>
@@ -6209,7 +6212,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B80" s="5">
         <v>46092.542492141205</v>
@@ -6219,7 +6222,7 @@
         <v>46092.56213928241</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>25</v>
@@ -6243,7 +6246,7 @@
         <v>26</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>26</v>
@@ -6262,7 +6265,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B81" s="8">
         <v>46092.542531493054</v>
@@ -6272,7 +6275,7 @@
         <v>46175.16778667824</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
@@ -6299,13 +6302,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="9" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="Q81" s="8">
         <v>46167</v>
@@ -6325,7 +6328,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B82" s="5">
         <v>46092.542669120376</v>
@@ -6335,7 +6338,7 @@
         <v>46185.18163831018</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
@@ -6362,13 +6365,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="Q82" s="5">
         <v>46176</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-22 13:21 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -5753,7 +5753,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46092.56213851852</v>
+        <v>46195.505563136576</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>258</v>
@@ -5859,9 +5859,11 @@
       <c r="B74" s="5">
         <v>46077.794069456024</v>
       </c>
-      <c r="C74" s="6"/>
+      <c r="C74" s="5">
+        <v>46195.50555773148</v>
+      </c>
       <c r="D74" s="5">
-        <v>46161.2503321875</v>
+        <v>46195.50557284722</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5904,13 +5906,13 @@
         <v>46161</v>
       </c>
       <c r="S74" s="6">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="T74" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U74" s="10" t="s">
-        <v>117</v>
+      <c r="U74" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -5920,9 +5922,11 @@
       <c r="B75" s="8">
         <v>46077.79406971065</v>
       </c>
-      <c r="C75" s="9"/>
+      <c r="C75" s="8">
+        <v>46195.50534894676</v>
+      </c>
       <c r="D75" s="8">
-        <v>46162.25043027778</v>
+        <v>46195.50557208333</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>271</v>
@@ -5967,13 +5971,13 @@
         <v>46162</v>
       </c>
       <c r="S75" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T75" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U75" s="10" t="s">
-        <v>117</v>
+      <c r="U75" s="12" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -5983,9 +5987,11 @@
       <c r="B76" s="5">
         <v>46077.79407002315</v>
       </c>
-      <c r="C76" s="6"/>
+      <c r="C76" s="5">
+        <v>46195.50540096065</v>
+      </c>
       <c r="D76" s="5">
-        <v>46164.250411307876</v>
+        <v>46195.505416203705</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>276</v>
@@ -6028,13 +6034,13 @@
         <v>46164</v>
       </c>
       <c r="S76" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T76" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U76" s="10" t="s">
-        <v>117</v>
+      <c r="U76" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -6093,7 +6099,7 @@
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46175.16763520833</v>
+        <v>46195.505419849535</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>282</v>
@@ -6143,8 +6149,8 @@
       <c r="T78" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U78" s="10" t="s">
-        <v>117</v>
+      <c r="U78" s="12" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
@@ -6156,7 +6162,7 @@
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46175.167637245366</v>
+        <v>46195.50541993056</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>286</v>
@@ -6206,8 +6212,8 @@
       <c r="T79" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U79" s="10" t="s">
-        <v>117</v>
+      <c r="U79" s="12" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
@@ -6272,7 +6278,7 @@
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46175.16778667824</v>
+        <v>46195.505421145834</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>292</v>
@@ -6322,8 +6328,8 @@
       <c r="T81" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U81" s="10" t="s">
-        <v>117</v>
+      <c r="U81" s="12" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-23 18:28 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -2948,7 +2948,7 @@
         <v>46175.58050744213</v>
       </c>
       <c r="D27" s="8">
-        <v>46175.58051010416</v>
+        <v>46196.708100289354</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>106</v>
@@ -2993,11 +2993,9 @@
       <c r="B28" s="5">
         <v>46077.794068773146</v>
       </c>
-      <c r="C28" s="5">
-        <v>46094.72648195602</v>
-      </c>
+      <c r="C28" s="6"/>
       <c r="D28" s="5">
-        <v>46106.16592788194</v>
+        <v>46196.70809677083</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>109</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-23 19:48 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="296">
   <si>
     <t>50001415-ZITRON PERU METRO DE LIMA  E05</t>
   </si>
@@ -190,151 +190,151 @@
     <t>Ingenieria Servicios:,Embalaje,Coordinacion Entrega con Cliente</t>
   </si>
   <si>
+    <t>1213425187968718</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete,Ingenieria Basica Alabes,Analisis de costeo</t>
+  </si>
+  <si>
+    <t>1213425187968719</t>
+  </si>
+  <si>
+    <t>Ingenieria Basica Motor</t>
+  </si>
+  <si>
+    <t>DAVID BLAZQUEZ</t>
+  </si>
+  <si>
+    <t>dbserrano@zitron.com</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
+  </si>
+  <si>
+    <t>1213425187968720</t>
+  </si>
+  <si>
+    <t>Ingenieria Basica Alabes</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta alabes</t>
+  </si>
+  <si>
+    <t>1213425187968721</t>
+  </si>
+  <si>
+    <t>Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta rodete</t>
+  </si>
+  <si>
+    <t>1213425187968722</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta compras a codigo // aprovisionamiento,Propuesta Sensores,Propuesta Fabricacion Externa,Planos preliminar</t>
+  </si>
+  <si>
+    <t>1213425187968723</t>
+  </si>
+  <si>
+    <t>Analisis de costeo</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete,Ingenieria Basica Alabes</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:,Costos</t>
+  </si>
+  <si>
+    <t>1213425187968724</t>
+  </si>
+  <si>
+    <t>Propuesta compras:</t>
+  </si>
+  <si>
+    <t>propuesta motor,propuesta tableros,propuesta tableros,propuesta rodete,propuesta alabes,Propuesta Sensores,propuesta alabes</t>
+  </si>
+  <si>
+    <t>1213425187968726</t>
+  </si>
+  <si>
+    <t>propuesta motor</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC motor</t>
+  </si>
+  <si>
+    <t>1213425187968725</t>
+  </si>
+  <si>
+    <t>propuesta alabes</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Alabe</t>
+  </si>
+  <si>
+    <t>1213425187968728</t>
+  </si>
+  <si>
+    <t>propuesta rodete</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Rodete</t>
+  </si>
+  <si>
+    <t>1213425187968727</t>
+  </si>
+  <si>
+    <t>propuesta tableros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta compras:,Generación OC Tableros OT 4115 - 4116 - 4117 - 4118 </t>
+  </si>
+  <si>
+    <t>1213425187968729</t>
+  </si>
+  <si>
+    <t>propuesta compras a codigo // aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Generación OC materiales</t>
+  </si>
+  <si>
+    <t>1213435315647799</t>
+  </si>
+  <si>
+    <t>Propuesta Sensores</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generacion OC Sensor</t>
+  </si>
+  <si>
+    <t>1213435315647800</t>
+  </si>
+  <si>
+    <t>Propuesta Fabricacion Externa</t>
+  </si>
+  <si>
+    <t>Generacion OC Fabricacion Externa</t>
+  </si>
+  <si>
+    <t>1213425187968730</t>
+  </si>
+  <si>
+    <t>Compras:</t>
+  </si>
+  <si>
+    <t>Alabe,Tablero OT 4115 - 4116 - 4117 - 4118 ,Rodete,Motor,Materiales a codigo // compras locales aprovisionamientomiento:,Sensores,Fabricacion Externa</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1213425187968718</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete,Ingenieria Basica Alabes,Analisis de costeo</t>
-  </si>
-  <si>
-    <t>1213425187968719</t>
-  </si>
-  <si>
-    <t>Ingenieria Basica Motor</t>
-  </si>
-  <si>
-    <t>DAVID BLAZQUEZ</t>
-  </si>
-  <si>
-    <t>dbserrano@zitron.com</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
-  </si>
-  <si>
-    <t>1213425187968720</t>
-  </si>
-  <si>
-    <t>Ingenieria Basica Alabes</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta alabes</t>
-  </si>
-  <si>
-    <t>1213425187968721</t>
-  </si>
-  <si>
-    <t>Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta rodete</t>
-  </si>
-  <si>
-    <t>1213425187968722</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta compras a codigo // aprovisionamiento,Propuesta Sensores,Propuesta Fabricacion Externa,Planos preliminar</t>
-  </si>
-  <si>
-    <t>1213425187968723</t>
-  </si>
-  <si>
-    <t>Analisis de costeo</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete,Ingenieria Basica Alabes</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:,Costos</t>
-  </si>
-  <si>
-    <t>1213425187968724</t>
-  </si>
-  <si>
-    <t>Propuesta compras:</t>
-  </si>
-  <si>
-    <t>propuesta motor,propuesta tableros,propuesta tableros,propuesta rodete,propuesta alabes,Propuesta Sensores,propuesta alabes</t>
-  </si>
-  <si>
-    <t>1213425187968726</t>
-  </si>
-  <si>
-    <t>propuesta motor</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC motor</t>
-  </si>
-  <si>
-    <t>1213425187968725</t>
-  </si>
-  <si>
-    <t>propuesta alabes</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Alabe</t>
-  </si>
-  <si>
-    <t>1213425187968728</t>
-  </si>
-  <si>
-    <t>propuesta rodete</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Rodete</t>
-  </si>
-  <si>
-    <t>1213425187968727</t>
-  </si>
-  <si>
-    <t>propuesta tableros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propuesta compras:,Generación OC Tableros OT 4115 - 4116 - 4117 - 4118 </t>
-  </si>
-  <si>
-    <t>1213425187968729</t>
-  </si>
-  <si>
-    <t>propuesta compras a codigo // aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Generación OC materiales</t>
-  </si>
-  <si>
-    <t>1213435315647799</t>
-  </si>
-  <si>
-    <t>Propuesta Sensores</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generacion OC Sensor</t>
-  </si>
-  <si>
-    <t>1213435315647800</t>
-  </si>
-  <si>
-    <t>Propuesta Fabricacion Externa</t>
-  </si>
-  <si>
-    <t>Generacion OC Fabricacion Externa</t>
-  </si>
-  <si>
-    <t>1213425187968730</t>
-  </si>
-  <si>
-    <t>Compras:</t>
-  </si>
-  <si>
-    <t>Alabe,Tablero OT 4115 - 4116 - 4117 - 4118 ,Rodete,Motor,Materiales a codigo // compras locales aprovisionamientomiento:,Sensores,Fabricacion Externa</t>
   </si>
   <si>
     <t>1213425187968731</t>
@@ -1891,9 +1891,11 @@
       <c r="B10" s="5">
         <v>46077.7940699537</v>
       </c>
-      <c r="C10" s="6"/>
+      <c r="C10" s="5">
+        <v>46196.78443082176</v>
+      </c>
       <c r="D10" s="5">
-        <v>46127.61337875</v>
+        <v>46196.78444497685</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -1927,9 +1929,13 @@
       </c>
       <c r="Q10" s="6"/>
       <c r="R10" s="6"/>
-      <c r="S10" s="6"/>
+      <c r="S10" s="6">
+        <v>1</v>
+      </c>
       <c r="T10" s="6"/>
-      <c r="U10" s="6"/>
+      <c r="U10" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
@@ -2003,9 +2009,11 @@
       <c r="B12" s="5">
         <v>46077.79407052083</v>
       </c>
-      <c r="C12" s="6"/>
+      <c r="C12" s="5">
+        <v>46196.7844127662</v>
+      </c>
       <c r="D12" s="5">
-        <v>46194.68600292824</v>
+        <v>46196.78442833333</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -2050,18 +2058,18 @@
         <v>46101</v>
       </c>
       <c r="S12" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T12" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U12" s="12" t="s">
-        <v>59</v>
+      <c r="U12" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="8">
         <v>46077.79407081018</v>
@@ -2073,7 +2081,7 @@
         <v>46108.78193280092</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>25</v>
@@ -2097,7 +2105,7 @@
         <v>26</v>
       </c>
       <c r="O13" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P13" s="9" t="s">
         <v>26</v>
@@ -2110,7 +2118,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B14" s="5">
         <v>46077.794067939816</v>
@@ -2122,16 +2130,16 @@
         <v>46093.75107269676</v>
       </c>
       <c r="E14" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="F14" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="I14" s="5">
         <v>45972</v>
@@ -2149,13 +2157,13 @@
         <v>26</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>41</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q14" s="5">
         <v>45972</v>
@@ -2175,7 +2183,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B15" s="8">
         <v>46077.79406833333</v>
@@ -2187,16 +2195,16 @@
         <v>46093.75110184027</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G15" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H15" s="9" t="s">
         <v>65</v>
-      </c>
-      <c r="H15" s="9" t="s">
-        <v>66</v>
       </c>
       <c r="I15" s="8">
         <v>45972</v>
@@ -2214,13 +2222,13 @@
         <v>26</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O15" s="9" t="s">
         <v>41</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Q15" s="8">
         <v>45972</v>
@@ -2240,7 +2248,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B16" s="5">
         <v>46077.79406863426</v>
@@ -2252,16 +2260,16 @@
         <v>46093.75114815972</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G16" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="I16" s="5">
         <v>45972</v>
@@ -2279,13 +2287,13 @@
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>41</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q16" s="5">
         <v>45972</v>
@@ -2305,7 +2313,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B17" s="8">
         <v>46077.7940689699</v>
@@ -2317,16 +2325,16 @@
         <v>46093.75116991898</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G17" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H17" s="9" t="s">
         <v>65</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>66</v>
       </c>
       <c r="I17" s="8">
         <v>45972</v>
@@ -2344,13 +2352,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O17" s="9" t="s">
         <v>41</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Q17" s="8">
         <v>45972</v>
@@ -2370,7 +2378,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B18" s="5">
         <v>46077.794069247684</v>
@@ -2382,16 +2390,16 @@
         <v>46093.75198266204</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G18" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H18" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="I18" s="5">
         <v>45972</v>
@@ -2409,13 +2417,13 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O18" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="P18" s="6" t="s">
         <v>79</v>
-      </c>
-      <c r="P18" s="6" t="s">
-        <v>80</v>
       </c>
       <c r="Q18" s="5">
         <v>45972</v>
@@ -2435,7 +2443,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B19" s="8">
         <v>46077.79406954861</v>
@@ -2447,7 +2455,7 @@
         <v>46132.82815025463</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>25</v>
@@ -2471,7 +2479,7 @@
         <v>26</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="P19" s="9" t="s">
         <v>26</v>
@@ -2484,7 +2492,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B20" s="5">
         <v>46077.79407017361</v>
@@ -2496,16 +2504,16 @@
         <v>46093.75213300926</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G20" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H20" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="I20" s="5">
         <v>45974</v>
@@ -2523,13 +2531,13 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="Q20" s="5">
         <v>45974</v>
@@ -2549,7 +2557,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B21" s="8">
         <v>46077.794069826385</v>
@@ -2561,16 +2569,16 @@
         <v>46093.75214115741</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G21" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H21" s="9" t="s">
         <v>65</v>
-      </c>
-      <c r="H21" s="9" t="s">
-        <v>66</v>
       </c>
       <c r="I21" s="8">
         <v>45981</v>
@@ -2588,13 +2596,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="Q21" s="8">
         <v>45981</v>
@@ -2614,7 +2622,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B22" s="5">
         <v>46077.79407089121</v>
@@ -2626,16 +2634,16 @@
         <v>46093.752320381944</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G22" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H22" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="I22" s="5">
         <v>45981</v>
@@ -2653,13 +2661,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="Q22" s="5">
         <v>45981</v>
@@ -2679,7 +2687,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B23" s="8">
         <v>46077.79407056713</v>
@@ -2691,16 +2699,16 @@
         <v>46093.87275758102</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H23" s="9" t="s">
         <v>65</v>
-      </c>
-      <c r="H23" s="9" t="s">
-        <v>66</v>
       </c>
       <c r="I23" s="8">
         <v>45975</v>
@@ -2718,13 +2726,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O23" s="9" t="s">
         <v>49</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="Q23" s="8">
         <v>45975</v>
@@ -2744,7 +2752,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B24" s="5">
         <v>46077.79406818287</v>
@@ -2756,16 +2764,16 @@
         <v>46093.752364050924</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H24" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="I24" s="5">
         <v>45981</v>
@@ -2783,13 +2791,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Q24" s="5">
         <v>45981</v>
@@ -2809,7 +2817,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B25" s="8">
         <v>46078.639615821754</v>
@@ -2821,16 +2829,16 @@
         <v>46093.75238938657</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H25" s="9" t="s">
         <v>65</v>
-      </c>
-      <c r="H25" s="9" t="s">
-        <v>66</v>
       </c>
       <c r="I25" s="8">
         <v>45981</v>
@@ -2848,13 +2856,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P25" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q25" s="8">
         <v>45981</v>
@@ -2874,7 +2882,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B26" s="5">
         <v>46078.63966699074</v>
@@ -2886,16 +2894,16 @@
         <v>46093.752569606484</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H26" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="I26" s="5">
         <v>45981</v>
@@ -2913,13 +2921,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="Q26" s="5">
         <v>45981</v>
@@ -2939,7 +2947,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B27" s="8">
         <v>46077.79406851852</v>
@@ -2948,10 +2956,10 @@
         <v>46175.58050744213</v>
       </c>
       <c r="D27" s="8">
-        <v>46196.708100289354</v>
+        <v>46196.81887502315</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>25</v>
@@ -2975,7 +2983,7 @@
         <v>26</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P27" s="9" t="s">
         <v>26</v>
@@ -2984,7 +2992,9 @@
       <c r="R27" s="9"/>
       <c r="S27" s="9"/>
       <c r="T27" s="9"/>
-      <c r="U27" s="9"/>
+      <c r="U27" s="12" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
@@ -2993,9 +3003,11 @@
       <c r="B28" s="5">
         <v>46077.794068773146</v>
       </c>
-      <c r="C28" s="6"/>
+      <c r="C28" s="5">
+        <v>46196.81885747685</v>
+      </c>
       <c r="D28" s="5">
-        <v>46196.70809677083</v>
+        <v>46196.81885899305</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>109</v>
@@ -3025,13 +3037,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O28" s="6" t="s">
         <v>112</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q28" s="5">
         <v>45985</v>
@@ -3093,7 +3105,7 @@
         <v>109</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="P29" s="9" t="s">
         <v>115</v>
@@ -3220,13 +3232,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O31" s="9" t="s">
         <v>123</v>
       </c>
       <c r="P31" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q31" s="8">
         <v>45979</v>
@@ -3288,7 +3300,7 @@
         <v>122</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="P32" s="6" t="s">
         <v>126</v>
@@ -3413,13 +3425,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>132</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q34" s="5">
         <v>45985</v>
@@ -3481,7 +3493,7 @@
         <v>131</v>
       </c>
       <c r="O35" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P35" s="9" t="s">
         <v>135</v>
@@ -3608,13 +3620,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O37" s="9" t="s">
         <v>141</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q37" s="8">
         <v>45978</v>
@@ -3676,7 +3688,7 @@
         <v>140</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>144</v>
@@ -3868,13 +3880,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O41" s="9" t="s">
         <v>155</v>
       </c>
       <c r="P41" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q41" s="8">
         <v>45985</v>
@@ -3906,7 +3918,7 @@
         <v>46094.73822020833</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
@@ -3936,7 +3948,7 @@
         <v>152</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>157</v>
@@ -4001,7 +4013,7 @@
         <v>152</v>
       </c>
       <c r="O43" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P43" s="9" t="s">
         <v>160</v>
@@ -4063,13 +4075,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>163</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q44" s="5">
         <v>45985</v>
@@ -4131,7 +4143,7 @@
         <v>162</v>
       </c>
       <c r="O45" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P45" s="9" t="s">
         <v>166</v>
@@ -4238,13 +4250,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O47" s="9" t="s">
         <v>174</v>
       </c>
       <c r="P47" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q47" s="8">
         <v>45985</v>
@@ -4276,7 +4288,7 @@
         <v>46099.53788506944</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
@@ -4306,7 +4318,7 @@
         <v>171</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P48" s="6" t="s">
         <v>176</v>
@@ -4475,7 +4487,7 @@
         <v>182</v>
       </c>
       <c r="O51" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P51" s="9" t="s">
         <v>188</v>
@@ -5798,7 +5810,7 @@
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46194.685942372686</v>
+        <v>46196.78443601852</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5846,8 +5858,8 @@
       <c r="T73" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U73" s="10" t="s">
-        <v>117</v>
+      <c r="U73" s="12" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5861,7 +5873,7 @@
         <v>46195.50555773148</v>
       </c>
       <c r="D74" s="5">
-        <v>46195.50557284722</v>
+        <v>46196.784421944445</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5975,7 +5987,7 @@
         <v>116</v>
       </c>
       <c r="U75" s="12" t="s">
-        <v>59</v>
+        <v>107</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -6148,7 +6160,7 @@
         <v>116</v>
       </c>
       <c r="U78" s="12" t="s">
-        <v>59</v>
+        <v>107</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
@@ -6211,7 +6223,7 @@
         <v>116</v>
       </c>
       <c r="U79" s="12" t="s">
-        <v>59</v>
+        <v>107</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
@@ -6327,7 +6339,7 @@
         <v>116</v>
       </c>
       <c r="U81" s="12" t="s">
-        <v>59</v>
+        <v>107</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-24 14:31 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="296">
   <si>
     <t>50001415-ZITRON PERU METRO DE LIMA  E05</t>
   </si>
@@ -5265,7 +5265,7 @@
         <v>46181.69465158565</v>
       </c>
       <c r="D64" s="5">
-        <v>46181.699838125</v>
+        <v>46197.58530666667</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>233</v>
@@ -5761,9 +5761,11 @@
       <c r="B72" s="5">
         <v>46077.79406888889</v>
       </c>
-      <c r="C72" s="6"/>
+      <c r="C72" s="5">
+        <v>46197.586652777776</v>
+      </c>
       <c r="D72" s="5">
-        <v>46195.505563136576</v>
+        <v>46197.58666969907</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>258</v>
@@ -5797,9 +5799,13 @@
       </c>
       <c r="Q72" s="6"/>
       <c r="R72" s="6"/>
-      <c r="S72" s="6"/>
+      <c r="S72" s="6">
+        <v>1</v>
+      </c>
       <c r="T72" s="6"/>
-      <c r="U72" s="6"/>
+      <c r="U72" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
@@ -5808,9 +5814,11 @@
       <c r="B73" s="8">
         <v>46077.79406920139</v>
       </c>
-      <c r="C73" s="9"/>
+      <c r="C73" s="8">
+        <v>46197.58663336806</v>
+      </c>
       <c r="D73" s="8">
-        <v>46196.78443601852</v>
+        <v>46197.586652858794</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5853,13 +5861,13 @@
         <v>46160</v>
       </c>
       <c r="S73" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T73" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U73" s="12" t="s">
-        <v>107</v>
+      <c r="U73" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5873,7 +5881,7 @@
         <v>46195.50555773148</v>
       </c>
       <c r="D74" s="5">
-        <v>46196.784421944445</v>
+        <v>46197.58665158565</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5921,8 +5929,8 @@
       <c r="T74" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U74" s="11" t="s">
-        <v>33</v>
+      <c r="U74" s="12" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-24 16:50 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -1525,13 +1525,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46077.79406804398</v>
+        <v>46077.627401377315</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.723517129634</v>
+        <v>46092.55685046296</v>
       </c>
       <c r="D4" s="5">
-        <v>46109.700906631944</v>
+        <v>46109.53423996527</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1574,13 +1574,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46077.794068449075</v>
+        <v>46077.6274017824</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.723485636576</v>
+        <v>46092.55681896991</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.877652152776</v>
+        <v>46133.71098548611</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1637,13 +1637,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46077.794068738425</v>
+        <v>46077.62740207176</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.72348622685</v>
+        <v>46092.55681956018</v>
       </c>
       <c r="D6" s="5">
-        <v>46092.723518032406</v>
+        <v>46092.55685136574</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1700,13 +1700,13 @@
         <v>38</v>
       </c>
       <c r="B7" s="8">
-        <v>46077.79406903935</v>
+        <v>46077.62740237269</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.72348670139</v>
+        <v>46092.55682003472</v>
       </c>
       <c r="D7" s="8">
-        <v>46092.72351797453</v>
+        <v>46092.55685130787</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>39</v>
@@ -1763,13 +1763,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46077.794069317126</v>
+        <v>46077.62740265046</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.72348717593</v>
+        <v>46092.55682050926</v>
       </c>
       <c r="D8" s="5">
-        <v>46093.75078916667</v>
+        <v>46093.584122500004</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -1826,13 +1826,13 @@
         <v>43</v>
       </c>
       <c r="B9" s="8">
-        <v>46077.79406961806</v>
+        <v>46077.62740295139</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.72348797454</v>
+        <v>46092.556821307866</v>
       </c>
       <c r="D9" s="8">
-        <v>46092.72351859954</v>
+        <v>46092.556851932866</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>44</v>
@@ -1889,13 +1889,13 @@
         <v>45</v>
       </c>
       <c r="B10" s="5">
-        <v>46077.7940699537</v>
+        <v>46077.62740328704</v>
       </c>
       <c r="C10" s="5">
-        <v>46196.78443082176</v>
+        <v>46196.61776415509</v>
       </c>
       <c r="D10" s="5">
-        <v>46196.78444497685</v>
+        <v>46196.61777831019</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -1942,13 +1942,13 @@
         <v>48</v>
       </c>
       <c r="B11" s="8">
-        <v>46077.79407024306</v>
+        <v>46077.62740357639</v>
       </c>
       <c r="C11" s="8">
-        <v>46093.86130311343</v>
+        <v>46093.69463644676</v>
       </c>
       <c r="D11" s="8">
-        <v>46093.86132113426</v>
+        <v>46093.69465446759</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>49</v>
@@ -2007,13 +2007,13 @@
         <v>53</v>
       </c>
       <c r="B12" s="5">
-        <v>46077.79407052083</v>
+        <v>46077.62740385417</v>
       </c>
       <c r="C12" s="5">
-        <v>46196.7844127662</v>
+        <v>46196.61774609954</v>
       </c>
       <c r="D12" s="5">
-        <v>46196.78442833333</v>
+        <v>46196.61776166667</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -2072,13 +2072,13 @@
         <v>59</v>
       </c>
       <c r="B13" s="8">
-        <v>46077.79407081018</v>
+        <v>46077.62740414352</v>
       </c>
       <c r="C13" s="8">
-        <v>46093.75198055556</v>
+        <v>46093.58531388889</v>
       </c>
       <c r="D13" s="8">
-        <v>46108.78193280092</v>
+        <v>46108.615266134264</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>60</v>
@@ -2121,13 +2121,13 @@
         <v>62</v>
       </c>
       <c r="B14" s="5">
-        <v>46077.794067939816</v>
+        <v>46077.627401273145</v>
       </c>
       <c r="C14" s="5">
-        <v>46093.751054803244</v>
+        <v>46093.58438813657</v>
       </c>
       <c r="D14" s="5">
-        <v>46093.75107269676</v>
+        <v>46093.58440603009</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>63</v>
@@ -2186,13 +2186,13 @@
         <v>67</v>
       </c>
       <c r="B15" s="8">
-        <v>46077.79406833333</v>
+        <v>46077.62740166667</v>
       </c>
       <c r="C15" s="8">
-        <v>46093.75108634259</v>
+        <v>46093.58441967593</v>
       </c>
       <c r="D15" s="8">
-        <v>46093.75110184027</v>
+        <v>46093.584435173616</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>68</v>
@@ -2251,13 +2251,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="5">
-        <v>46077.79406863426</v>
+        <v>46077.62740196759</v>
       </c>
       <c r="C16" s="5">
-        <v>46093.75113149306</v>
+        <v>46093.58446482639</v>
       </c>
       <c r="D16" s="5">
-        <v>46093.75114815972</v>
+        <v>46093.58448149306</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>71</v>
@@ -2316,13 +2316,13 @@
         <v>73</v>
       </c>
       <c r="B17" s="8">
-        <v>46077.7940689699</v>
+        <v>46077.627402303246</v>
       </c>
       <c r="C17" s="8">
-        <v>46093.75114832176</v>
+        <v>46093.584481655096</v>
       </c>
       <c r="D17" s="8">
-        <v>46093.75116991898</v>
+        <v>46093.584503252314</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>74</v>
@@ -2381,13 +2381,13 @@
         <v>76</v>
       </c>
       <c r="B18" s="5">
-        <v>46077.794069247684</v>
+        <v>46077.62740258102</v>
       </c>
       <c r="C18" s="5">
-        <v>46093.75196043981</v>
+        <v>46093.58529377315</v>
       </c>
       <c r="D18" s="5">
-        <v>46093.75198266204</v>
+        <v>46093.58531599537</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>77</v>
@@ -2446,13 +2446,13 @@
         <v>80</v>
       </c>
       <c r="B19" s="8">
-        <v>46077.79406954861</v>
+        <v>46077.627402881946</v>
       </c>
       <c r="C19" s="8">
-        <v>46093.87275760417</v>
+        <v>46093.7060909375</v>
       </c>
       <c r="D19" s="8">
-        <v>46132.82815025463</v>
+        <v>46132.66148358796</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>81</v>
@@ -2495,13 +2495,13 @@
         <v>83</v>
       </c>
       <c r="B20" s="5">
-        <v>46077.79407017361</v>
+        <v>46077.627403506944</v>
       </c>
       <c r="C20" s="5">
-        <v>46093.75210856482</v>
+        <v>46093.58544189815</v>
       </c>
       <c r="D20" s="5">
-        <v>46093.75213300926</v>
+        <v>46093.58546634259</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>84</v>
@@ -2560,13 +2560,13 @@
         <v>86</v>
       </c>
       <c r="B21" s="8">
-        <v>46077.794069826385</v>
+        <v>46077.62740315972</v>
       </c>
       <c r="C21" s="8">
-        <v>46093.75212193287</v>
+        <v>46093.585455266206</v>
       </c>
       <c r="D21" s="8">
-        <v>46093.75214115741</v>
+        <v>46093.58547449074</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>87</v>
@@ -2625,13 +2625,13 @@
         <v>89</v>
       </c>
       <c r="B22" s="5">
-        <v>46077.79407089121</v>
+        <v>46077.627404224535</v>
       </c>
       <c r="C22" s="5">
-        <v>46093.75230475694</v>
+        <v>46093.58563809028</v>
       </c>
       <c r="D22" s="5">
-        <v>46093.752320381944</v>
+        <v>46093.58565371528</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>90</v>
@@ -2690,13 +2690,13 @@
         <v>92</v>
       </c>
       <c r="B23" s="8">
-        <v>46077.79407056713</v>
+        <v>46077.627403900464</v>
       </c>
       <c r="C23" s="8">
-        <v>46093.87273884259</v>
+        <v>46093.706072175926</v>
       </c>
       <c r="D23" s="8">
-        <v>46093.87275758102</v>
+        <v>46093.70609091435</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>93</v>
@@ -2755,13 +2755,13 @@
         <v>95</v>
       </c>
       <c r="B24" s="5">
-        <v>46077.79406818287</v>
+        <v>46077.627401516205</v>
       </c>
       <c r="C24" s="5">
-        <v>46093.752348344904</v>
+        <v>46093.58568167824</v>
       </c>
       <c r="D24" s="5">
-        <v>46093.752364050924</v>
+        <v>46093.58569738426</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>96</v>
@@ -2820,13 +2820,13 @@
         <v>98</v>
       </c>
       <c r="B25" s="8">
-        <v>46078.639615821754</v>
+        <v>46078.4729491551</v>
       </c>
       <c r="C25" s="8">
-        <v>46093.75237274305</v>
+        <v>46093.58570607639</v>
       </c>
       <c r="D25" s="8">
-        <v>46093.75238938657</v>
+        <v>46093.58572271991</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>99</v>
@@ -2885,13 +2885,13 @@
         <v>101</v>
       </c>
       <c r="B26" s="5">
-        <v>46078.63966699074</v>
+        <v>46078.47300032407</v>
       </c>
       <c r="C26" s="5">
-        <v>46093.75254957176</v>
+        <v>46093.58588290509</v>
       </c>
       <c r="D26" s="5">
-        <v>46093.752569606484</v>
+        <v>46093.58590293981</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>102</v>
@@ -2950,13 +2950,13 @@
         <v>104</v>
       </c>
       <c r="B27" s="8">
-        <v>46077.79406851852</v>
+        <v>46077.62740185185</v>
       </c>
       <c r="C27" s="8">
-        <v>46175.58050744213</v>
+        <v>46175.413840775465</v>
       </c>
       <c r="D27" s="8">
-        <v>46196.81887502315</v>
+        <v>46196.65220835648</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>105</v>
@@ -3001,13 +3001,13 @@
         <v>108</v>
       </c>
       <c r="B28" s="5">
-        <v>46077.794068773146</v>
+        <v>46077.62740210648</v>
       </c>
       <c r="C28" s="5">
-        <v>46196.81885747685</v>
+        <v>46196.652190810186</v>
       </c>
       <c r="D28" s="5">
-        <v>46196.81885899305</v>
+        <v>46196.65219232639</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>109</v>
@@ -3066,13 +3066,13 @@
         <v>113</v>
       </c>
       <c r="B29" s="8">
-        <v>46077.794069027776</v>
+        <v>46077.62740236111</v>
       </c>
       <c r="C29" s="8">
-        <v>46094.72641315972</v>
+        <v>46094.559746493054</v>
       </c>
       <c r="D29" s="8">
-        <v>46094.726415</v>
+        <v>46094.55974833333</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>114</v>
@@ -3131,13 +3131,13 @@
         <v>118</v>
       </c>
       <c r="B30" s="5">
-        <v>46077.794069270836</v>
+        <v>46077.627402604165</v>
       </c>
       <c r="C30" s="5">
-        <v>46094.726466493055</v>
+        <v>46094.559799826384</v>
       </c>
       <c r="D30" s="5">
-        <v>46094.72646796296</v>
+        <v>46094.559801296295</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>119</v>
@@ -3196,13 +3196,13 @@
         <v>121</v>
       </c>
       <c r="B31" s="8">
-        <v>46077.794069537034</v>
+        <v>46077.62740287037</v>
       </c>
       <c r="C31" s="8">
-        <v>46174.63943520833</v>
+        <v>46174.472768541666</v>
       </c>
       <c r="D31" s="8">
-        <v>46181.69497460648</v>
+        <v>46181.528307939814</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>122</v>
@@ -3261,13 +3261,13 @@
         <v>124</v>
       </c>
       <c r="B32" s="5">
-        <v>46077.79406980324</v>
+        <v>46077.627403136576</v>
       </c>
       <c r="C32" s="5">
-        <v>46094.72762815972</v>
+        <v>46094.56096149306</v>
       </c>
       <c r="D32" s="5">
-        <v>46169.82887452546</v>
+        <v>46169.6622078588</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>125</v>
@@ -3326,13 +3326,13 @@
         <v>127</v>
       </c>
       <c r="B33" s="8">
-        <v>46077.794070081014</v>
+        <v>46077.62740341436</v>
       </c>
       <c r="C33" s="8">
-        <v>46174.638556192134</v>
+        <v>46174.47188952546</v>
       </c>
       <c r="D33" s="8">
-        <v>46174.63855820602</v>
+        <v>46174.47189153935</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>128</v>
@@ -3389,13 +3389,13 @@
         <v>130</v>
       </c>
       <c r="B34" s="5">
-        <v>46077.79407034723</v>
+        <v>46077.627403680555</v>
       </c>
       <c r="C34" s="5">
-        <v>46094.72978902778</v>
+        <v>46094.56312236111</v>
       </c>
       <c r="D34" s="5">
-        <v>46094.729805462965</v>
+        <v>46094.56313879629</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>131</v>
@@ -3454,13 +3454,13 @@
         <v>133</v>
       </c>
       <c r="B35" s="8">
-        <v>46077.794070625</v>
+        <v>46077.62740395834</v>
       </c>
       <c r="C35" s="8">
-        <v>46094.7287584375</v>
+        <v>46094.56209177083</v>
       </c>
       <c r="D35" s="8">
-        <v>46094.72876005787</v>
+        <v>46094.5620933912</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>134</v>
@@ -3519,13 +3519,13 @@
         <v>136</v>
       </c>
       <c r="B36" s="5">
-        <v>46077.79406800926</v>
+        <v>46077.627401342594</v>
       </c>
       <c r="C36" s="5">
-        <v>46094.729772708335</v>
+        <v>46094.56310604166</v>
       </c>
       <c r="D36" s="5">
-        <v>46094.729774259264</v>
+        <v>46094.56310759259</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>137</v>
@@ -3584,13 +3584,13 @@
         <v>139</v>
       </c>
       <c r="B37" s="8">
-        <v>46077.79406834491</v>
+        <v>46077.62740167824</v>
       </c>
       <c r="C37" s="8">
-        <v>46094.72519538194</v>
+        <v>46094.55852871528</v>
       </c>
       <c r="D37" s="8">
-        <v>46130.168979560185</v>
+        <v>46130.00231289351</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>140</v>
@@ -3649,13 +3649,13 @@
         <v>142</v>
       </c>
       <c r="B38" s="5">
-        <v>46077.79406859954</v>
+        <v>46077.62740193287</v>
       </c>
       <c r="C38" s="5">
-        <v>46094.72491252315</v>
+        <v>46094.55824585648</v>
       </c>
       <c r="D38" s="5">
-        <v>46094.72491472222</v>
+        <v>46094.55824805556</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>143</v>
@@ -3714,13 +3714,13 @@
         <v>145</v>
       </c>
       <c r="B39" s="8">
-        <v>46077.79406886574</v>
+        <v>46077.627402199076</v>
       </c>
       <c r="C39" s="8">
-        <v>46094.725131388885</v>
+        <v>46094.55846472223</v>
       </c>
       <c r="D39" s="8">
-        <v>46094.72513274306</v>
+        <v>46094.558466076385</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>146</v>
@@ -3779,13 +3779,13 @@
         <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46077.79406912037</v>
+        <v>46077.627402453705</v>
       </c>
       <c r="C40" s="5">
-        <v>46094.72518011574</v>
+        <v>46094.558513449076</v>
       </c>
       <c r="D40" s="5">
-        <v>46094.7251815162</v>
+        <v>46094.55851484954</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>149</v>
@@ -3844,13 +3844,13 @@
         <v>151</v>
       </c>
       <c r="B41" s="8">
-        <v>46077.79406935185</v>
+        <v>46077.62740268519</v>
       </c>
       <c r="C41" s="8">
-        <v>46094.73862138889</v>
+        <v>46094.571954722225</v>
       </c>
       <c r="D41" s="8">
-        <v>46100.88799495371</v>
+        <v>46100.721328287036</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>152</v>
@@ -3909,13 +3909,13 @@
         <v>156</v>
       </c>
       <c r="B42" s="5">
-        <v>46077.79406958334</v>
+        <v>46077.62740291667</v>
       </c>
       <c r="C42" s="5">
-        <v>46094.73713944445</v>
+        <v>46094.57047277778</v>
       </c>
       <c r="D42" s="5">
-        <v>46094.73822020833</v>
+        <v>46094.57155354167</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>97</v>
@@ -3974,13 +3974,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46077.794069814816</v>
+        <v>46077.627403148144</v>
       </c>
       <c r="C43" s="8">
-        <v>46094.73860646991</v>
+        <v>46094.57193980324</v>
       </c>
       <c r="D43" s="8">
-        <v>46094.73860788194</v>
+        <v>46094.57194121528</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -4039,13 +4039,13 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46078.63983429398</v>
+        <v>46078.473167627315</v>
       </c>
       <c r="C44" s="5">
-        <v>46099.856573240744</v>
+        <v>46099.68990657407</v>
       </c>
       <c r="D44" s="5">
-        <v>46099.856649340276</v>
+        <v>46099.68998267361</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4104,13 +4104,13 @@
         <v>164</v>
       </c>
       <c r="B45" s="8">
-        <v>46078.63989878472</v>
+        <v>46078.473232118056</v>
       </c>
       <c r="C45" s="8">
-        <v>46099.856473287036</v>
+        <v>46099.68980662037</v>
       </c>
       <c r="D45" s="8">
-        <v>46099.85647474537</v>
+        <v>46099.68980807871</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>165</v>
@@ -4159,13 +4159,13 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46078.63997798611</v>
+        <v>46078.473311319445</v>
       </c>
       <c r="C46" s="5">
-        <v>46099.85655642361</v>
+        <v>46099.68988975695</v>
       </c>
       <c r="D46" s="5">
-        <v>46099.85655795139</v>
+        <v>46099.689891284725</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4214,13 +4214,13 @@
         <v>170</v>
       </c>
       <c r="B47" s="8">
-        <v>46078.637812500005</v>
+        <v>46078.47114583333</v>
       </c>
       <c r="C47" s="8">
-        <v>46099.838434375</v>
+        <v>46099.671767708336</v>
       </c>
       <c r="D47" s="8">
-        <v>46121.20616592593</v>
+        <v>46121.03949925926</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>171</v>
@@ -4279,13 +4279,13 @@
         <v>175</v>
       </c>
       <c r="B48" s="5">
-        <v>46078.63791627315</v>
+        <v>46078.47124960648</v>
       </c>
       <c r="C48" s="5">
-        <v>46094.75383356481</v>
+        <v>46094.58716689815</v>
       </c>
       <c r="D48" s="5">
-        <v>46099.53788506944</v>
+        <v>46099.37121840278</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>103</v>
@@ -4340,13 +4340,13 @@
         <v>177</v>
       </c>
       <c r="B49" s="8">
-        <v>46078.63808261574</v>
+        <v>46078.471415949076</v>
       </c>
       <c r="C49" s="8">
-        <v>46099.838418252315</v>
+        <v>46099.67175158564</v>
       </c>
       <c r="D49" s="8">
-        <v>46099.84112896991</v>
+        <v>46099.67446230324</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>178</v>
@@ -4395,13 +4395,13 @@
         <v>181</v>
       </c>
       <c r="B50" s="5">
-        <v>46077.79407005787</v>
+        <v>46077.627403391205</v>
       </c>
       <c r="C50" s="5">
-        <v>46181.69487049768</v>
+        <v>46181.52820383102</v>
       </c>
       <c r="D50" s="5">
-        <v>46181.69488571759</v>
+        <v>46181.528219050924</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>182</v>
@@ -4448,13 +4448,13 @@
         <v>184</v>
       </c>
       <c r="B51" s="8">
-        <v>46077.794070289354</v>
+        <v>46077.62740362268</v>
       </c>
       <c r="C51" s="8">
-        <v>46093.76443008102</v>
+        <v>46093.59776341435</v>
       </c>
       <c r="D51" s="8">
-        <v>46093.76444804398</v>
+        <v>46093.59778137731</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>185</v>
@@ -4513,13 +4513,13 @@
         <v>189</v>
       </c>
       <c r="B52" s="5">
-        <v>46077.79406836806</v>
+        <v>46077.62740170139</v>
       </c>
       <c r="C52" s="5">
-        <v>46097.53332418982</v>
+        <v>46097.36665752315</v>
       </c>
       <c r="D52" s="5">
-        <v>46097.53334462963</v>
+        <v>46097.366677962964</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>190</v>
@@ -4578,13 +4578,13 @@
         <v>195</v>
       </c>
       <c r="B53" s="8">
-        <v>46092.48310565972</v>
+        <v>46092.31643899306</v>
       </c>
       <c r="C53" s="8">
-        <v>46097.533368495366</v>
+        <v>46097.36670182871</v>
       </c>
       <c r="D53" s="8">
-        <v>46097.53338633102</v>
+        <v>46097.36671966435</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>196</v>
@@ -4641,13 +4641,13 @@
         <v>198</v>
       </c>
       <c r="B54" s="5">
-        <v>46092.48319758102</v>
+        <v>46092.31653091435</v>
       </c>
       <c r="C54" s="5">
-        <v>46181.69336679398</v>
+        <v>46181.52670012732</v>
       </c>
       <c r="D54" s="5">
-        <v>46181.694910763894</v>
+        <v>46181.52824409722</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>199</v>
@@ -4706,13 +4706,13 @@
         <v>204</v>
       </c>
       <c r="B55" s="8">
-        <v>46079.615135416665</v>
+        <v>46079.44846875</v>
       </c>
       <c r="C55" s="8">
-        <v>46100.46822152778</v>
+        <v>46100.301554861115</v>
       </c>
       <c r="D55" s="8">
-        <v>46135.75940972222</v>
+        <v>46135.59274305556</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>205</v>
@@ -4755,13 +4755,13 @@
         <v>207</v>
       </c>
       <c r="B56" s="5">
-        <v>46078.74941568287</v>
+        <v>46078.582749016205</v>
       </c>
       <c r="C56" s="5">
-        <v>46100.46820005787</v>
+        <v>46100.301533391204</v>
       </c>
       <c r="D56" s="5">
-        <v>46122.193223229166</v>
+        <v>46122.0265565625</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>206</v>
@@ -4820,13 +4820,13 @@
         <v>211</v>
       </c>
       <c r="B57" s="8">
-        <v>46077.794070601856</v>
+        <v>46077.627403935185</v>
       </c>
       <c r="C57" s="8">
-        <v>46181.69656722222</v>
+        <v>46181.52990055556</v>
       </c>
       <c r="D57" s="8">
-        <v>46181.880506643516</v>
+        <v>46181.71383997685</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>212</v>
@@ -4869,13 +4869,13 @@
         <v>214</v>
       </c>
       <c r="B58" s="5">
-        <v>46077.79407089121</v>
+        <v>46077.627404224535</v>
       </c>
       <c r="C58" s="5">
-        <v>46099.60850569444</v>
+        <v>46099.44183902778</v>
       </c>
       <c r="D58" s="5">
-        <v>46099.60852430556</v>
+        <v>46099.441857638885</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>215</v>
@@ -4934,13 +4934,13 @@
         <v>219</v>
       </c>
       <c r="B59" s="8">
-        <v>46077.79406847223</v>
+        <v>46077.627401805556</v>
       </c>
       <c r="C59" s="8">
-        <v>46181.696550555556</v>
+        <v>46181.529883888885</v>
       </c>
       <c r="D59" s="8">
-        <v>46181.69656733796</v>
+        <v>46181.529900671296</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>57</v>
@@ -4999,13 +4999,13 @@
         <v>221</v>
       </c>
       <c r="B60" s="5">
-        <v>46077.79406880787</v>
+        <v>46077.6274021412</v>
       </c>
       <c r="C60" s="5">
-        <v>46099.608517685185</v>
+        <v>46099.44185101852</v>
       </c>
       <c r="D60" s="5">
-        <v>46108.14717359954</v>
+        <v>46107.98050693287</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>222</v>
@@ -5064,13 +5064,13 @@
         <v>224</v>
       </c>
       <c r="B61" s="8">
-        <v>46077.79406909722</v>
+        <v>46077.62740243056</v>
       </c>
       <c r="C61" s="8">
-        <v>46099.6085555787</v>
+        <v>46099.44188891204</v>
       </c>
       <c r="D61" s="8">
-        <v>46134.20545793981</v>
+        <v>46134.03879127315</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>225</v>
@@ -5129,13 +5129,13 @@
         <v>227</v>
       </c>
       <c r="B62" s="5">
-        <v>46078.64006494213</v>
+        <v>46078.47339827546</v>
       </c>
       <c r="C62" s="5">
-        <v>46099.856724178244</v>
+        <v>46099.69005751157</v>
       </c>
       <c r="D62" s="5">
-        <v>46099.856817928245</v>
+        <v>46099.69015126157</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>228</v>
@@ -5194,13 +5194,13 @@
         <v>230</v>
       </c>
       <c r="B63" s="8">
-        <v>46078.63913549768</v>
+        <v>46078.47246883102</v>
       </c>
       <c r="C63" s="8">
-        <v>46120.627901562504</v>
+        <v>46120.46123489583</v>
       </c>
       <c r="D63" s="8">
-        <v>46120.62792370371</v>
+        <v>46120.46125703704</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>231</v>
@@ -5259,13 +5259,13 @@
         <v>232</v>
       </c>
       <c r="B64" s="5">
-        <v>46077.794069386575</v>
+        <v>46077.62740271991</v>
       </c>
       <c r="C64" s="5">
-        <v>46181.69465158565</v>
+        <v>46181.52798491898</v>
       </c>
       <c r="D64" s="5">
-        <v>46197.58530666667</v>
+        <v>46197.41864</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>233</v>
@@ -5308,13 +5308,13 @@
         <v>235</v>
       </c>
       <c r="B65" s="8">
-        <v>46077.79406965278</v>
+        <v>46077.62740298611</v>
       </c>
       <c r="C65" s="8">
-        <v>46140.56150293982</v>
+        <v>46140.394836273146</v>
       </c>
       <c r="D65" s="8">
-        <v>46181.69470346065</v>
+        <v>46181.528036793985</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>236</v>
@@ -5373,13 +5373,13 @@
         <v>240</v>
       </c>
       <c r="B66" s="5">
-        <v>46077.79406990741</v>
+        <v>46077.62740324074</v>
       </c>
       <c r="C66" s="5">
-        <v>46181.69321660879</v>
+        <v>46181.52654994213</v>
       </c>
       <c r="D66" s="5">
-        <v>46181.69470399305</v>
+        <v>46181.52803732639</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>241</v>
@@ -5438,13 +5438,13 @@
         <v>244</v>
       </c>
       <c r="B67" s="8">
-        <v>46077.79407016204</v>
+        <v>46077.62740349537</v>
       </c>
       <c r="C67" s="8">
-        <v>46113.56087353009</v>
+        <v>46113.39420686342</v>
       </c>
       <c r="D67" s="8">
-        <v>46140.561511990745</v>
+        <v>46140.394845324074</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>245</v>
@@ -5503,13 +5503,13 @@
         <v>247</v>
       </c>
       <c r="B68" s="5">
-        <v>46077.79407042824</v>
+        <v>46077.62740376157</v>
       </c>
       <c r="C68" s="5">
-        <v>46181.69323842593</v>
+        <v>46181.526571759256</v>
       </c>
       <c r="D68" s="5">
-        <v>46181.694704525464</v>
+        <v>46181.52803785879</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>248</v>
@@ -5568,13 +5568,13 @@
         <v>250</v>
       </c>
       <c r="B69" s="8">
-        <v>46078.640146562495</v>
+        <v>46078.47347989584</v>
       </c>
       <c r="C69" s="8">
-        <v>46181.69324881944</v>
+        <v>46181.52658215278</v>
       </c>
       <c r="D69" s="8">
-        <v>46181.694705092596</v>
+        <v>46181.528038425924</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>229</v>
@@ -5633,13 +5633,13 @@
         <v>252</v>
       </c>
       <c r="B70" s="5">
-        <v>46077.79407070602</v>
+        <v>46077.62740403935</v>
       </c>
       <c r="C70" s="5">
-        <v>46181.69329174768</v>
+        <v>46181.526625081024</v>
       </c>
       <c r="D70" s="5">
-        <v>46181.694705671296</v>
+        <v>46181.528039004625</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>202</v>
@@ -5696,13 +5696,13 @@
         <v>255</v>
       </c>
       <c r="B71" s="8">
-        <v>46077.794071296295</v>
+        <v>46077.62740462963</v>
       </c>
       <c r="C71" s="8">
-        <v>46181.693661944446</v>
+        <v>46181.526995277774</v>
       </c>
       <c r="D71" s="8">
-        <v>46181.69470625</v>
+        <v>46181.52803958333</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>203</v>
@@ -5759,13 +5759,13 @@
         <v>257</v>
       </c>
       <c r="B72" s="5">
-        <v>46077.79406888889</v>
+        <v>46077.62740222222</v>
       </c>
       <c r="C72" s="5">
-        <v>46197.586652777776</v>
+        <v>46197.41998611111</v>
       </c>
       <c r="D72" s="5">
-        <v>46197.58666969907</v>
+        <v>46197.42000303241</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>258</v>
@@ -5812,13 +5812,13 @@
         <v>260</v>
       </c>
       <c r="B73" s="8">
-        <v>46077.79406920139</v>
+        <v>46077.62740253472</v>
       </c>
       <c r="C73" s="8">
-        <v>46197.58663336806</v>
+        <v>46197.41996670139</v>
       </c>
       <c r="D73" s="8">
-        <v>46197.586652858794</v>
+        <v>46197.41998619213</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5875,13 +5875,13 @@
         <v>266</v>
       </c>
       <c r="B74" s="5">
-        <v>46077.794069456024</v>
+        <v>46077.62740278935</v>
       </c>
       <c r="C74" s="5">
-        <v>46195.50555773148</v>
+        <v>46195.338891064814</v>
       </c>
       <c r="D74" s="5">
-        <v>46197.58665158565</v>
+        <v>46197.41998491898</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5938,13 +5938,13 @@
         <v>270</v>
       </c>
       <c r="B75" s="8">
-        <v>46077.79406971065</v>
+        <v>46077.62740304398</v>
       </c>
       <c r="C75" s="8">
-        <v>46195.50534894676</v>
+        <v>46195.3386822801</v>
       </c>
       <c r="D75" s="8">
-        <v>46195.50557208333</v>
+        <v>46195.33890541666</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>271</v>
@@ -6003,13 +6003,13 @@
         <v>275</v>
       </c>
       <c r="B76" s="5">
-        <v>46077.79407002315</v>
+        <v>46077.627403356484</v>
       </c>
       <c r="C76" s="5">
-        <v>46195.50540096065</v>
+        <v>46195.33873429398</v>
       </c>
       <c r="D76" s="5">
-        <v>46195.505416203705</v>
+        <v>46195.33874953704</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>276</v>
@@ -6066,11 +6066,11 @@
         <v>278</v>
       </c>
       <c r="B77" s="8">
-        <v>46077.794070289354</v>
+        <v>46077.62740362268</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46092.562138657406</v>
+        <v>46092.39547199074</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>279</v>
@@ -6113,11 +6113,11 @@
         <v>281</v>
       </c>
       <c r="B78" s="5">
-        <v>46077.794070578704</v>
+        <v>46077.62740391203</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46195.505419849535</v>
+        <v>46195.33875318287</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>282</v>
@@ -6176,11 +6176,11 @@
         <v>285</v>
       </c>
       <c r="B79" s="8">
-        <v>46077.794070856486</v>
+        <v>46077.627404189814</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46195.50541993056</v>
+        <v>46195.33875326389</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>286</v>
@@ -6239,11 +6239,11 @@
         <v>288</v>
       </c>
       <c r="B80" s="5">
-        <v>46092.542492141205</v>
+        <v>46092.37582547453</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46092.56213928241</v>
+        <v>46092.39547261574</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>289</v>
@@ -6292,11 +6292,11 @@
         <v>291</v>
       </c>
       <c r="B81" s="8">
-        <v>46092.542531493054</v>
+        <v>46092.37586482639</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46195.505421145834</v>
+        <v>46195.33875447916</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>292</v>
@@ -6355,11 +6355,11 @@
         <v>294</v>
       </c>
       <c r="B82" s="5">
-        <v>46092.542669120376</v>
+        <v>46092.376002453704</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46185.18163831018</v>
+        <v>46185.01497164352</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>295</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-24 17:55 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -1525,13 +1525,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46077.627401377315</v>
+        <v>46077.79406804398</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.55685046296</v>
+        <v>46092.723517129634</v>
       </c>
       <c r="D4" s="5">
-        <v>46109.53423996527</v>
+        <v>46109.700906631944</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1574,13 +1574,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46077.6274017824</v>
+        <v>46077.794068449075</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.55681896991</v>
+        <v>46092.723485636576</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.71098548611</v>
+        <v>46133.877652152776</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1637,13 +1637,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46077.62740207176</v>
+        <v>46077.794068738425</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.55681956018</v>
+        <v>46092.72348622685</v>
       </c>
       <c r="D6" s="5">
-        <v>46092.55685136574</v>
+        <v>46092.723518032406</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1700,13 +1700,13 @@
         <v>38</v>
       </c>
       <c r="B7" s="8">
-        <v>46077.62740237269</v>
+        <v>46077.79406903935</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.55682003472</v>
+        <v>46092.72348670139</v>
       </c>
       <c r="D7" s="8">
-        <v>46092.55685130787</v>
+        <v>46092.72351797453</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>39</v>
@@ -1763,13 +1763,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46077.62740265046</v>
+        <v>46077.794069317126</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.55682050926</v>
+        <v>46092.72348717593</v>
       </c>
       <c r="D8" s="5">
-        <v>46093.584122500004</v>
+        <v>46093.75078916667</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -1826,13 +1826,13 @@
         <v>43</v>
       </c>
       <c r="B9" s="8">
-        <v>46077.62740295139</v>
+        <v>46077.79406961806</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.556821307866</v>
+        <v>46092.72348797454</v>
       </c>
       <c r="D9" s="8">
-        <v>46092.556851932866</v>
+        <v>46092.72351859954</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>44</v>
@@ -1889,13 +1889,13 @@
         <v>45</v>
       </c>
       <c r="B10" s="5">
-        <v>46077.62740328704</v>
+        <v>46077.7940699537</v>
       </c>
       <c r="C10" s="5">
-        <v>46196.61776415509</v>
+        <v>46196.78443082176</v>
       </c>
       <c r="D10" s="5">
-        <v>46196.61777831019</v>
+        <v>46196.78444497685</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -1942,13 +1942,13 @@
         <v>48</v>
       </c>
       <c r="B11" s="8">
-        <v>46077.62740357639</v>
+        <v>46077.79407024306</v>
       </c>
       <c r="C11" s="8">
-        <v>46093.69463644676</v>
+        <v>46093.86130311343</v>
       </c>
       <c r="D11" s="8">
-        <v>46093.69465446759</v>
+        <v>46093.86132113426</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>49</v>
@@ -2007,13 +2007,13 @@
         <v>53</v>
       </c>
       <c r="B12" s="5">
-        <v>46077.62740385417</v>
+        <v>46077.79407052083</v>
       </c>
       <c r="C12" s="5">
-        <v>46196.61774609954</v>
+        <v>46196.7844127662</v>
       </c>
       <c r="D12" s="5">
-        <v>46196.61776166667</v>
+        <v>46196.78442833333</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -2072,13 +2072,13 @@
         <v>59</v>
       </c>
       <c r="B13" s="8">
-        <v>46077.62740414352</v>
+        <v>46077.79407081018</v>
       </c>
       <c r="C13" s="8">
-        <v>46093.58531388889</v>
+        <v>46093.75198055556</v>
       </c>
       <c r="D13" s="8">
-        <v>46108.615266134264</v>
+        <v>46108.78193280092</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>60</v>
@@ -2121,13 +2121,13 @@
         <v>62</v>
       </c>
       <c r="B14" s="5">
-        <v>46077.627401273145</v>
+        <v>46077.794067939816</v>
       </c>
       <c r="C14" s="5">
-        <v>46093.58438813657</v>
+        <v>46093.751054803244</v>
       </c>
       <c r="D14" s="5">
-        <v>46093.58440603009</v>
+        <v>46093.75107269676</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>63</v>
@@ -2186,13 +2186,13 @@
         <v>67</v>
       </c>
       <c r="B15" s="8">
-        <v>46077.62740166667</v>
+        <v>46077.79406833333</v>
       </c>
       <c r="C15" s="8">
-        <v>46093.58441967593</v>
+        <v>46093.75108634259</v>
       </c>
       <c r="D15" s="8">
-        <v>46093.584435173616</v>
+        <v>46093.75110184027</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>68</v>
@@ -2251,13 +2251,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="5">
-        <v>46077.62740196759</v>
+        <v>46077.79406863426</v>
       </c>
       <c r="C16" s="5">
-        <v>46093.58446482639</v>
+        <v>46093.75113149306</v>
       </c>
       <c r="D16" s="5">
-        <v>46093.58448149306</v>
+        <v>46093.75114815972</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>71</v>
@@ -2316,13 +2316,13 @@
         <v>73</v>
       </c>
       <c r="B17" s="8">
-        <v>46077.627402303246</v>
+        <v>46077.7940689699</v>
       </c>
       <c r="C17" s="8">
-        <v>46093.584481655096</v>
+        <v>46093.75114832176</v>
       </c>
       <c r="D17" s="8">
-        <v>46093.584503252314</v>
+        <v>46093.75116991898</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>74</v>
@@ -2381,13 +2381,13 @@
         <v>76</v>
       </c>
       <c r="B18" s="5">
-        <v>46077.62740258102</v>
+        <v>46077.794069247684</v>
       </c>
       <c r="C18" s="5">
-        <v>46093.58529377315</v>
+        <v>46093.75196043981</v>
       </c>
       <c r="D18" s="5">
-        <v>46093.58531599537</v>
+        <v>46093.75198266204</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>77</v>
@@ -2446,13 +2446,13 @@
         <v>80</v>
       </c>
       <c r="B19" s="8">
-        <v>46077.627402881946</v>
+        <v>46077.79406954861</v>
       </c>
       <c r="C19" s="8">
-        <v>46093.7060909375</v>
+        <v>46093.87275760417</v>
       </c>
       <c r="D19" s="8">
-        <v>46132.66148358796</v>
+        <v>46132.82815025463</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>81</v>
@@ -2495,13 +2495,13 @@
         <v>83</v>
       </c>
       <c r="B20" s="5">
-        <v>46077.627403506944</v>
+        <v>46077.79407017361</v>
       </c>
       <c r="C20" s="5">
-        <v>46093.58544189815</v>
+        <v>46093.75210856482</v>
       </c>
       <c r="D20" s="5">
-        <v>46093.58546634259</v>
+        <v>46093.75213300926</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>84</v>
@@ -2560,13 +2560,13 @@
         <v>86</v>
       </c>
       <c r="B21" s="8">
-        <v>46077.62740315972</v>
+        <v>46077.794069826385</v>
       </c>
       <c r="C21" s="8">
-        <v>46093.585455266206</v>
+        <v>46093.75212193287</v>
       </c>
       <c r="D21" s="8">
-        <v>46093.58547449074</v>
+        <v>46093.75214115741</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>87</v>
@@ -2625,13 +2625,13 @@
         <v>89</v>
       </c>
       <c r="B22" s="5">
-        <v>46077.627404224535</v>
+        <v>46077.79407089121</v>
       </c>
       <c r="C22" s="5">
-        <v>46093.58563809028</v>
+        <v>46093.75230475694</v>
       </c>
       <c r="D22" s="5">
-        <v>46093.58565371528</v>
+        <v>46093.752320381944</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>90</v>
@@ -2690,13 +2690,13 @@
         <v>92</v>
       </c>
       <c r="B23" s="8">
-        <v>46077.627403900464</v>
+        <v>46077.79407056713</v>
       </c>
       <c r="C23" s="8">
-        <v>46093.706072175926</v>
+        <v>46093.87273884259</v>
       </c>
       <c r="D23" s="8">
-        <v>46093.70609091435</v>
+        <v>46093.87275758102</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>93</v>
@@ -2755,13 +2755,13 @@
         <v>95</v>
       </c>
       <c r="B24" s="5">
-        <v>46077.627401516205</v>
+        <v>46077.79406818287</v>
       </c>
       <c r="C24" s="5">
-        <v>46093.58568167824</v>
+        <v>46093.752348344904</v>
       </c>
       <c r="D24" s="5">
-        <v>46093.58569738426</v>
+        <v>46093.752364050924</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>96</v>
@@ -2820,13 +2820,13 @@
         <v>98</v>
       </c>
       <c r="B25" s="8">
-        <v>46078.4729491551</v>
+        <v>46078.639615821754</v>
       </c>
       <c r="C25" s="8">
-        <v>46093.58570607639</v>
+        <v>46093.75237274305</v>
       </c>
       <c r="D25" s="8">
-        <v>46093.58572271991</v>
+        <v>46093.75238938657</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>99</v>
@@ -2885,13 +2885,13 @@
         <v>101</v>
       </c>
       <c r="B26" s="5">
-        <v>46078.47300032407</v>
+        <v>46078.63966699074</v>
       </c>
       <c r="C26" s="5">
-        <v>46093.58588290509</v>
+        <v>46093.75254957176</v>
       </c>
       <c r="D26" s="5">
-        <v>46093.58590293981</v>
+        <v>46093.752569606484</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>102</v>
@@ -2950,13 +2950,13 @@
         <v>104</v>
       </c>
       <c r="B27" s="8">
-        <v>46077.62740185185</v>
+        <v>46077.79406851852</v>
       </c>
       <c r="C27" s="8">
-        <v>46175.413840775465</v>
+        <v>46175.58050744213</v>
       </c>
       <c r="D27" s="8">
-        <v>46196.65220835648</v>
+        <v>46196.81887502315</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>105</v>
@@ -3001,13 +3001,13 @@
         <v>108</v>
       </c>
       <c r="B28" s="5">
-        <v>46077.62740210648</v>
+        <v>46077.794068773146</v>
       </c>
       <c r="C28" s="5">
-        <v>46196.652190810186</v>
+        <v>46196.81885747685</v>
       </c>
       <c r="D28" s="5">
-        <v>46196.65219232639</v>
+        <v>46196.81885899305</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>109</v>
@@ -3066,13 +3066,13 @@
         <v>113</v>
       </c>
       <c r="B29" s="8">
-        <v>46077.62740236111</v>
+        <v>46077.794069027776</v>
       </c>
       <c r="C29" s="8">
-        <v>46094.559746493054</v>
+        <v>46094.72641315972</v>
       </c>
       <c r="D29" s="8">
-        <v>46094.55974833333</v>
+        <v>46094.726415</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>114</v>
@@ -3131,13 +3131,13 @@
         <v>118</v>
       </c>
       <c r="B30" s="5">
-        <v>46077.627402604165</v>
+        <v>46077.794069270836</v>
       </c>
       <c r="C30" s="5">
-        <v>46094.559799826384</v>
+        <v>46094.726466493055</v>
       </c>
       <c r="D30" s="5">
-        <v>46094.559801296295</v>
+        <v>46094.72646796296</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>119</v>
@@ -3196,13 +3196,13 @@
         <v>121</v>
       </c>
       <c r="B31" s="8">
-        <v>46077.62740287037</v>
+        <v>46077.794069537034</v>
       </c>
       <c r="C31" s="8">
-        <v>46174.472768541666</v>
+        <v>46174.63943520833</v>
       </c>
       <c r="D31" s="8">
-        <v>46181.528307939814</v>
+        <v>46181.69497460648</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>122</v>
@@ -3261,13 +3261,13 @@
         <v>124</v>
       </c>
       <c r="B32" s="5">
-        <v>46077.627403136576</v>
+        <v>46077.79406980324</v>
       </c>
       <c r="C32" s="5">
-        <v>46094.56096149306</v>
+        <v>46094.72762815972</v>
       </c>
       <c r="D32" s="5">
-        <v>46169.6622078588</v>
+        <v>46169.82887452546</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>125</v>
@@ -3326,13 +3326,13 @@
         <v>127</v>
       </c>
       <c r="B33" s="8">
-        <v>46077.62740341436</v>
+        <v>46077.794070081014</v>
       </c>
       <c r="C33" s="8">
-        <v>46174.47188952546</v>
+        <v>46174.638556192134</v>
       </c>
       <c r="D33" s="8">
-        <v>46174.47189153935</v>
+        <v>46174.63855820602</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>128</v>
@@ -3389,13 +3389,13 @@
         <v>130</v>
       </c>
       <c r="B34" s="5">
-        <v>46077.627403680555</v>
+        <v>46077.79407034723</v>
       </c>
       <c r="C34" s="5">
-        <v>46094.56312236111</v>
+        <v>46094.72978902778</v>
       </c>
       <c r="D34" s="5">
-        <v>46094.56313879629</v>
+        <v>46094.729805462965</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>131</v>
@@ -3454,13 +3454,13 @@
         <v>133</v>
       </c>
       <c r="B35" s="8">
-        <v>46077.62740395834</v>
+        <v>46077.794070625</v>
       </c>
       <c r="C35" s="8">
-        <v>46094.56209177083</v>
+        <v>46094.7287584375</v>
       </c>
       <c r="D35" s="8">
-        <v>46094.5620933912</v>
+        <v>46094.72876005787</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>134</v>
@@ -3519,13 +3519,13 @@
         <v>136</v>
       </c>
       <c r="B36" s="5">
-        <v>46077.627401342594</v>
+        <v>46077.79406800926</v>
       </c>
       <c r="C36" s="5">
-        <v>46094.56310604166</v>
+        <v>46094.729772708335</v>
       </c>
       <c r="D36" s="5">
-        <v>46094.56310759259</v>
+        <v>46094.729774259264</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>137</v>
@@ -3584,13 +3584,13 @@
         <v>139</v>
       </c>
       <c r="B37" s="8">
-        <v>46077.62740167824</v>
+        <v>46077.79406834491</v>
       </c>
       <c r="C37" s="8">
-        <v>46094.55852871528</v>
+        <v>46094.72519538194</v>
       </c>
       <c r="D37" s="8">
-        <v>46130.00231289351</v>
+        <v>46130.168979560185</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>140</v>
@@ -3649,13 +3649,13 @@
         <v>142</v>
       </c>
       <c r="B38" s="5">
-        <v>46077.62740193287</v>
+        <v>46077.79406859954</v>
       </c>
       <c r="C38" s="5">
-        <v>46094.55824585648</v>
+        <v>46094.72491252315</v>
       </c>
       <c r="D38" s="5">
-        <v>46094.55824805556</v>
+        <v>46094.72491472222</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>143</v>
@@ -3714,13 +3714,13 @@
         <v>145</v>
       </c>
       <c r="B39" s="8">
-        <v>46077.627402199076</v>
+        <v>46077.79406886574</v>
       </c>
       <c r="C39" s="8">
-        <v>46094.55846472223</v>
+        <v>46094.725131388885</v>
       </c>
       <c r="D39" s="8">
-        <v>46094.558466076385</v>
+        <v>46094.72513274306</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>146</v>
@@ -3779,13 +3779,13 @@
         <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46077.627402453705</v>
+        <v>46077.79406912037</v>
       </c>
       <c r="C40" s="5">
-        <v>46094.558513449076</v>
+        <v>46094.72518011574</v>
       </c>
       <c r="D40" s="5">
-        <v>46094.55851484954</v>
+        <v>46094.7251815162</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>149</v>
@@ -3844,13 +3844,13 @@
         <v>151</v>
       </c>
       <c r="B41" s="8">
-        <v>46077.62740268519</v>
+        <v>46077.79406935185</v>
       </c>
       <c r="C41" s="8">
-        <v>46094.571954722225</v>
+        <v>46094.73862138889</v>
       </c>
       <c r="D41" s="8">
-        <v>46100.721328287036</v>
+        <v>46100.88799495371</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>152</v>
@@ -3909,13 +3909,13 @@
         <v>156</v>
       </c>
       <c r="B42" s="5">
-        <v>46077.62740291667</v>
+        <v>46077.79406958334</v>
       </c>
       <c r="C42" s="5">
-        <v>46094.57047277778</v>
+        <v>46094.73713944445</v>
       </c>
       <c r="D42" s="5">
-        <v>46094.57155354167</v>
+        <v>46094.73822020833</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>97</v>
@@ -3974,13 +3974,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46077.627403148144</v>
+        <v>46077.794069814816</v>
       </c>
       <c r="C43" s="8">
-        <v>46094.57193980324</v>
+        <v>46094.73860646991</v>
       </c>
       <c r="D43" s="8">
-        <v>46094.57194121528</v>
+        <v>46094.73860788194</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -4039,13 +4039,13 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46078.473167627315</v>
+        <v>46078.63983429398</v>
       </c>
       <c r="C44" s="5">
-        <v>46099.68990657407</v>
+        <v>46099.856573240744</v>
       </c>
       <c r="D44" s="5">
-        <v>46099.68998267361</v>
+        <v>46099.856649340276</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4104,13 +4104,13 @@
         <v>164</v>
       </c>
       <c r="B45" s="8">
-        <v>46078.473232118056</v>
+        <v>46078.63989878472</v>
       </c>
       <c r="C45" s="8">
-        <v>46099.68980662037</v>
+        <v>46099.856473287036</v>
       </c>
       <c r="D45" s="8">
-        <v>46099.68980807871</v>
+        <v>46099.85647474537</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>165</v>
@@ -4159,13 +4159,13 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46078.473311319445</v>
+        <v>46078.63997798611</v>
       </c>
       <c r="C46" s="5">
-        <v>46099.68988975695</v>
+        <v>46099.85655642361</v>
       </c>
       <c r="D46" s="5">
-        <v>46099.689891284725</v>
+        <v>46099.85655795139</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4214,13 +4214,13 @@
         <v>170</v>
       </c>
       <c r="B47" s="8">
-        <v>46078.47114583333</v>
+        <v>46078.637812500005</v>
       </c>
       <c r="C47" s="8">
-        <v>46099.671767708336</v>
+        <v>46099.838434375</v>
       </c>
       <c r="D47" s="8">
-        <v>46121.03949925926</v>
+        <v>46121.20616592593</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>171</v>
@@ -4279,13 +4279,13 @@
         <v>175</v>
       </c>
       <c r="B48" s="5">
-        <v>46078.47124960648</v>
+        <v>46078.63791627315</v>
       </c>
       <c r="C48" s="5">
-        <v>46094.58716689815</v>
+        <v>46094.75383356481</v>
       </c>
       <c r="D48" s="5">
-        <v>46099.37121840278</v>
+        <v>46099.53788506944</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>103</v>
@@ -4340,13 +4340,13 @@
         <v>177</v>
       </c>
       <c r="B49" s="8">
-        <v>46078.471415949076</v>
+        <v>46078.63808261574</v>
       </c>
       <c r="C49" s="8">
-        <v>46099.67175158564</v>
+        <v>46099.838418252315</v>
       </c>
       <c r="D49" s="8">
-        <v>46099.67446230324</v>
+        <v>46099.84112896991</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>178</v>
@@ -4395,13 +4395,13 @@
         <v>181</v>
       </c>
       <c r="B50" s="5">
-        <v>46077.627403391205</v>
+        <v>46077.79407005787</v>
       </c>
       <c r="C50" s="5">
-        <v>46181.52820383102</v>
+        <v>46181.69487049768</v>
       </c>
       <c r="D50" s="5">
-        <v>46181.528219050924</v>
+        <v>46181.69488571759</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>182</v>
@@ -4448,13 +4448,13 @@
         <v>184</v>
       </c>
       <c r="B51" s="8">
-        <v>46077.62740362268</v>
+        <v>46077.794070289354</v>
       </c>
       <c r="C51" s="8">
-        <v>46093.59776341435</v>
+        <v>46093.76443008102</v>
       </c>
       <c r="D51" s="8">
-        <v>46093.59778137731</v>
+        <v>46093.76444804398</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>185</v>
@@ -4513,13 +4513,13 @@
         <v>189</v>
       </c>
       <c r="B52" s="5">
-        <v>46077.62740170139</v>
+        <v>46077.79406836806</v>
       </c>
       <c r="C52" s="5">
-        <v>46097.36665752315</v>
+        <v>46097.53332418982</v>
       </c>
       <c r="D52" s="5">
-        <v>46097.366677962964</v>
+        <v>46097.53334462963</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>190</v>
@@ -4578,13 +4578,13 @@
         <v>195</v>
       </c>
       <c r="B53" s="8">
-        <v>46092.31643899306</v>
+        <v>46092.48310565972</v>
       </c>
       <c r="C53" s="8">
-        <v>46097.36670182871</v>
+        <v>46097.533368495366</v>
       </c>
       <c r="D53" s="8">
-        <v>46097.36671966435</v>
+        <v>46097.53338633102</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>196</v>
@@ -4641,13 +4641,13 @@
         <v>198</v>
       </c>
       <c r="B54" s="5">
-        <v>46092.31653091435</v>
+        <v>46092.48319758102</v>
       </c>
       <c r="C54" s="5">
-        <v>46181.52670012732</v>
+        <v>46181.69336679398</v>
       </c>
       <c r="D54" s="5">
-        <v>46181.52824409722</v>
+        <v>46181.694910763894</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>199</v>
@@ -4706,13 +4706,13 @@
         <v>204</v>
       </c>
       <c r="B55" s="8">
-        <v>46079.44846875</v>
+        <v>46079.615135416665</v>
       </c>
       <c r="C55" s="8">
-        <v>46100.301554861115</v>
+        <v>46100.46822152778</v>
       </c>
       <c r="D55" s="8">
-        <v>46135.59274305556</v>
+        <v>46135.75940972222</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>205</v>
@@ -4755,13 +4755,13 @@
         <v>207</v>
       </c>
       <c r="B56" s="5">
-        <v>46078.582749016205</v>
+        <v>46078.74941568287</v>
       </c>
       <c r="C56" s="5">
-        <v>46100.301533391204</v>
+        <v>46100.46820005787</v>
       </c>
       <c r="D56" s="5">
-        <v>46122.0265565625</v>
+        <v>46122.193223229166</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>206</v>
@@ -4820,13 +4820,13 @@
         <v>211</v>
       </c>
       <c r="B57" s="8">
-        <v>46077.627403935185</v>
+        <v>46077.794070601856</v>
       </c>
       <c r="C57" s="8">
-        <v>46181.52990055556</v>
+        <v>46181.69656722222</v>
       </c>
       <c r="D57" s="8">
-        <v>46181.71383997685</v>
+        <v>46181.880506643516</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>212</v>
@@ -4869,13 +4869,13 @@
         <v>214</v>
       </c>
       <c r="B58" s="5">
-        <v>46077.627404224535</v>
+        <v>46077.79407089121</v>
       </c>
       <c r="C58" s="5">
-        <v>46099.44183902778</v>
+        <v>46099.60850569444</v>
       </c>
       <c r="D58" s="5">
-        <v>46099.441857638885</v>
+        <v>46099.60852430556</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>215</v>
@@ -4934,13 +4934,13 @@
         <v>219</v>
       </c>
       <c r="B59" s="8">
-        <v>46077.627401805556</v>
+        <v>46077.79406847223</v>
       </c>
       <c r="C59" s="8">
-        <v>46181.529883888885</v>
+        <v>46181.696550555556</v>
       </c>
       <c r="D59" s="8">
-        <v>46181.529900671296</v>
+        <v>46181.69656733796</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>57</v>
@@ -4999,13 +4999,13 @@
         <v>221</v>
       </c>
       <c r="B60" s="5">
-        <v>46077.6274021412</v>
+        <v>46077.79406880787</v>
       </c>
       <c r="C60" s="5">
-        <v>46099.44185101852</v>
+        <v>46099.608517685185</v>
       </c>
       <c r="D60" s="5">
-        <v>46107.98050693287</v>
+        <v>46108.14717359954</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>222</v>
@@ -5064,13 +5064,13 @@
         <v>224</v>
       </c>
       <c r="B61" s="8">
-        <v>46077.62740243056</v>
+        <v>46077.79406909722</v>
       </c>
       <c r="C61" s="8">
-        <v>46099.44188891204</v>
+        <v>46099.6085555787</v>
       </c>
       <c r="D61" s="8">
-        <v>46134.03879127315</v>
+        <v>46134.20545793981</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>225</v>
@@ -5129,13 +5129,13 @@
         <v>227</v>
       </c>
       <c r="B62" s="5">
-        <v>46078.47339827546</v>
+        <v>46078.64006494213</v>
       </c>
       <c r="C62" s="5">
-        <v>46099.69005751157</v>
+        <v>46099.856724178244</v>
       </c>
       <c r="D62" s="5">
-        <v>46099.69015126157</v>
+        <v>46099.856817928245</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>228</v>
@@ -5194,13 +5194,13 @@
         <v>230</v>
       </c>
       <c r="B63" s="8">
-        <v>46078.47246883102</v>
+        <v>46078.63913549768</v>
       </c>
       <c r="C63" s="8">
-        <v>46120.46123489583</v>
+        <v>46120.627901562504</v>
       </c>
       <c r="D63" s="8">
-        <v>46120.46125703704</v>
+        <v>46120.62792370371</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>231</v>
@@ -5259,13 +5259,13 @@
         <v>232</v>
       </c>
       <c r="B64" s="5">
-        <v>46077.62740271991</v>
+        <v>46077.794069386575</v>
       </c>
       <c r="C64" s="5">
-        <v>46181.52798491898</v>
+        <v>46181.69465158565</v>
       </c>
       <c r="D64" s="5">
-        <v>46197.41864</v>
+        <v>46197.58530666667</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>233</v>
@@ -5308,13 +5308,13 @@
         <v>235</v>
       </c>
       <c r="B65" s="8">
-        <v>46077.62740298611</v>
+        <v>46077.79406965278</v>
       </c>
       <c r="C65" s="8">
-        <v>46140.394836273146</v>
+        <v>46140.56150293982</v>
       </c>
       <c r="D65" s="8">
-        <v>46181.528036793985</v>
+        <v>46181.69470346065</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>236</v>
@@ -5373,13 +5373,13 @@
         <v>240</v>
       </c>
       <c r="B66" s="5">
-        <v>46077.62740324074</v>
+        <v>46077.79406990741</v>
       </c>
       <c r="C66" s="5">
-        <v>46181.52654994213</v>
+        <v>46181.69321660879</v>
       </c>
       <c r="D66" s="5">
-        <v>46181.52803732639</v>
+        <v>46181.69470399305</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>241</v>
@@ -5438,13 +5438,13 @@
         <v>244</v>
       </c>
       <c r="B67" s="8">
-        <v>46077.62740349537</v>
+        <v>46077.79407016204</v>
       </c>
       <c r="C67" s="8">
-        <v>46113.39420686342</v>
+        <v>46113.56087353009</v>
       </c>
       <c r="D67" s="8">
-        <v>46140.394845324074</v>
+        <v>46140.561511990745</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>245</v>
@@ -5503,13 +5503,13 @@
         <v>247</v>
       </c>
       <c r="B68" s="5">
-        <v>46077.62740376157</v>
+        <v>46077.79407042824</v>
       </c>
       <c r="C68" s="5">
-        <v>46181.526571759256</v>
+        <v>46181.69323842593</v>
       </c>
       <c r="D68" s="5">
-        <v>46181.52803785879</v>
+        <v>46181.694704525464</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>248</v>
@@ -5568,13 +5568,13 @@
         <v>250</v>
       </c>
       <c r="B69" s="8">
-        <v>46078.47347989584</v>
+        <v>46078.640146562495</v>
       </c>
       <c r="C69" s="8">
-        <v>46181.52658215278</v>
+        <v>46181.69324881944</v>
       </c>
       <c r="D69" s="8">
-        <v>46181.528038425924</v>
+        <v>46181.694705092596</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>229</v>
@@ -5633,13 +5633,13 @@
         <v>252</v>
       </c>
       <c r="B70" s="5">
-        <v>46077.62740403935</v>
+        <v>46077.79407070602</v>
       </c>
       <c r="C70" s="5">
-        <v>46181.526625081024</v>
+        <v>46181.69329174768</v>
       </c>
       <c r="D70" s="5">
-        <v>46181.528039004625</v>
+        <v>46181.694705671296</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>202</v>
@@ -5696,13 +5696,13 @@
         <v>255</v>
       </c>
       <c r="B71" s="8">
-        <v>46077.62740462963</v>
+        <v>46077.794071296295</v>
       </c>
       <c r="C71" s="8">
-        <v>46181.526995277774</v>
+        <v>46181.693661944446</v>
       </c>
       <c r="D71" s="8">
-        <v>46181.52803958333</v>
+        <v>46181.69470625</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>203</v>
@@ -5759,13 +5759,13 @@
         <v>257</v>
       </c>
       <c r="B72" s="5">
-        <v>46077.62740222222</v>
+        <v>46077.79406888889</v>
       </c>
       <c r="C72" s="5">
-        <v>46197.41998611111</v>
+        <v>46197.586652777776</v>
       </c>
       <c r="D72" s="5">
-        <v>46197.42000303241</v>
+        <v>46197.58666969907</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>258</v>
@@ -5812,13 +5812,13 @@
         <v>260</v>
       </c>
       <c r="B73" s="8">
-        <v>46077.62740253472</v>
+        <v>46077.79406920139</v>
       </c>
       <c r="C73" s="8">
-        <v>46197.41996670139</v>
+        <v>46197.58663336806</v>
       </c>
       <c r="D73" s="8">
-        <v>46197.41998619213</v>
+        <v>46197.586652858794</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5875,13 +5875,13 @@
         <v>266</v>
       </c>
       <c r="B74" s="5">
-        <v>46077.62740278935</v>
+        <v>46077.794069456024</v>
       </c>
       <c r="C74" s="5">
-        <v>46195.338891064814</v>
+        <v>46195.50555773148</v>
       </c>
       <c r="D74" s="5">
-        <v>46197.41998491898</v>
+        <v>46197.58665158565</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5938,13 +5938,13 @@
         <v>270</v>
       </c>
       <c r="B75" s="8">
-        <v>46077.62740304398</v>
+        <v>46077.79406971065</v>
       </c>
       <c r="C75" s="8">
-        <v>46195.3386822801</v>
+        <v>46195.50534894676</v>
       </c>
       <c r="D75" s="8">
-        <v>46195.33890541666</v>
+        <v>46195.50557208333</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>271</v>
@@ -6003,13 +6003,13 @@
         <v>275</v>
       </c>
       <c r="B76" s="5">
-        <v>46077.627403356484</v>
+        <v>46077.79407002315</v>
       </c>
       <c r="C76" s="5">
-        <v>46195.33873429398</v>
+        <v>46195.50540096065</v>
       </c>
       <c r="D76" s="5">
-        <v>46195.33874953704</v>
+        <v>46195.505416203705</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>276</v>
@@ -6066,11 +6066,11 @@
         <v>278</v>
       </c>
       <c r="B77" s="8">
-        <v>46077.62740362268</v>
+        <v>46077.794070289354</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46092.39547199074</v>
+        <v>46092.562138657406</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>279</v>
@@ -6113,11 +6113,11 @@
         <v>281</v>
       </c>
       <c r="B78" s="5">
-        <v>46077.62740391203</v>
+        <v>46077.794070578704</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46195.33875318287</v>
+        <v>46195.505419849535</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>282</v>
@@ -6176,11 +6176,11 @@
         <v>285</v>
       </c>
       <c r="B79" s="8">
-        <v>46077.627404189814</v>
+        <v>46077.794070856486</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46195.33875326389</v>
+        <v>46195.50541993056</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>286</v>
@@ -6239,11 +6239,11 @@
         <v>288</v>
       </c>
       <c r="B80" s="5">
-        <v>46092.37582547453</v>
+        <v>46092.542492141205</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46092.39547261574</v>
+        <v>46092.56213928241</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>289</v>
@@ -6292,11 +6292,11 @@
         <v>291</v>
       </c>
       <c r="B81" s="8">
-        <v>46092.37586482639</v>
+        <v>46092.542531493054</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46195.33875447916</v>
+        <v>46195.505421145834</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>292</v>
@@ -6355,11 +6355,11 @@
         <v>294</v>
       </c>
       <c r="B82" s="5">
-        <v>46092.376002453704</v>
+        <v>46092.542669120376</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46185.01497164352</v>
+        <v>46185.18163831018</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>295</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-25 15:52 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -1525,13 +1525,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46077.79406804398</v>
+        <v>46077.627401377315</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.723517129634</v>
+        <v>46092.55685046296</v>
       </c>
       <c r="D4" s="5">
-        <v>46109.700906631944</v>
+        <v>46109.53423996527</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1574,13 +1574,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46077.794068449075</v>
+        <v>46077.6274017824</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.723485636576</v>
+        <v>46092.55681896991</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.877652152776</v>
+        <v>46133.71098548611</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1637,13 +1637,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46077.794068738425</v>
+        <v>46077.62740207176</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.72348622685</v>
+        <v>46092.55681956018</v>
       </c>
       <c r="D6" s="5">
-        <v>46092.723518032406</v>
+        <v>46092.55685136574</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1700,13 +1700,13 @@
         <v>38</v>
       </c>
       <c r="B7" s="8">
-        <v>46077.79406903935</v>
+        <v>46077.62740237269</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.72348670139</v>
+        <v>46092.55682003472</v>
       </c>
       <c r="D7" s="8">
-        <v>46092.72351797453</v>
+        <v>46092.55685130787</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>39</v>
@@ -1763,13 +1763,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46077.794069317126</v>
+        <v>46077.62740265046</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.72348717593</v>
+        <v>46092.55682050926</v>
       </c>
       <c r="D8" s="5">
-        <v>46093.75078916667</v>
+        <v>46093.584122500004</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -1826,13 +1826,13 @@
         <v>43</v>
       </c>
       <c r="B9" s="8">
-        <v>46077.79406961806</v>
+        <v>46077.62740295139</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.72348797454</v>
+        <v>46092.556821307866</v>
       </c>
       <c r="D9" s="8">
-        <v>46092.72351859954</v>
+        <v>46092.556851932866</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>44</v>
@@ -1889,13 +1889,13 @@
         <v>45</v>
       </c>
       <c r="B10" s="5">
-        <v>46077.7940699537</v>
+        <v>46077.62740328704</v>
       </c>
       <c r="C10" s="5">
-        <v>46196.78443082176</v>
+        <v>46196.61776415509</v>
       </c>
       <c r="D10" s="5">
-        <v>46196.78444497685</v>
+        <v>46196.61777831019</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -1942,13 +1942,13 @@
         <v>48</v>
       </c>
       <c r="B11" s="8">
-        <v>46077.79407024306</v>
+        <v>46077.62740357639</v>
       </c>
       <c r="C11" s="8">
-        <v>46093.86130311343</v>
+        <v>46093.69463644676</v>
       </c>
       <c r="D11" s="8">
-        <v>46093.86132113426</v>
+        <v>46093.69465446759</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>49</v>
@@ -2007,13 +2007,13 @@
         <v>53</v>
       </c>
       <c r="B12" s="5">
-        <v>46077.79407052083</v>
+        <v>46077.62740385417</v>
       </c>
       <c r="C12" s="5">
-        <v>46196.7844127662</v>
+        <v>46196.61774609954</v>
       </c>
       <c r="D12" s="5">
-        <v>46196.78442833333</v>
+        <v>46196.61776166667</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -2072,13 +2072,13 @@
         <v>59</v>
       </c>
       <c r="B13" s="8">
-        <v>46077.79407081018</v>
+        <v>46077.62740414352</v>
       </c>
       <c r="C13" s="8">
-        <v>46093.75198055556</v>
+        <v>46093.58531388889</v>
       </c>
       <c r="D13" s="8">
-        <v>46108.78193280092</v>
+        <v>46108.615266134264</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>60</v>
@@ -2121,13 +2121,13 @@
         <v>62</v>
       </c>
       <c r="B14" s="5">
-        <v>46077.794067939816</v>
+        <v>46077.627401273145</v>
       </c>
       <c r="C14" s="5">
-        <v>46093.751054803244</v>
+        <v>46093.58438813657</v>
       </c>
       <c r="D14" s="5">
-        <v>46093.75107269676</v>
+        <v>46093.58440603009</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>63</v>
@@ -2186,13 +2186,13 @@
         <v>67</v>
       </c>
       <c r="B15" s="8">
-        <v>46077.79406833333</v>
+        <v>46077.62740166667</v>
       </c>
       <c r="C15" s="8">
-        <v>46093.75108634259</v>
+        <v>46093.58441967593</v>
       </c>
       <c r="D15" s="8">
-        <v>46093.75110184027</v>
+        <v>46093.584435173616</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>68</v>
@@ -2251,13 +2251,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="5">
-        <v>46077.79406863426</v>
+        <v>46077.62740196759</v>
       </c>
       <c r="C16" s="5">
-        <v>46093.75113149306</v>
+        <v>46093.58446482639</v>
       </c>
       <c r="D16" s="5">
-        <v>46093.75114815972</v>
+        <v>46093.58448149306</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>71</v>
@@ -2316,13 +2316,13 @@
         <v>73</v>
       </c>
       <c r="B17" s="8">
-        <v>46077.7940689699</v>
+        <v>46077.627402303246</v>
       </c>
       <c r="C17" s="8">
-        <v>46093.75114832176</v>
+        <v>46093.584481655096</v>
       </c>
       <c r="D17" s="8">
-        <v>46093.75116991898</v>
+        <v>46093.584503252314</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>74</v>
@@ -2381,13 +2381,13 @@
         <v>76</v>
       </c>
       <c r="B18" s="5">
-        <v>46077.794069247684</v>
+        <v>46077.62740258102</v>
       </c>
       <c r="C18" s="5">
-        <v>46093.75196043981</v>
+        <v>46093.58529377315</v>
       </c>
       <c r="D18" s="5">
-        <v>46093.75198266204</v>
+        <v>46093.58531599537</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>77</v>
@@ -2446,13 +2446,13 @@
         <v>80</v>
       </c>
       <c r="B19" s="8">
-        <v>46077.79406954861</v>
+        <v>46077.627402881946</v>
       </c>
       <c r="C19" s="8">
-        <v>46093.87275760417</v>
+        <v>46093.7060909375</v>
       </c>
       <c r="D19" s="8">
-        <v>46132.82815025463</v>
+        <v>46132.66148358796</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>81</v>
@@ -2495,13 +2495,13 @@
         <v>83</v>
       </c>
       <c r="B20" s="5">
-        <v>46077.79407017361</v>
+        <v>46077.627403506944</v>
       </c>
       <c r="C20" s="5">
-        <v>46093.75210856482</v>
+        <v>46093.58544189815</v>
       </c>
       <c r="D20" s="5">
-        <v>46093.75213300926</v>
+        <v>46093.58546634259</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>84</v>
@@ -2560,13 +2560,13 @@
         <v>86</v>
       </c>
       <c r="B21" s="8">
-        <v>46077.794069826385</v>
+        <v>46077.62740315972</v>
       </c>
       <c r="C21" s="8">
-        <v>46093.75212193287</v>
+        <v>46093.585455266206</v>
       </c>
       <c r="D21" s="8">
-        <v>46093.75214115741</v>
+        <v>46093.58547449074</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>87</v>
@@ -2625,13 +2625,13 @@
         <v>89</v>
       </c>
       <c r="B22" s="5">
-        <v>46077.79407089121</v>
+        <v>46077.627404224535</v>
       </c>
       <c r="C22" s="5">
-        <v>46093.75230475694</v>
+        <v>46093.58563809028</v>
       </c>
       <c r="D22" s="5">
-        <v>46093.752320381944</v>
+        <v>46093.58565371528</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>90</v>
@@ -2690,13 +2690,13 @@
         <v>92</v>
       </c>
       <c r="B23" s="8">
-        <v>46077.79407056713</v>
+        <v>46077.627403900464</v>
       </c>
       <c r="C23" s="8">
-        <v>46093.87273884259</v>
+        <v>46093.706072175926</v>
       </c>
       <c r="D23" s="8">
-        <v>46093.87275758102</v>
+        <v>46093.70609091435</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>93</v>
@@ -2755,13 +2755,13 @@
         <v>95</v>
       </c>
       <c r="B24" s="5">
-        <v>46077.79406818287</v>
+        <v>46077.627401516205</v>
       </c>
       <c r="C24" s="5">
-        <v>46093.752348344904</v>
+        <v>46093.58568167824</v>
       </c>
       <c r="D24" s="5">
-        <v>46093.752364050924</v>
+        <v>46093.58569738426</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>96</v>
@@ -2820,13 +2820,13 @@
         <v>98</v>
       </c>
       <c r="B25" s="8">
-        <v>46078.639615821754</v>
+        <v>46078.4729491551</v>
       </c>
       <c r="C25" s="8">
-        <v>46093.75237274305</v>
+        <v>46093.58570607639</v>
       </c>
       <c r="D25" s="8">
-        <v>46093.75238938657</v>
+        <v>46093.58572271991</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>99</v>
@@ -2885,13 +2885,13 @@
         <v>101</v>
       </c>
       <c r="B26" s="5">
-        <v>46078.63966699074</v>
+        <v>46078.47300032407</v>
       </c>
       <c r="C26" s="5">
-        <v>46093.75254957176</v>
+        <v>46093.58588290509</v>
       </c>
       <c r="D26" s="5">
-        <v>46093.752569606484</v>
+        <v>46093.58590293981</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>102</v>
@@ -2950,13 +2950,13 @@
         <v>104</v>
       </c>
       <c r="B27" s="8">
-        <v>46077.79406851852</v>
+        <v>46077.62740185185</v>
       </c>
       <c r="C27" s="8">
-        <v>46175.58050744213</v>
+        <v>46175.413840775465</v>
       </c>
       <c r="D27" s="8">
-        <v>46196.81887502315</v>
+        <v>46196.65220835648</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>105</v>
@@ -3001,13 +3001,13 @@
         <v>108</v>
       </c>
       <c r="B28" s="5">
-        <v>46077.794068773146</v>
+        <v>46077.62740210648</v>
       </c>
       <c r="C28" s="5">
-        <v>46196.81885747685</v>
+        <v>46196.652190810186</v>
       </c>
       <c r="D28" s="5">
-        <v>46196.81885899305</v>
+        <v>46196.65219232639</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>109</v>
@@ -3066,13 +3066,13 @@
         <v>113</v>
       </c>
       <c r="B29" s="8">
-        <v>46077.794069027776</v>
+        <v>46077.62740236111</v>
       </c>
       <c r="C29" s="8">
-        <v>46094.72641315972</v>
+        <v>46094.559746493054</v>
       </c>
       <c r="D29" s="8">
-        <v>46094.726415</v>
+        <v>46094.55974833333</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>114</v>
@@ -3131,13 +3131,13 @@
         <v>118</v>
       </c>
       <c r="B30" s="5">
-        <v>46077.794069270836</v>
+        <v>46077.627402604165</v>
       </c>
       <c r="C30" s="5">
-        <v>46094.726466493055</v>
+        <v>46094.559799826384</v>
       </c>
       <c r="D30" s="5">
-        <v>46094.72646796296</v>
+        <v>46094.559801296295</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>119</v>
@@ -3196,13 +3196,13 @@
         <v>121</v>
       </c>
       <c r="B31" s="8">
-        <v>46077.794069537034</v>
+        <v>46077.62740287037</v>
       </c>
       <c r="C31" s="8">
-        <v>46174.63943520833</v>
+        <v>46174.472768541666</v>
       </c>
       <c r="D31" s="8">
-        <v>46181.69497460648</v>
+        <v>46181.528307939814</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>122</v>
@@ -3261,13 +3261,13 @@
         <v>124</v>
       </c>
       <c r="B32" s="5">
-        <v>46077.79406980324</v>
+        <v>46077.627403136576</v>
       </c>
       <c r="C32" s="5">
-        <v>46094.72762815972</v>
+        <v>46094.56096149306</v>
       </c>
       <c r="D32" s="5">
-        <v>46169.82887452546</v>
+        <v>46169.6622078588</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>125</v>
@@ -3326,13 +3326,13 @@
         <v>127</v>
       </c>
       <c r="B33" s="8">
-        <v>46077.794070081014</v>
+        <v>46077.62740341436</v>
       </c>
       <c r="C33" s="8">
-        <v>46174.638556192134</v>
+        <v>46174.47188952546</v>
       </c>
       <c r="D33" s="8">
-        <v>46174.63855820602</v>
+        <v>46174.47189153935</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>128</v>
@@ -3389,13 +3389,13 @@
         <v>130</v>
       </c>
       <c r="B34" s="5">
-        <v>46077.79407034723</v>
+        <v>46077.627403680555</v>
       </c>
       <c r="C34" s="5">
-        <v>46094.72978902778</v>
+        <v>46094.56312236111</v>
       </c>
       <c r="D34" s="5">
-        <v>46094.729805462965</v>
+        <v>46094.56313879629</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>131</v>
@@ -3454,13 +3454,13 @@
         <v>133</v>
       </c>
       <c r="B35" s="8">
-        <v>46077.794070625</v>
+        <v>46077.62740395834</v>
       </c>
       <c r="C35" s="8">
-        <v>46094.7287584375</v>
+        <v>46094.56209177083</v>
       </c>
       <c r="D35" s="8">
-        <v>46094.72876005787</v>
+        <v>46094.5620933912</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>134</v>
@@ -3519,13 +3519,13 @@
         <v>136</v>
       </c>
       <c r="B36" s="5">
-        <v>46077.79406800926</v>
+        <v>46077.627401342594</v>
       </c>
       <c r="C36" s="5">
-        <v>46094.729772708335</v>
+        <v>46094.56310604166</v>
       </c>
       <c r="D36" s="5">
-        <v>46094.729774259264</v>
+        <v>46094.56310759259</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>137</v>
@@ -3584,13 +3584,13 @@
         <v>139</v>
       </c>
       <c r="B37" s="8">
-        <v>46077.79406834491</v>
+        <v>46077.62740167824</v>
       </c>
       <c r="C37" s="8">
-        <v>46094.72519538194</v>
+        <v>46094.55852871528</v>
       </c>
       <c r="D37" s="8">
-        <v>46130.168979560185</v>
+        <v>46130.00231289351</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>140</v>
@@ -3649,13 +3649,13 @@
         <v>142</v>
       </c>
       <c r="B38" s="5">
-        <v>46077.79406859954</v>
+        <v>46077.62740193287</v>
       </c>
       <c r="C38" s="5">
-        <v>46094.72491252315</v>
+        <v>46094.55824585648</v>
       </c>
       <c r="D38" s="5">
-        <v>46094.72491472222</v>
+        <v>46094.55824805556</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>143</v>
@@ -3714,13 +3714,13 @@
         <v>145</v>
       </c>
       <c r="B39" s="8">
-        <v>46077.79406886574</v>
+        <v>46077.627402199076</v>
       </c>
       <c r="C39" s="8">
-        <v>46094.725131388885</v>
+        <v>46094.55846472223</v>
       </c>
       <c r="D39" s="8">
-        <v>46094.72513274306</v>
+        <v>46094.558466076385</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>146</v>
@@ -3779,13 +3779,13 @@
         <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46077.79406912037</v>
+        <v>46077.627402453705</v>
       </c>
       <c r="C40" s="5">
-        <v>46094.72518011574</v>
+        <v>46094.558513449076</v>
       </c>
       <c r="D40" s="5">
-        <v>46094.7251815162</v>
+        <v>46094.55851484954</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>149</v>
@@ -3844,13 +3844,13 @@
         <v>151</v>
       </c>
       <c r="B41" s="8">
-        <v>46077.79406935185</v>
+        <v>46077.62740268519</v>
       </c>
       <c r="C41" s="8">
-        <v>46094.73862138889</v>
+        <v>46094.571954722225</v>
       </c>
       <c r="D41" s="8">
-        <v>46100.88799495371</v>
+        <v>46100.721328287036</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>152</v>
@@ -3909,13 +3909,13 @@
         <v>156</v>
       </c>
       <c r="B42" s="5">
-        <v>46077.79406958334</v>
+        <v>46077.62740291667</v>
       </c>
       <c r="C42" s="5">
-        <v>46094.73713944445</v>
+        <v>46094.57047277778</v>
       </c>
       <c r="D42" s="5">
-        <v>46094.73822020833</v>
+        <v>46094.57155354167</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>97</v>
@@ -3974,13 +3974,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46077.794069814816</v>
+        <v>46077.627403148144</v>
       </c>
       <c r="C43" s="8">
-        <v>46094.73860646991</v>
+        <v>46094.57193980324</v>
       </c>
       <c r="D43" s="8">
-        <v>46094.73860788194</v>
+        <v>46094.57194121528</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -4039,13 +4039,13 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46078.63983429398</v>
+        <v>46078.473167627315</v>
       </c>
       <c r="C44" s="5">
-        <v>46099.856573240744</v>
+        <v>46099.68990657407</v>
       </c>
       <c r="D44" s="5">
-        <v>46099.856649340276</v>
+        <v>46099.68998267361</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4104,13 +4104,13 @@
         <v>164</v>
       </c>
       <c r="B45" s="8">
-        <v>46078.63989878472</v>
+        <v>46078.473232118056</v>
       </c>
       <c r="C45" s="8">
-        <v>46099.856473287036</v>
+        <v>46099.68980662037</v>
       </c>
       <c r="D45" s="8">
-        <v>46099.85647474537</v>
+        <v>46099.68980807871</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>165</v>
@@ -4159,13 +4159,13 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46078.63997798611</v>
+        <v>46078.473311319445</v>
       </c>
       <c r="C46" s="5">
-        <v>46099.85655642361</v>
+        <v>46099.68988975695</v>
       </c>
       <c r="D46" s="5">
-        <v>46099.85655795139</v>
+        <v>46099.689891284725</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4214,13 +4214,13 @@
         <v>170</v>
       </c>
       <c r="B47" s="8">
-        <v>46078.637812500005</v>
+        <v>46078.47114583333</v>
       </c>
       <c r="C47" s="8">
-        <v>46099.838434375</v>
+        <v>46099.671767708336</v>
       </c>
       <c r="D47" s="8">
-        <v>46121.20616592593</v>
+        <v>46121.03949925926</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>171</v>
@@ -4279,13 +4279,13 @@
         <v>175</v>
       </c>
       <c r="B48" s="5">
-        <v>46078.63791627315</v>
+        <v>46078.47124960648</v>
       </c>
       <c r="C48" s="5">
-        <v>46094.75383356481</v>
+        <v>46094.58716689815</v>
       </c>
       <c r="D48" s="5">
-        <v>46099.53788506944</v>
+        <v>46099.37121840278</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>103</v>
@@ -4340,13 +4340,13 @@
         <v>177</v>
       </c>
       <c r="B49" s="8">
-        <v>46078.63808261574</v>
+        <v>46078.471415949076</v>
       </c>
       <c r="C49" s="8">
-        <v>46099.838418252315</v>
+        <v>46099.67175158564</v>
       </c>
       <c r="D49" s="8">
-        <v>46099.84112896991</v>
+        <v>46099.67446230324</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>178</v>
@@ -4395,13 +4395,13 @@
         <v>181</v>
       </c>
       <c r="B50" s="5">
-        <v>46077.79407005787</v>
+        <v>46077.627403391205</v>
       </c>
       <c r="C50" s="5">
-        <v>46181.69487049768</v>
+        <v>46181.52820383102</v>
       </c>
       <c r="D50" s="5">
-        <v>46181.69488571759</v>
+        <v>46181.528219050924</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>182</v>
@@ -4448,13 +4448,13 @@
         <v>184</v>
       </c>
       <c r="B51" s="8">
-        <v>46077.794070289354</v>
+        <v>46077.62740362268</v>
       </c>
       <c r="C51" s="8">
-        <v>46093.76443008102</v>
+        <v>46093.59776341435</v>
       </c>
       <c r="D51" s="8">
-        <v>46093.76444804398</v>
+        <v>46093.59778137731</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>185</v>
@@ -4513,13 +4513,13 @@
         <v>189</v>
       </c>
       <c r="B52" s="5">
-        <v>46077.79406836806</v>
+        <v>46077.62740170139</v>
       </c>
       <c r="C52" s="5">
-        <v>46097.53332418982</v>
+        <v>46097.36665752315</v>
       </c>
       <c r="D52" s="5">
-        <v>46097.53334462963</v>
+        <v>46097.366677962964</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>190</v>
@@ -4578,13 +4578,13 @@
         <v>195</v>
       </c>
       <c r="B53" s="8">
-        <v>46092.48310565972</v>
+        <v>46092.31643899306</v>
       </c>
       <c r="C53" s="8">
-        <v>46097.533368495366</v>
+        <v>46097.36670182871</v>
       </c>
       <c r="D53" s="8">
-        <v>46097.53338633102</v>
+        <v>46097.36671966435</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>196</v>
@@ -4641,13 +4641,13 @@
         <v>198</v>
       </c>
       <c r="B54" s="5">
-        <v>46092.48319758102</v>
+        <v>46092.31653091435</v>
       </c>
       <c r="C54" s="5">
-        <v>46181.69336679398</v>
+        <v>46181.52670012732</v>
       </c>
       <c r="D54" s="5">
-        <v>46181.694910763894</v>
+        <v>46181.52824409722</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>199</v>
@@ -4706,13 +4706,13 @@
         <v>204</v>
       </c>
       <c r="B55" s="8">
-        <v>46079.615135416665</v>
+        <v>46079.44846875</v>
       </c>
       <c r="C55" s="8">
-        <v>46100.46822152778</v>
+        <v>46100.301554861115</v>
       </c>
       <c r="D55" s="8">
-        <v>46135.75940972222</v>
+        <v>46135.59274305556</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>205</v>
@@ -4755,13 +4755,13 @@
         <v>207</v>
       </c>
       <c r="B56" s="5">
-        <v>46078.74941568287</v>
+        <v>46078.582749016205</v>
       </c>
       <c r="C56" s="5">
-        <v>46100.46820005787</v>
+        <v>46100.301533391204</v>
       </c>
       <c r="D56" s="5">
-        <v>46122.193223229166</v>
+        <v>46122.0265565625</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>206</v>
@@ -4820,13 +4820,13 @@
         <v>211</v>
       </c>
       <c r="B57" s="8">
-        <v>46077.794070601856</v>
+        <v>46077.627403935185</v>
       </c>
       <c r="C57" s="8">
-        <v>46181.69656722222</v>
+        <v>46181.52990055556</v>
       </c>
       <c r="D57" s="8">
-        <v>46181.880506643516</v>
+        <v>46181.71383997685</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>212</v>
@@ -4869,13 +4869,13 @@
         <v>214</v>
       </c>
       <c r="B58" s="5">
-        <v>46077.79407089121</v>
+        <v>46077.627404224535</v>
       </c>
       <c r="C58" s="5">
-        <v>46099.60850569444</v>
+        <v>46099.44183902778</v>
       </c>
       <c r="D58" s="5">
-        <v>46099.60852430556</v>
+        <v>46099.441857638885</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>215</v>
@@ -4934,13 +4934,13 @@
         <v>219</v>
       </c>
       <c r="B59" s="8">
-        <v>46077.79406847223</v>
+        <v>46077.627401805556</v>
       </c>
       <c r="C59" s="8">
-        <v>46181.696550555556</v>
+        <v>46181.529883888885</v>
       </c>
       <c r="D59" s="8">
-        <v>46181.69656733796</v>
+        <v>46181.529900671296</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>57</v>
@@ -4999,13 +4999,13 @@
         <v>221</v>
       </c>
       <c r="B60" s="5">
-        <v>46077.79406880787</v>
+        <v>46077.6274021412</v>
       </c>
       <c r="C60" s="5">
-        <v>46099.608517685185</v>
+        <v>46099.44185101852</v>
       </c>
       <c r="D60" s="5">
-        <v>46108.14717359954</v>
+        <v>46107.98050693287</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>222</v>
@@ -5064,13 +5064,13 @@
         <v>224</v>
       </c>
       <c r="B61" s="8">
-        <v>46077.79406909722</v>
+        <v>46077.62740243056</v>
       </c>
       <c r="C61" s="8">
-        <v>46099.6085555787</v>
+        <v>46099.44188891204</v>
       </c>
       <c r="D61" s="8">
-        <v>46134.20545793981</v>
+        <v>46134.03879127315</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>225</v>
@@ -5129,13 +5129,13 @@
         <v>227</v>
       </c>
       <c r="B62" s="5">
-        <v>46078.64006494213</v>
+        <v>46078.47339827546</v>
       </c>
       <c r="C62" s="5">
-        <v>46099.856724178244</v>
+        <v>46099.69005751157</v>
       </c>
       <c r="D62" s="5">
-        <v>46099.856817928245</v>
+        <v>46099.69015126157</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>228</v>
@@ -5194,13 +5194,13 @@
         <v>230</v>
       </c>
       <c r="B63" s="8">
-        <v>46078.63913549768</v>
+        <v>46078.47246883102</v>
       </c>
       <c r="C63" s="8">
-        <v>46120.627901562504</v>
+        <v>46120.46123489583</v>
       </c>
       <c r="D63" s="8">
-        <v>46120.62792370371</v>
+        <v>46120.46125703704</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>231</v>
@@ -5259,13 +5259,13 @@
         <v>232</v>
       </c>
       <c r="B64" s="5">
-        <v>46077.794069386575</v>
+        <v>46077.62740271991</v>
       </c>
       <c r="C64" s="5">
-        <v>46181.69465158565</v>
+        <v>46181.52798491898</v>
       </c>
       <c r="D64" s="5">
-        <v>46197.58530666667</v>
+        <v>46197.41864</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>233</v>
@@ -5308,13 +5308,13 @@
         <v>235</v>
       </c>
       <c r="B65" s="8">
-        <v>46077.79406965278</v>
+        <v>46077.62740298611</v>
       </c>
       <c r="C65" s="8">
-        <v>46140.56150293982</v>
+        <v>46140.394836273146</v>
       </c>
       <c r="D65" s="8">
-        <v>46181.69470346065</v>
+        <v>46181.528036793985</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>236</v>
@@ -5373,13 +5373,13 @@
         <v>240</v>
       </c>
       <c r="B66" s="5">
-        <v>46077.79406990741</v>
+        <v>46077.62740324074</v>
       </c>
       <c r="C66" s="5">
-        <v>46181.69321660879</v>
+        <v>46181.52654994213</v>
       </c>
       <c r="D66" s="5">
-        <v>46181.69470399305</v>
+        <v>46181.52803732639</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>241</v>
@@ -5438,13 +5438,13 @@
         <v>244</v>
       </c>
       <c r="B67" s="8">
-        <v>46077.79407016204</v>
+        <v>46077.62740349537</v>
       </c>
       <c r="C67" s="8">
-        <v>46113.56087353009</v>
+        <v>46113.39420686342</v>
       </c>
       <c r="D67" s="8">
-        <v>46140.561511990745</v>
+        <v>46140.394845324074</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>245</v>
@@ -5503,13 +5503,13 @@
         <v>247</v>
       </c>
       <c r="B68" s="5">
-        <v>46077.79407042824</v>
+        <v>46077.62740376157</v>
       </c>
       <c r="C68" s="5">
-        <v>46181.69323842593</v>
+        <v>46181.526571759256</v>
       </c>
       <c r="D68" s="5">
-        <v>46181.694704525464</v>
+        <v>46181.52803785879</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>248</v>
@@ -5568,13 +5568,13 @@
         <v>250</v>
       </c>
       <c r="B69" s="8">
-        <v>46078.640146562495</v>
+        <v>46078.47347989584</v>
       </c>
       <c r="C69" s="8">
-        <v>46181.69324881944</v>
+        <v>46181.52658215278</v>
       </c>
       <c r="D69" s="8">
-        <v>46181.694705092596</v>
+        <v>46181.528038425924</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>229</v>
@@ -5633,13 +5633,13 @@
         <v>252</v>
       </c>
       <c r="B70" s="5">
-        <v>46077.79407070602</v>
+        <v>46077.62740403935</v>
       </c>
       <c r="C70" s="5">
-        <v>46181.69329174768</v>
+        <v>46181.526625081024</v>
       </c>
       <c r="D70" s="5">
-        <v>46181.694705671296</v>
+        <v>46181.528039004625</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>202</v>
@@ -5696,13 +5696,13 @@
         <v>255</v>
       </c>
       <c r="B71" s="8">
-        <v>46077.794071296295</v>
+        <v>46077.62740462963</v>
       </c>
       <c r="C71" s="8">
-        <v>46181.693661944446</v>
+        <v>46181.526995277774</v>
       </c>
       <c r="D71" s="8">
-        <v>46181.69470625</v>
+        <v>46181.52803958333</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>203</v>
@@ -5759,13 +5759,13 @@
         <v>257</v>
       </c>
       <c r="B72" s="5">
-        <v>46077.79406888889</v>
+        <v>46077.62740222222</v>
       </c>
       <c r="C72" s="5">
-        <v>46197.586652777776</v>
+        <v>46197.41998611111</v>
       </c>
       <c r="D72" s="5">
-        <v>46197.58666969907</v>
+        <v>46197.42000303241</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>258</v>
@@ -5812,13 +5812,13 @@
         <v>260</v>
       </c>
       <c r="B73" s="8">
-        <v>46077.79406920139</v>
+        <v>46077.62740253472</v>
       </c>
       <c r="C73" s="8">
-        <v>46197.58663336806</v>
+        <v>46197.41996670139</v>
       </c>
       <c r="D73" s="8">
-        <v>46197.586652858794</v>
+        <v>46197.41998619213</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5875,13 +5875,13 @@
         <v>266</v>
       </c>
       <c r="B74" s="5">
-        <v>46077.794069456024</v>
+        <v>46077.62740278935</v>
       </c>
       <c r="C74" s="5">
-        <v>46195.50555773148</v>
+        <v>46195.338891064814</v>
       </c>
       <c r="D74" s="5">
-        <v>46197.58665158565</v>
+        <v>46197.41998491898</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5938,13 +5938,13 @@
         <v>270</v>
       </c>
       <c r="B75" s="8">
-        <v>46077.79406971065</v>
+        <v>46077.62740304398</v>
       </c>
       <c r="C75" s="8">
-        <v>46195.50534894676</v>
+        <v>46195.3386822801</v>
       </c>
       <c r="D75" s="8">
-        <v>46195.50557208333</v>
+        <v>46195.33890541666</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>271</v>
@@ -6003,13 +6003,13 @@
         <v>275</v>
       </c>
       <c r="B76" s="5">
-        <v>46077.79407002315</v>
+        <v>46077.627403356484</v>
       </c>
       <c r="C76" s="5">
-        <v>46195.50540096065</v>
+        <v>46195.33873429398</v>
       </c>
       <c r="D76" s="5">
-        <v>46195.505416203705</v>
+        <v>46195.33874953704</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>276</v>
@@ -6066,11 +6066,11 @@
         <v>278</v>
       </c>
       <c r="B77" s="8">
-        <v>46077.794070289354</v>
+        <v>46077.62740362268</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46092.562138657406</v>
+        <v>46092.39547199074</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>279</v>
@@ -6113,11 +6113,11 @@
         <v>281</v>
       </c>
       <c r="B78" s="5">
-        <v>46077.794070578704</v>
+        <v>46077.62740391203</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46195.505419849535</v>
+        <v>46195.33875318287</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>282</v>
@@ -6176,11 +6176,11 @@
         <v>285</v>
       </c>
       <c r="B79" s="8">
-        <v>46077.794070856486</v>
+        <v>46077.627404189814</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46195.50541993056</v>
+        <v>46195.33875326389</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>286</v>
@@ -6239,11 +6239,11 @@
         <v>288</v>
       </c>
       <c r="B80" s="5">
-        <v>46092.542492141205</v>
+        <v>46092.37582547453</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46092.56213928241</v>
+        <v>46092.39547261574</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>289</v>
@@ -6292,11 +6292,11 @@
         <v>291</v>
       </c>
       <c r="B81" s="8">
-        <v>46092.542531493054</v>
+        <v>46092.37586482639</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46195.505421145834</v>
+        <v>46195.33875447916</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>292</v>
@@ -6355,11 +6355,11 @@
         <v>294</v>
       </c>
       <c r="B82" s="5">
-        <v>46092.542669120376</v>
+        <v>46092.376002453704</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46185.18163831018</v>
+        <v>46185.01497164352</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>295</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-25 16:07 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -1525,13 +1525,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46077.627401377315</v>
+        <v>46077.79406804398</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.55685046296</v>
+        <v>46092.723517129634</v>
       </c>
       <c r="D4" s="5">
-        <v>46109.53423996527</v>
+        <v>46109.700906631944</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1574,13 +1574,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46077.6274017824</v>
+        <v>46077.794068449075</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.55681896991</v>
+        <v>46092.723485636576</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.71098548611</v>
+        <v>46133.877652152776</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1637,13 +1637,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46077.62740207176</v>
+        <v>46077.794068738425</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.55681956018</v>
+        <v>46092.72348622685</v>
       </c>
       <c r="D6" s="5">
-        <v>46092.55685136574</v>
+        <v>46092.723518032406</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1700,13 +1700,13 @@
         <v>38</v>
       </c>
       <c r="B7" s="8">
-        <v>46077.62740237269</v>
+        <v>46077.79406903935</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.55682003472</v>
+        <v>46092.72348670139</v>
       </c>
       <c r="D7" s="8">
-        <v>46092.55685130787</v>
+        <v>46092.72351797453</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>39</v>
@@ -1763,13 +1763,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46077.62740265046</v>
+        <v>46077.794069317126</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.55682050926</v>
+        <v>46092.72348717593</v>
       </c>
       <c r="D8" s="5">
-        <v>46093.584122500004</v>
+        <v>46093.75078916667</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -1826,13 +1826,13 @@
         <v>43</v>
       </c>
       <c r="B9" s="8">
-        <v>46077.62740295139</v>
+        <v>46077.79406961806</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.556821307866</v>
+        <v>46092.72348797454</v>
       </c>
       <c r="D9" s="8">
-        <v>46092.556851932866</v>
+        <v>46092.72351859954</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>44</v>
@@ -1889,13 +1889,13 @@
         <v>45</v>
       </c>
       <c r="B10" s="5">
-        <v>46077.62740328704</v>
+        <v>46077.7940699537</v>
       </c>
       <c r="C10" s="5">
-        <v>46196.61776415509</v>
+        <v>46196.78443082176</v>
       </c>
       <c r="D10" s="5">
-        <v>46196.61777831019</v>
+        <v>46196.78444497685</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -1942,13 +1942,13 @@
         <v>48</v>
       </c>
       <c r="B11" s="8">
-        <v>46077.62740357639</v>
+        <v>46077.79407024306</v>
       </c>
       <c r="C11" s="8">
-        <v>46093.69463644676</v>
+        <v>46093.86130311343</v>
       </c>
       <c r="D11" s="8">
-        <v>46093.69465446759</v>
+        <v>46093.86132113426</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>49</v>
@@ -2007,13 +2007,13 @@
         <v>53</v>
       </c>
       <c r="B12" s="5">
-        <v>46077.62740385417</v>
+        <v>46077.79407052083</v>
       </c>
       <c r="C12" s="5">
-        <v>46196.61774609954</v>
+        <v>46196.7844127662</v>
       </c>
       <c r="D12" s="5">
-        <v>46196.61776166667</v>
+        <v>46196.78442833333</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -2072,13 +2072,13 @@
         <v>59</v>
       </c>
       <c r="B13" s="8">
-        <v>46077.62740414352</v>
+        <v>46077.79407081018</v>
       </c>
       <c r="C13" s="8">
-        <v>46093.58531388889</v>
+        <v>46093.75198055556</v>
       </c>
       <c r="D13" s="8">
-        <v>46108.615266134264</v>
+        <v>46108.78193280092</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>60</v>
@@ -2121,13 +2121,13 @@
         <v>62</v>
       </c>
       <c r="B14" s="5">
-        <v>46077.627401273145</v>
+        <v>46077.794067939816</v>
       </c>
       <c r="C14" s="5">
-        <v>46093.58438813657</v>
+        <v>46093.751054803244</v>
       </c>
       <c r="D14" s="5">
-        <v>46093.58440603009</v>
+        <v>46093.75107269676</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>63</v>
@@ -2186,13 +2186,13 @@
         <v>67</v>
       </c>
       <c r="B15" s="8">
-        <v>46077.62740166667</v>
+        <v>46077.79406833333</v>
       </c>
       <c r="C15" s="8">
-        <v>46093.58441967593</v>
+        <v>46093.75108634259</v>
       </c>
       <c r="D15" s="8">
-        <v>46093.584435173616</v>
+        <v>46093.75110184027</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>68</v>
@@ -2251,13 +2251,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="5">
-        <v>46077.62740196759</v>
+        <v>46077.79406863426</v>
       </c>
       <c r="C16" s="5">
-        <v>46093.58446482639</v>
+        <v>46093.75113149306</v>
       </c>
       <c r="D16" s="5">
-        <v>46093.58448149306</v>
+        <v>46093.75114815972</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>71</v>
@@ -2316,13 +2316,13 @@
         <v>73</v>
       </c>
       <c r="B17" s="8">
-        <v>46077.627402303246</v>
+        <v>46077.7940689699</v>
       </c>
       <c r="C17" s="8">
-        <v>46093.584481655096</v>
+        <v>46093.75114832176</v>
       </c>
       <c r="D17" s="8">
-        <v>46093.584503252314</v>
+        <v>46093.75116991898</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>74</v>
@@ -2381,13 +2381,13 @@
         <v>76</v>
       </c>
       <c r="B18" s="5">
-        <v>46077.62740258102</v>
+        <v>46077.794069247684</v>
       </c>
       <c r="C18" s="5">
-        <v>46093.58529377315</v>
+        <v>46093.75196043981</v>
       </c>
       <c r="D18" s="5">
-        <v>46093.58531599537</v>
+        <v>46093.75198266204</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>77</v>
@@ -2446,13 +2446,13 @@
         <v>80</v>
       </c>
       <c r="B19" s="8">
-        <v>46077.627402881946</v>
+        <v>46077.79406954861</v>
       </c>
       <c r="C19" s="8">
-        <v>46093.7060909375</v>
+        <v>46093.87275760417</v>
       </c>
       <c r="D19" s="8">
-        <v>46132.66148358796</v>
+        <v>46132.82815025463</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>81</v>
@@ -2495,13 +2495,13 @@
         <v>83</v>
       </c>
       <c r="B20" s="5">
-        <v>46077.627403506944</v>
+        <v>46077.79407017361</v>
       </c>
       <c r="C20" s="5">
-        <v>46093.58544189815</v>
+        <v>46093.75210856482</v>
       </c>
       <c r="D20" s="5">
-        <v>46093.58546634259</v>
+        <v>46093.75213300926</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>84</v>
@@ -2560,13 +2560,13 @@
         <v>86</v>
       </c>
       <c r="B21" s="8">
-        <v>46077.62740315972</v>
+        <v>46077.794069826385</v>
       </c>
       <c r="C21" s="8">
-        <v>46093.585455266206</v>
+        <v>46093.75212193287</v>
       </c>
       <c r="D21" s="8">
-        <v>46093.58547449074</v>
+        <v>46093.75214115741</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>87</v>
@@ -2625,13 +2625,13 @@
         <v>89</v>
       </c>
       <c r="B22" s="5">
-        <v>46077.627404224535</v>
+        <v>46077.79407089121</v>
       </c>
       <c r="C22" s="5">
-        <v>46093.58563809028</v>
+        <v>46093.75230475694</v>
       </c>
       <c r="D22" s="5">
-        <v>46093.58565371528</v>
+        <v>46093.752320381944</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>90</v>
@@ -2690,13 +2690,13 @@
         <v>92</v>
       </c>
       <c r="B23" s="8">
-        <v>46077.627403900464</v>
+        <v>46077.79407056713</v>
       </c>
       <c r="C23" s="8">
-        <v>46093.706072175926</v>
+        <v>46093.87273884259</v>
       </c>
       <c r="D23" s="8">
-        <v>46093.70609091435</v>
+        <v>46093.87275758102</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>93</v>
@@ -2755,13 +2755,13 @@
         <v>95</v>
       </c>
       <c r="B24" s="5">
-        <v>46077.627401516205</v>
+        <v>46077.79406818287</v>
       </c>
       <c r="C24" s="5">
-        <v>46093.58568167824</v>
+        <v>46093.752348344904</v>
       </c>
       <c r="D24" s="5">
-        <v>46093.58569738426</v>
+        <v>46093.752364050924</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>96</v>
@@ -2820,13 +2820,13 @@
         <v>98</v>
       </c>
       <c r="B25" s="8">
-        <v>46078.4729491551</v>
+        <v>46078.639615821754</v>
       </c>
       <c r="C25" s="8">
-        <v>46093.58570607639</v>
+        <v>46093.75237274305</v>
       </c>
       <c r="D25" s="8">
-        <v>46093.58572271991</v>
+        <v>46093.75238938657</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>99</v>
@@ -2885,13 +2885,13 @@
         <v>101</v>
       </c>
       <c r="B26" s="5">
-        <v>46078.47300032407</v>
+        <v>46078.63966699074</v>
       </c>
       <c r="C26" s="5">
-        <v>46093.58588290509</v>
+        <v>46093.75254957176</v>
       </c>
       <c r="D26" s="5">
-        <v>46093.58590293981</v>
+        <v>46093.752569606484</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>102</v>
@@ -2950,13 +2950,13 @@
         <v>104</v>
       </c>
       <c r="B27" s="8">
-        <v>46077.62740185185</v>
+        <v>46077.79406851852</v>
       </c>
       <c r="C27" s="8">
-        <v>46175.413840775465</v>
+        <v>46175.58050744213</v>
       </c>
       <c r="D27" s="8">
-        <v>46196.65220835648</v>
+        <v>46196.81887502315</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>105</v>
@@ -3001,13 +3001,13 @@
         <v>108</v>
       </c>
       <c r="B28" s="5">
-        <v>46077.62740210648</v>
+        <v>46077.794068773146</v>
       </c>
       <c r="C28" s="5">
-        <v>46196.652190810186</v>
+        <v>46196.81885747685</v>
       </c>
       <c r="D28" s="5">
-        <v>46196.65219232639</v>
+        <v>46196.81885899305</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>109</v>
@@ -3066,13 +3066,13 @@
         <v>113</v>
       </c>
       <c r="B29" s="8">
-        <v>46077.62740236111</v>
+        <v>46077.794069027776</v>
       </c>
       <c r="C29" s="8">
-        <v>46094.559746493054</v>
+        <v>46094.72641315972</v>
       </c>
       <c r="D29" s="8">
-        <v>46094.55974833333</v>
+        <v>46094.726415</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>114</v>
@@ -3131,13 +3131,13 @@
         <v>118</v>
       </c>
       <c r="B30" s="5">
-        <v>46077.627402604165</v>
+        <v>46077.794069270836</v>
       </c>
       <c r="C30" s="5">
-        <v>46094.559799826384</v>
+        <v>46094.726466493055</v>
       </c>
       <c r="D30" s="5">
-        <v>46094.559801296295</v>
+        <v>46094.72646796296</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>119</v>
@@ -3196,13 +3196,13 @@
         <v>121</v>
       </c>
       <c r="B31" s="8">
-        <v>46077.62740287037</v>
+        <v>46077.794069537034</v>
       </c>
       <c r="C31" s="8">
-        <v>46174.472768541666</v>
+        <v>46174.63943520833</v>
       </c>
       <c r="D31" s="8">
-        <v>46181.528307939814</v>
+        <v>46181.69497460648</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>122</v>
@@ -3261,13 +3261,13 @@
         <v>124</v>
       </c>
       <c r="B32" s="5">
-        <v>46077.627403136576</v>
+        <v>46077.79406980324</v>
       </c>
       <c r="C32" s="5">
-        <v>46094.56096149306</v>
+        <v>46094.72762815972</v>
       </c>
       <c r="D32" s="5">
-        <v>46169.6622078588</v>
+        <v>46169.82887452546</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>125</v>
@@ -3326,13 +3326,13 @@
         <v>127</v>
       </c>
       <c r="B33" s="8">
-        <v>46077.62740341436</v>
+        <v>46077.794070081014</v>
       </c>
       <c r="C33" s="8">
-        <v>46174.47188952546</v>
+        <v>46174.638556192134</v>
       </c>
       <c r="D33" s="8">
-        <v>46174.47189153935</v>
+        <v>46174.63855820602</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>128</v>
@@ -3389,13 +3389,13 @@
         <v>130</v>
       </c>
       <c r="B34" s="5">
-        <v>46077.627403680555</v>
+        <v>46077.79407034723</v>
       </c>
       <c r="C34" s="5">
-        <v>46094.56312236111</v>
+        <v>46094.72978902778</v>
       </c>
       <c r="D34" s="5">
-        <v>46094.56313879629</v>
+        <v>46094.729805462965</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>131</v>
@@ -3454,13 +3454,13 @@
         <v>133</v>
       </c>
       <c r="B35" s="8">
-        <v>46077.62740395834</v>
+        <v>46077.794070625</v>
       </c>
       <c r="C35" s="8">
-        <v>46094.56209177083</v>
+        <v>46094.7287584375</v>
       </c>
       <c r="D35" s="8">
-        <v>46094.5620933912</v>
+        <v>46094.72876005787</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>134</v>
@@ -3519,13 +3519,13 @@
         <v>136</v>
       </c>
       <c r="B36" s="5">
-        <v>46077.627401342594</v>
+        <v>46077.79406800926</v>
       </c>
       <c r="C36" s="5">
-        <v>46094.56310604166</v>
+        <v>46094.729772708335</v>
       </c>
       <c r="D36" s="5">
-        <v>46094.56310759259</v>
+        <v>46094.729774259264</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>137</v>
@@ -3584,13 +3584,13 @@
         <v>139</v>
       </c>
       <c r="B37" s="8">
-        <v>46077.62740167824</v>
+        <v>46077.79406834491</v>
       </c>
       <c r="C37" s="8">
-        <v>46094.55852871528</v>
+        <v>46094.72519538194</v>
       </c>
       <c r="D37" s="8">
-        <v>46130.00231289351</v>
+        <v>46130.168979560185</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>140</v>
@@ -3649,13 +3649,13 @@
         <v>142</v>
       </c>
       <c r="B38" s="5">
-        <v>46077.62740193287</v>
+        <v>46077.79406859954</v>
       </c>
       <c r="C38" s="5">
-        <v>46094.55824585648</v>
+        <v>46094.72491252315</v>
       </c>
       <c r="D38" s="5">
-        <v>46094.55824805556</v>
+        <v>46094.72491472222</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>143</v>
@@ -3714,13 +3714,13 @@
         <v>145</v>
       </c>
       <c r="B39" s="8">
-        <v>46077.627402199076</v>
+        <v>46077.79406886574</v>
       </c>
       <c r="C39" s="8">
-        <v>46094.55846472223</v>
+        <v>46094.725131388885</v>
       </c>
       <c r="D39" s="8">
-        <v>46094.558466076385</v>
+        <v>46094.72513274306</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>146</v>
@@ -3779,13 +3779,13 @@
         <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46077.627402453705</v>
+        <v>46077.79406912037</v>
       </c>
       <c r="C40" s="5">
-        <v>46094.558513449076</v>
+        <v>46094.72518011574</v>
       </c>
       <c r="D40" s="5">
-        <v>46094.55851484954</v>
+        <v>46094.7251815162</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>149</v>
@@ -3844,13 +3844,13 @@
         <v>151</v>
       </c>
       <c r="B41" s="8">
-        <v>46077.62740268519</v>
+        <v>46077.79406935185</v>
       </c>
       <c r="C41" s="8">
-        <v>46094.571954722225</v>
+        <v>46094.73862138889</v>
       </c>
       <c r="D41" s="8">
-        <v>46100.721328287036</v>
+        <v>46100.88799495371</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>152</v>
@@ -3909,13 +3909,13 @@
         <v>156</v>
       </c>
       <c r="B42" s="5">
-        <v>46077.62740291667</v>
+        <v>46077.79406958334</v>
       </c>
       <c r="C42" s="5">
-        <v>46094.57047277778</v>
+        <v>46094.73713944445</v>
       </c>
       <c r="D42" s="5">
-        <v>46094.57155354167</v>
+        <v>46094.73822020833</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>97</v>
@@ -3974,13 +3974,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46077.627403148144</v>
+        <v>46077.794069814816</v>
       </c>
       <c r="C43" s="8">
-        <v>46094.57193980324</v>
+        <v>46094.73860646991</v>
       </c>
       <c r="D43" s="8">
-        <v>46094.57194121528</v>
+        <v>46094.73860788194</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -4039,13 +4039,13 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46078.473167627315</v>
+        <v>46078.63983429398</v>
       </c>
       <c r="C44" s="5">
-        <v>46099.68990657407</v>
+        <v>46099.856573240744</v>
       </c>
       <c r="D44" s="5">
-        <v>46099.68998267361</v>
+        <v>46099.856649340276</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4104,13 +4104,13 @@
         <v>164</v>
       </c>
       <c r="B45" s="8">
-        <v>46078.473232118056</v>
+        <v>46078.63989878472</v>
       </c>
       <c r="C45" s="8">
-        <v>46099.68980662037</v>
+        <v>46099.856473287036</v>
       </c>
       <c r="D45" s="8">
-        <v>46099.68980807871</v>
+        <v>46099.85647474537</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>165</v>
@@ -4159,13 +4159,13 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46078.473311319445</v>
+        <v>46078.63997798611</v>
       </c>
       <c r="C46" s="5">
-        <v>46099.68988975695</v>
+        <v>46099.85655642361</v>
       </c>
       <c r="D46" s="5">
-        <v>46099.689891284725</v>
+        <v>46099.85655795139</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4214,13 +4214,13 @@
         <v>170</v>
       </c>
       <c r="B47" s="8">
-        <v>46078.47114583333</v>
+        <v>46078.637812500005</v>
       </c>
       <c r="C47" s="8">
-        <v>46099.671767708336</v>
+        <v>46099.838434375</v>
       </c>
       <c r="D47" s="8">
-        <v>46121.03949925926</v>
+        <v>46121.20616592593</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>171</v>
@@ -4279,13 +4279,13 @@
         <v>175</v>
       </c>
       <c r="B48" s="5">
-        <v>46078.47124960648</v>
+        <v>46078.63791627315</v>
       </c>
       <c r="C48" s="5">
-        <v>46094.58716689815</v>
+        <v>46094.75383356481</v>
       </c>
       <c r="D48" s="5">
-        <v>46099.37121840278</v>
+        <v>46099.53788506944</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>103</v>
@@ -4340,13 +4340,13 @@
         <v>177</v>
       </c>
       <c r="B49" s="8">
-        <v>46078.471415949076</v>
+        <v>46078.63808261574</v>
       </c>
       <c r="C49" s="8">
-        <v>46099.67175158564</v>
+        <v>46099.838418252315</v>
       </c>
       <c r="D49" s="8">
-        <v>46099.67446230324</v>
+        <v>46099.84112896991</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>178</v>
@@ -4395,13 +4395,13 @@
         <v>181</v>
       </c>
       <c r="B50" s="5">
-        <v>46077.627403391205</v>
+        <v>46077.79407005787</v>
       </c>
       <c r="C50" s="5">
-        <v>46181.52820383102</v>
+        <v>46181.69487049768</v>
       </c>
       <c r="D50" s="5">
-        <v>46181.528219050924</v>
+        <v>46181.69488571759</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>182</v>
@@ -4448,13 +4448,13 @@
         <v>184</v>
       </c>
       <c r="B51" s="8">
-        <v>46077.62740362268</v>
+        <v>46077.794070289354</v>
       </c>
       <c r="C51" s="8">
-        <v>46093.59776341435</v>
+        <v>46093.76443008102</v>
       </c>
       <c r="D51" s="8">
-        <v>46093.59778137731</v>
+        <v>46093.76444804398</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>185</v>
@@ -4513,13 +4513,13 @@
         <v>189</v>
       </c>
       <c r="B52" s="5">
-        <v>46077.62740170139</v>
+        <v>46077.79406836806</v>
       </c>
       <c r="C52" s="5">
-        <v>46097.36665752315</v>
+        <v>46097.53332418982</v>
       </c>
       <c r="D52" s="5">
-        <v>46097.366677962964</v>
+        <v>46097.53334462963</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>190</v>
@@ -4578,13 +4578,13 @@
         <v>195</v>
       </c>
       <c r="B53" s="8">
-        <v>46092.31643899306</v>
+        <v>46092.48310565972</v>
       </c>
       <c r="C53" s="8">
-        <v>46097.36670182871</v>
+        <v>46097.533368495366</v>
       </c>
       <c r="D53" s="8">
-        <v>46097.36671966435</v>
+        <v>46097.53338633102</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>196</v>
@@ -4641,13 +4641,13 @@
         <v>198</v>
       </c>
       <c r="B54" s="5">
-        <v>46092.31653091435</v>
+        <v>46092.48319758102</v>
       </c>
       <c r="C54" s="5">
-        <v>46181.52670012732</v>
+        <v>46181.69336679398</v>
       </c>
       <c r="D54" s="5">
-        <v>46181.52824409722</v>
+        <v>46181.694910763894</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>199</v>
@@ -4706,13 +4706,13 @@
         <v>204</v>
       </c>
       <c r="B55" s="8">
-        <v>46079.44846875</v>
+        <v>46079.615135416665</v>
       </c>
       <c r="C55" s="8">
-        <v>46100.301554861115</v>
+        <v>46100.46822152778</v>
       </c>
       <c r="D55" s="8">
-        <v>46135.59274305556</v>
+        <v>46135.75940972222</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>205</v>
@@ -4755,13 +4755,13 @@
         <v>207</v>
       </c>
       <c r="B56" s="5">
-        <v>46078.582749016205</v>
+        <v>46078.74941568287</v>
       </c>
       <c r="C56" s="5">
-        <v>46100.301533391204</v>
+        <v>46100.46820005787</v>
       </c>
       <c r="D56" s="5">
-        <v>46122.0265565625</v>
+        <v>46122.193223229166</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>206</v>
@@ -4820,13 +4820,13 @@
         <v>211</v>
       </c>
       <c r="B57" s="8">
-        <v>46077.627403935185</v>
+        <v>46077.794070601856</v>
       </c>
       <c r="C57" s="8">
-        <v>46181.52990055556</v>
+        <v>46181.69656722222</v>
       </c>
       <c r="D57" s="8">
-        <v>46181.71383997685</v>
+        <v>46181.880506643516</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>212</v>
@@ -4869,13 +4869,13 @@
         <v>214</v>
       </c>
       <c r="B58" s="5">
-        <v>46077.627404224535</v>
+        <v>46077.79407089121</v>
       </c>
       <c r="C58" s="5">
-        <v>46099.44183902778</v>
+        <v>46099.60850569444</v>
       </c>
       <c r="D58" s="5">
-        <v>46099.441857638885</v>
+        <v>46099.60852430556</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>215</v>
@@ -4934,13 +4934,13 @@
         <v>219</v>
       </c>
       <c r="B59" s="8">
-        <v>46077.627401805556</v>
+        <v>46077.79406847223</v>
       </c>
       <c r="C59" s="8">
-        <v>46181.529883888885</v>
+        <v>46181.696550555556</v>
       </c>
       <c r="D59" s="8">
-        <v>46181.529900671296</v>
+        <v>46181.69656733796</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>57</v>
@@ -4999,13 +4999,13 @@
         <v>221</v>
       </c>
       <c r="B60" s="5">
-        <v>46077.6274021412</v>
+        <v>46077.79406880787</v>
       </c>
       <c r="C60" s="5">
-        <v>46099.44185101852</v>
+        <v>46099.608517685185</v>
       </c>
       <c r="D60" s="5">
-        <v>46107.98050693287</v>
+        <v>46108.14717359954</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>222</v>
@@ -5064,13 +5064,13 @@
         <v>224</v>
       </c>
       <c r="B61" s="8">
-        <v>46077.62740243056</v>
+        <v>46077.79406909722</v>
       </c>
       <c r="C61" s="8">
-        <v>46099.44188891204</v>
+        <v>46099.6085555787</v>
       </c>
       <c r="D61" s="8">
-        <v>46134.03879127315</v>
+        <v>46134.20545793981</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>225</v>
@@ -5129,13 +5129,13 @@
         <v>227</v>
       </c>
       <c r="B62" s="5">
-        <v>46078.47339827546</v>
+        <v>46078.64006494213</v>
       </c>
       <c r="C62" s="5">
-        <v>46099.69005751157</v>
+        <v>46099.856724178244</v>
       </c>
       <c r="D62" s="5">
-        <v>46099.69015126157</v>
+        <v>46099.856817928245</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>228</v>
@@ -5194,13 +5194,13 @@
         <v>230</v>
       </c>
       <c r="B63" s="8">
-        <v>46078.47246883102</v>
+        <v>46078.63913549768</v>
       </c>
       <c r="C63" s="8">
-        <v>46120.46123489583</v>
+        <v>46120.627901562504</v>
       </c>
       <c r="D63" s="8">
-        <v>46120.46125703704</v>
+        <v>46120.62792370371</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>231</v>
@@ -5259,13 +5259,13 @@
         <v>232</v>
       </c>
       <c r="B64" s="5">
-        <v>46077.62740271991</v>
+        <v>46077.794069386575</v>
       </c>
       <c r="C64" s="5">
-        <v>46181.52798491898</v>
+        <v>46181.69465158565</v>
       </c>
       <c r="D64" s="5">
-        <v>46197.41864</v>
+        <v>46197.58530666667</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>233</v>
@@ -5308,13 +5308,13 @@
         <v>235</v>
       </c>
       <c r="B65" s="8">
-        <v>46077.62740298611</v>
+        <v>46077.79406965278</v>
       </c>
       <c r="C65" s="8">
-        <v>46140.394836273146</v>
+        <v>46140.56150293982</v>
       </c>
       <c r="D65" s="8">
-        <v>46181.528036793985</v>
+        <v>46181.69470346065</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>236</v>
@@ -5373,13 +5373,13 @@
         <v>240</v>
       </c>
       <c r="B66" s="5">
-        <v>46077.62740324074</v>
+        <v>46077.79406990741</v>
       </c>
       <c r="C66" s="5">
-        <v>46181.52654994213</v>
+        <v>46181.69321660879</v>
       </c>
       <c r="D66" s="5">
-        <v>46181.52803732639</v>
+        <v>46181.69470399305</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>241</v>
@@ -5438,13 +5438,13 @@
         <v>244</v>
       </c>
       <c r="B67" s="8">
-        <v>46077.62740349537</v>
+        <v>46077.79407016204</v>
       </c>
       <c r="C67" s="8">
-        <v>46113.39420686342</v>
+        <v>46113.56087353009</v>
       </c>
       <c r="D67" s="8">
-        <v>46140.394845324074</v>
+        <v>46140.561511990745</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>245</v>
@@ -5503,13 +5503,13 @@
         <v>247</v>
       </c>
       <c r="B68" s="5">
-        <v>46077.62740376157</v>
+        <v>46077.79407042824</v>
       </c>
       <c r="C68" s="5">
-        <v>46181.526571759256</v>
+        <v>46181.69323842593</v>
       </c>
       <c r="D68" s="5">
-        <v>46181.52803785879</v>
+        <v>46181.694704525464</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>248</v>
@@ -5568,13 +5568,13 @@
         <v>250</v>
       </c>
       <c r="B69" s="8">
-        <v>46078.47347989584</v>
+        <v>46078.640146562495</v>
       </c>
       <c r="C69" s="8">
-        <v>46181.52658215278</v>
+        <v>46181.69324881944</v>
       </c>
       <c r="D69" s="8">
-        <v>46181.528038425924</v>
+        <v>46181.694705092596</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>229</v>
@@ -5633,13 +5633,13 @@
         <v>252</v>
       </c>
       <c r="B70" s="5">
-        <v>46077.62740403935</v>
+        <v>46077.79407070602</v>
       </c>
       <c r="C70" s="5">
-        <v>46181.526625081024</v>
+        <v>46181.69329174768</v>
       </c>
       <c r="D70" s="5">
-        <v>46181.528039004625</v>
+        <v>46181.694705671296</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>202</v>
@@ -5696,13 +5696,13 @@
         <v>255</v>
       </c>
       <c r="B71" s="8">
-        <v>46077.62740462963</v>
+        <v>46077.794071296295</v>
       </c>
       <c r="C71" s="8">
-        <v>46181.526995277774</v>
+        <v>46181.693661944446</v>
       </c>
       <c r="D71" s="8">
-        <v>46181.52803958333</v>
+        <v>46181.69470625</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>203</v>
@@ -5759,13 +5759,13 @@
         <v>257</v>
       </c>
       <c r="B72" s="5">
-        <v>46077.62740222222</v>
+        <v>46077.79406888889</v>
       </c>
       <c r="C72" s="5">
-        <v>46197.41998611111</v>
+        <v>46197.586652777776</v>
       </c>
       <c r="D72" s="5">
-        <v>46197.42000303241</v>
+        <v>46197.58666969907</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>258</v>
@@ -5812,13 +5812,13 @@
         <v>260</v>
       </c>
       <c r="B73" s="8">
-        <v>46077.62740253472</v>
+        <v>46077.79406920139</v>
       </c>
       <c r="C73" s="8">
-        <v>46197.41996670139</v>
+        <v>46197.58663336806</v>
       </c>
       <c r="D73" s="8">
-        <v>46197.41998619213</v>
+        <v>46197.586652858794</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5875,13 +5875,13 @@
         <v>266</v>
       </c>
       <c r="B74" s="5">
-        <v>46077.62740278935</v>
+        <v>46077.794069456024</v>
       </c>
       <c r="C74" s="5">
-        <v>46195.338891064814</v>
+        <v>46195.50555773148</v>
       </c>
       <c r="D74" s="5">
-        <v>46197.41998491898</v>
+        <v>46197.58665158565</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5938,13 +5938,13 @@
         <v>270</v>
       </c>
       <c r="B75" s="8">
-        <v>46077.62740304398</v>
+        <v>46077.79406971065</v>
       </c>
       <c r="C75" s="8">
-        <v>46195.3386822801</v>
+        <v>46195.50534894676</v>
       </c>
       <c r="D75" s="8">
-        <v>46195.33890541666</v>
+        <v>46195.50557208333</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>271</v>
@@ -6003,13 +6003,13 @@
         <v>275</v>
       </c>
       <c r="B76" s="5">
-        <v>46077.627403356484</v>
+        <v>46077.79407002315</v>
       </c>
       <c r="C76" s="5">
-        <v>46195.33873429398</v>
+        <v>46195.50540096065</v>
       </c>
       <c r="D76" s="5">
-        <v>46195.33874953704</v>
+        <v>46195.505416203705</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>276</v>
@@ -6066,11 +6066,11 @@
         <v>278</v>
       </c>
       <c r="B77" s="8">
-        <v>46077.62740362268</v>
+        <v>46077.794070289354</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46092.39547199074</v>
+        <v>46092.562138657406</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>279</v>
@@ -6113,11 +6113,11 @@
         <v>281</v>
       </c>
       <c r="B78" s="5">
-        <v>46077.62740391203</v>
+        <v>46077.794070578704</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46195.33875318287</v>
+        <v>46195.505419849535</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>282</v>
@@ -6176,11 +6176,11 @@
         <v>285</v>
       </c>
       <c r="B79" s="8">
-        <v>46077.627404189814</v>
+        <v>46077.794070856486</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46195.33875326389</v>
+        <v>46195.50541993056</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>286</v>
@@ -6239,11 +6239,11 @@
         <v>288</v>
       </c>
       <c r="B80" s="5">
-        <v>46092.37582547453</v>
+        <v>46092.542492141205</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46092.39547261574</v>
+        <v>46092.56213928241</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>289</v>
@@ -6292,11 +6292,11 @@
         <v>291</v>
       </c>
       <c r="B81" s="8">
-        <v>46092.37586482639</v>
+        <v>46092.542531493054</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46195.33875447916</v>
+        <v>46195.505421145834</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>292</v>
@@ -6355,11 +6355,11 @@
         <v>294</v>
       </c>
       <c r="B82" s="5">
-        <v>46092.376002453704</v>
+        <v>46092.542669120376</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46185.01497164352</v>
+        <v>46185.18163831018</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>295</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-02 14:23 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -1525,13 +1525,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46077.79406804398</v>
+        <v>46077.627401377315</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.723517129634</v>
+        <v>46092.55685046296</v>
       </c>
       <c r="D4" s="5">
-        <v>46109.700906631944</v>
+        <v>46109.53423996527</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1574,13 +1574,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46077.794068449075</v>
+        <v>46077.6274017824</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.723485636576</v>
+        <v>46092.55681896991</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.877652152776</v>
+        <v>46133.71098548611</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1637,13 +1637,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46077.794068738425</v>
+        <v>46077.62740207176</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.72348622685</v>
+        <v>46092.55681956018</v>
       </c>
       <c r="D6" s="5">
-        <v>46092.723518032406</v>
+        <v>46092.55685136574</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1700,13 +1700,13 @@
         <v>38</v>
       </c>
       <c r="B7" s="8">
-        <v>46077.79406903935</v>
+        <v>46077.62740237269</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.72348670139</v>
+        <v>46092.55682003472</v>
       </c>
       <c r="D7" s="8">
-        <v>46092.72351797453</v>
+        <v>46092.55685130787</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>39</v>
@@ -1763,13 +1763,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46077.794069317126</v>
+        <v>46077.62740265046</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.72348717593</v>
+        <v>46092.55682050926</v>
       </c>
       <c r="D8" s="5">
-        <v>46093.75078916667</v>
+        <v>46093.584122500004</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -1826,13 +1826,13 @@
         <v>43</v>
       </c>
       <c r="B9" s="8">
-        <v>46077.79406961806</v>
+        <v>46077.62740295139</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.72348797454</v>
+        <v>46092.556821307866</v>
       </c>
       <c r="D9" s="8">
-        <v>46092.72351859954</v>
+        <v>46092.556851932866</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>44</v>
@@ -1889,13 +1889,13 @@
         <v>45</v>
       </c>
       <c r="B10" s="5">
-        <v>46077.7940699537</v>
+        <v>46077.62740328704</v>
       </c>
       <c r="C10" s="5">
-        <v>46196.78443082176</v>
+        <v>46196.61776415509</v>
       </c>
       <c r="D10" s="5">
-        <v>46196.78444497685</v>
+        <v>46196.61777831019</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -1942,13 +1942,13 @@
         <v>48</v>
       </c>
       <c r="B11" s="8">
-        <v>46077.79407024306</v>
+        <v>46077.62740357639</v>
       </c>
       <c r="C11" s="8">
-        <v>46093.86130311343</v>
+        <v>46093.69463644676</v>
       </c>
       <c r="D11" s="8">
-        <v>46093.86132113426</v>
+        <v>46093.69465446759</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>49</v>
@@ -2007,13 +2007,13 @@
         <v>53</v>
       </c>
       <c r="B12" s="5">
-        <v>46077.79407052083</v>
+        <v>46077.62740385417</v>
       </c>
       <c r="C12" s="5">
-        <v>46196.7844127662</v>
+        <v>46196.61774609954</v>
       </c>
       <c r="D12" s="5">
-        <v>46196.78442833333</v>
+        <v>46196.61776166667</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -2072,13 +2072,13 @@
         <v>59</v>
       </c>
       <c r="B13" s="8">
-        <v>46077.79407081018</v>
+        <v>46077.62740414352</v>
       </c>
       <c r="C13" s="8">
-        <v>46093.75198055556</v>
+        <v>46093.58531388889</v>
       </c>
       <c r="D13" s="8">
-        <v>46108.78193280092</v>
+        <v>46108.615266134264</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>60</v>
@@ -2121,13 +2121,13 @@
         <v>62</v>
       </c>
       <c r="B14" s="5">
-        <v>46077.794067939816</v>
+        <v>46077.627401273145</v>
       </c>
       <c r="C14" s="5">
-        <v>46093.751054803244</v>
+        <v>46093.58438813657</v>
       </c>
       <c r="D14" s="5">
-        <v>46093.75107269676</v>
+        <v>46093.58440603009</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>63</v>
@@ -2186,13 +2186,13 @@
         <v>67</v>
       </c>
       <c r="B15" s="8">
-        <v>46077.79406833333</v>
+        <v>46077.62740166667</v>
       </c>
       <c r="C15" s="8">
-        <v>46093.75108634259</v>
+        <v>46093.58441967593</v>
       </c>
       <c r="D15" s="8">
-        <v>46093.75110184027</v>
+        <v>46093.584435173616</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>68</v>
@@ -2251,13 +2251,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="5">
-        <v>46077.79406863426</v>
+        <v>46077.62740196759</v>
       </c>
       <c r="C16" s="5">
-        <v>46093.75113149306</v>
+        <v>46093.58446482639</v>
       </c>
       <c r="D16" s="5">
-        <v>46093.75114815972</v>
+        <v>46093.58448149306</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>71</v>
@@ -2316,13 +2316,13 @@
         <v>73</v>
       </c>
       <c r="B17" s="8">
-        <v>46077.7940689699</v>
+        <v>46077.627402303246</v>
       </c>
       <c r="C17" s="8">
-        <v>46093.75114832176</v>
+        <v>46093.584481655096</v>
       </c>
       <c r="D17" s="8">
-        <v>46093.75116991898</v>
+        <v>46093.584503252314</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>74</v>
@@ -2381,13 +2381,13 @@
         <v>76</v>
       </c>
       <c r="B18" s="5">
-        <v>46077.794069247684</v>
+        <v>46077.62740258102</v>
       </c>
       <c r="C18" s="5">
-        <v>46093.75196043981</v>
+        <v>46093.58529377315</v>
       </c>
       <c r="D18" s="5">
-        <v>46093.75198266204</v>
+        <v>46093.58531599537</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>77</v>
@@ -2446,13 +2446,13 @@
         <v>80</v>
       </c>
       <c r="B19" s="8">
-        <v>46077.79406954861</v>
+        <v>46077.627402881946</v>
       </c>
       <c r="C19" s="8">
-        <v>46093.87275760417</v>
+        <v>46093.7060909375</v>
       </c>
       <c r="D19" s="8">
-        <v>46132.82815025463</v>
+        <v>46132.66148358796</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>81</v>
@@ -2495,13 +2495,13 @@
         <v>83</v>
       </c>
       <c r="B20" s="5">
-        <v>46077.79407017361</v>
+        <v>46077.627403506944</v>
       </c>
       <c r="C20" s="5">
-        <v>46093.75210856482</v>
+        <v>46093.58544189815</v>
       </c>
       <c r="D20" s="5">
-        <v>46093.75213300926</v>
+        <v>46093.58546634259</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>84</v>
@@ -2560,13 +2560,13 @@
         <v>86</v>
       </c>
       <c r="B21" s="8">
-        <v>46077.794069826385</v>
+        <v>46077.62740315972</v>
       </c>
       <c r="C21" s="8">
-        <v>46093.75212193287</v>
+        <v>46093.585455266206</v>
       </c>
       <c r="D21" s="8">
-        <v>46093.75214115741</v>
+        <v>46093.58547449074</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>87</v>
@@ -2625,13 +2625,13 @@
         <v>89</v>
       </c>
       <c r="B22" s="5">
-        <v>46077.79407089121</v>
+        <v>46077.627404224535</v>
       </c>
       <c r="C22" s="5">
-        <v>46093.75230475694</v>
+        <v>46093.58563809028</v>
       </c>
       <c r="D22" s="5">
-        <v>46093.752320381944</v>
+        <v>46093.58565371528</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>90</v>
@@ -2690,13 +2690,13 @@
         <v>92</v>
       </c>
       <c r="B23" s="8">
-        <v>46077.79407056713</v>
+        <v>46077.627403900464</v>
       </c>
       <c r="C23" s="8">
-        <v>46093.87273884259</v>
+        <v>46093.706072175926</v>
       </c>
       <c r="D23" s="8">
-        <v>46093.87275758102</v>
+        <v>46093.70609091435</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>93</v>
@@ -2755,13 +2755,13 @@
         <v>95</v>
       </c>
       <c r="B24" s="5">
-        <v>46077.79406818287</v>
+        <v>46077.627401516205</v>
       </c>
       <c r="C24" s="5">
-        <v>46093.752348344904</v>
+        <v>46093.58568167824</v>
       </c>
       <c r="D24" s="5">
-        <v>46093.752364050924</v>
+        <v>46093.58569738426</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>96</v>
@@ -2820,13 +2820,13 @@
         <v>98</v>
       </c>
       <c r="B25" s="8">
-        <v>46078.639615821754</v>
+        <v>46078.4729491551</v>
       </c>
       <c r="C25" s="8">
-        <v>46093.75237274305</v>
+        <v>46093.58570607639</v>
       </c>
       <c r="D25" s="8">
-        <v>46093.75238938657</v>
+        <v>46093.58572271991</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>99</v>
@@ -2885,13 +2885,13 @@
         <v>101</v>
       </c>
       <c r="B26" s="5">
-        <v>46078.63966699074</v>
+        <v>46078.47300032407</v>
       </c>
       <c r="C26" s="5">
-        <v>46093.75254957176</v>
+        <v>46093.58588290509</v>
       </c>
       <c r="D26" s="5">
-        <v>46093.752569606484</v>
+        <v>46093.58590293981</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>102</v>
@@ -2950,13 +2950,13 @@
         <v>104</v>
       </c>
       <c r="B27" s="8">
-        <v>46077.79406851852</v>
+        <v>46077.62740185185</v>
       </c>
       <c r="C27" s="8">
-        <v>46175.58050744213</v>
+        <v>46175.413840775465</v>
       </c>
       <c r="D27" s="8">
-        <v>46196.81887502315</v>
+        <v>46196.65220835648</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>105</v>
@@ -3001,13 +3001,13 @@
         <v>108</v>
       </c>
       <c r="B28" s="5">
-        <v>46077.794068773146</v>
+        <v>46077.62740210648</v>
       </c>
       <c r="C28" s="5">
-        <v>46196.81885747685</v>
+        <v>46196.652190810186</v>
       </c>
       <c r="D28" s="5">
-        <v>46196.81885899305</v>
+        <v>46196.65219232639</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>109</v>
@@ -3066,13 +3066,13 @@
         <v>113</v>
       </c>
       <c r="B29" s="8">
-        <v>46077.794069027776</v>
+        <v>46077.62740236111</v>
       </c>
       <c r="C29" s="8">
-        <v>46094.72641315972</v>
+        <v>46094.559746493054</v>
       </c>
       <c r="D29" s="8">
-        <v>46094.726415</v>
+        <v>46094.55974833333</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>114</v>
@@ -3131,13 +3131,13 @@
         <v>118</v>
       </c>
       <c r="B30" s="5">
-        <v>46077.794069270836</v>
+        <v>46077.627402604165</v>
       </c>
       <c r="C30" s="5">
-        <v>46094.726466493055</v>
+        <v>46094.559799826384</v>
       </c>
       <c r="D30" s="5">
-        <v>46094.72646796296</v>
+        <v>46094.559801296295</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>119</v>
@@ -3196,13 +3196,13 @@
         <v>121</v>
       </c>
       <c r="B31" s="8">
-        <v>46077.794069537034</v>
+        <v>46077.62740287037</v>
       </c>
       <c r="C31" s="8">
-        <v>46174.63943520833</v>
+        <v>46174.472768541666</v>
       </c>
       <c r="D31" s="8">
-        <v>46181.69497460648</v>
+        <v>46181.528307939814</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>122</v>
@@ -3261,13 +3261,13 @@
         <v>124</v>
       </c>
       <c r="B32" s="5">
-        <v>46077.79406980324</v>
+        <v>46077.627403136576</v>
       </c>
       <c r="C32" s="5">
-        <v>46094.72762815972</v>
+        <v>46094.56096149306</v>
       </c>
       <c r="D32" s="5">
-        <v>46169.82887452546</v>
+        <v>46169.6622078588</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>125</v>
@@ -3326,13 +3326,13 @@
         <v>127</v>
       </c>
       <c r="B33" s="8">
-        <v>46077.794070081014</v>
+        <v>46077.62740341436</v>
       </c>
       <c r="C33" s="8">
-        <v>46174.638556192134</v>
+        <v>46174.47188952546</v>
       </c>
       <c r="D33" s="8">
-        <v>46174.63855820602</v>
+        <v>46174.47189153935</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>128</v>
@@ -3389,13 +3389,13 @@
         <v>130</v>
       </c>
       <c r="B34" s="5">
-        <v>46077.79407034723</v>
+        <v>46077.627403680555</v>
       </c>
       <c r="C34" s="5">
-        <v>46094.72978902778</v>
+        <v>46094.56312236111</v>
       </c>
       <c r="D34" s="5">
-        <v>46094.729805462965</v>
+        <v>46094.56313879629</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>131</v>
@@ -3454,13 +3454,13 @@
         <v>133</v>
       </c>
       <c r="B35" s="8">
-        <v>46077.794070625</v>
+        <v>46077.62740395834</v>
       </c>
       <c r="C35" s="8">
-        <v>46094.7287584375</v>
+        <v>46094.56209177083</v>
       </c>
       <c r="D35" s="8">
-        <v>46094.72876005787</v>
+        <v>46094.5620933912</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>134</v>
@@ -3519,13 +3519,13 @@
         <v>136</v>
       </c>
       <c r="B36" s="5">
-        <v>46077.79406800926</v>
+        <v>46077.627401342594</v>
       </c>
       <c r="C36" s="5">
-        <v>46094.729772708335</v>
+        <v>46094.56310604166</v>
       </c>
       <c r="D36" s="5">
-        <v>46094.729774259264</v>
+        <v>46094.56310759259</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>137</v>
@@ -3584,13 +3584,13 @@
         <v>139</v>
       </c>
       <c r="B37" s="8">
-        <v>46077.79406834491</v>
+        <v>46077.62740167824</v>
       </c>
       <c r="C37" s="8">
-        <v>46094.72519538194</v>
+        <v>46094.55852871528</v>
       </c>
       <c r="D37" s="8">
-        <v>46130.168979560185</v>
+        <v>46130.00231289351</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>140</v>
@@ -3649,13 +3649,13 @@
         <v>142</v>
       </c>
       <c r="B38" s="5">
-        <v>46077.79406859954</v>
+        <v>46077.62740193287</v>
       </c>
       <c r="C38" s="5">
-        <v>46094.72491252315</v>
+        <v>46094.55824585648</v>
       </c>
       <c r="D38" s="5">
-        <v>46094.72491472222</v>
+        <v>46094.55824805556</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>143</v>
@@ -3714,13 +3714,13 @@
         <v>145</v>
       </c>
       <c r="B39" s="8">
-        <v>46077.79406886574</v>
+        <v>46077.627402199076</v>
       </c>
       <c r="C39" s="8">
-        <v>46094.725131388885</v>
+        <v>46094.55846472223</v>
       </c>
       <c r="D39" s="8">
-        <v>46094.72513274306</v>
+        <v>46094.558466076385</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>146</v>
@@ -3779,13 +3779,13 @@
         <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46077.79406912037</v>
+        <v>46077.627402453705</v>
       </c>
       <c r="C40" s="5">
-        <v>46094.72518011574</v>
+        <v>46094.558513449076</v>
       </c>
       <c r="D40" s="5">
-        <v>46094.7251815162</v>
+        <v>46094.55851484954</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>149</v>
@@ -3844,13 +3844,13 @@
         <v>151</v>
       </c>
       <c r="B41" s="8">
-        <v>46077.79406935185</v>
+        <v>46077.62740268519</v>
       </c>
       <c r="C41" s="8">
-        <v>46094.73862138889</v>
+        <v>46094.571954722225</v>
       </c>
       <c r="D41" s="8">
-        <v>46100.88799495371</v>
+        <v>46100.721328287036</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>152</v>
@@ -3909,13 +3909,13 @@
         <v>156</v>
       </c>
       <c r="B42" s="5">
-        <v>46077.79406958334</v>
+        <v>46077.62740291667</v>
       </c>
       <c r="C42" s="5">
-        <v>46094.73713944445</v>
+        <v>46094.57047277778</v>
       </c>
       <c r="D42" s="5">
-        <v>46094.73822020833</v>
+        <v>46094.57155354167</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>97</v>
@@ -3974,13 +3974,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46077.794069814816</v>
+        <v>46077.627403148144</v>
       </c>
       <c r="C43" s="8">
-        <v>46094.73860646991</v>
+        <v>46094.57193980324</v>
       </c>
       <c r="D43" s="8">
-        <v>46094.73860788194</v>
+        <v>46094.57194121528</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -4039,13 +4039,13 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46078.63983429398</v>
+        <v>46078.473167627315</v>
       </c>
       <c r="C44" s="5">
-        <v>46099.856573240744</v>
+        <v>46099.68990657407</v>
       </c>
       <c r="D44" s="5">
-        <v>46099.856649340276</v>
+        <v>46099.68998267361</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4104,13 +4104,13 @@
         <v>164</v>
       </c>
       <c r="B45" s="8">
-        <v>46078.63989878472</v>
+        <v>46078.473232118056</v>
       </c>
       <c r="C45" s="8">
-        <v>46099.856473287036</v>
+        <v>46099.68980662037</v>
       </c>
       <c r="D45" s="8">
-        <v>46099.85647474537</v>
+        <v>46099.68980807871</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>165</v>
@@ -4159,13 +4159,13 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46078.63997798611</v>
+        <v>46078.473311319445</v>
       </c>
       <c r="C46" s="5">
-        <v>46099.85655642361</v>
+        <v>46099.68988975695</v>
       </c>
       <c r="D46" s="5">
-        <v>46099.85655795139</v>
+        <v>46099.689891284725</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4214,13 +4214,13 @@
         <v>170</v>
       </c>
       <c r="B47" s="8">
-        <v>46078.637812500005</v>
+        <v>46078.47114583333</v>
       </c>
       <c r="C47" s="8">
-        <v>46099.838434375</v>
+        <v>46099.671767708336</v>
       </c>
       <c r="D47" s="8">
-        <v>46121.20616592593</v>
+        <v>46121.03949925926</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>171</v>
@@ -4279,13 +4279,13 @@
         <v>175</v>
       </c>
       <c r="B48" s="5">
-        <v>46078.63791627315</v>
+        <v>46078.47124960648</v>
       </c>
       <c r="C48" s="5">
-        <v>46094.75383356481</v>
+        <v>46094.58716689815</v>
       </c>
       <c r="D48" s="5">
-        <v>46099.53788506944</v>
+        <v>46099.37121840278</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>103</v>
@@ -4340,13 +4340,13 @@
         <v>177</v>
       </c>
       <c r="B49" s="8">
-        <v>46078.63808261574</v>
+        <v>46078.471415949076</v>
       </c>
       <c r="C49" s="8">
-        <v>46099.838418252315</v>
+        <v>46099.67175158564</v>
       </c>
       <c r="D49" s="8">
-        <v>46099.84112896991</v>
+        <v>46099.67446230324</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>178</v>
@@ -4395,13 +4395,13 @@
         <v>181</v>
       </c>
       <c r="B50" s="5">
-        <v>46077.79407005787</v>
+        <v>46077.627403391205</v>
       </c>
       <c r="C50" s="5">
-        <v>46181.69487049768</v>
+        <v>46181.52820383102</v>
       </c>
       <c r="D50" s="5">
-        <v>46181.69488571759</v>
+        <v>46181.528219050924</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>182</v>
@@ -4448,13 +4448,13 @@
         <v>184</v>
       </c>
       <c r="B51" s="8">
-        <v>46077.794070289354</v>
+        <v>46077.62740362268</v>
       </c>
       <c r="C51" s="8">
-        <v>46093.76443008102</v>
+        <v>46093.59776341435</v>
       </c>
       <c r="D51" s="8">
-        <v>46093.76444804398</v>
+        <v>46093.59778137731</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>185</v>
@@ -4513,13 +4513,13 @@
         <v>189</v>
       </c>
       <c r="B52" s="5">
-        <v>46077.79406836806</v>
+        <v>46077.62740170139</v>
       </c>
       <c r="C52" s="5">
-        <v>46097.53332418982</v>
+        <v>46097.36665752315</v>
       </c>
       <c r="D52" s="5">
-        <v>46097.53334462963</v>
+        <v>46097.366677962964</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>190</v>
@@ -4578,13 +4578,13 @@
         <v>195</v>
       </c>
       <c r="B53" s="8">
-        <v>46092.48310565972</v>
+        <v>46092.31643899306</v>
       </c>
       <c r="C53" s="8">
-        <v>46097.533368495366</v>
+        <v>46097.36670182871</v>
       </c>
       <c r="D53" s="8">
-        <v>46097.53338633102</v>
+        <v>46097.36671966435</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>196</v>
@@ -4641,13 +4641,13 @@
         <v>198</v>
       </c>
       <c r="B54" s="5">
-        <v>46092.48319758102</v>
+        <v>46092.31653091435</v>
       </c>
       <c r="C54" s="5">
-        <v>46181.69336679398</v>
+        <v>46181.52670012732</v>
       </c>
       <c r="D54" s="5">
-        <v>46181.694910763894</v>
+        <v>46181.52824409722</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>199</v>
@@ -4706,13 +4706,13 @@
         <v>204</v>
       </c>
       <c r="B55" s="8">
-        <v>46079.615135416665</v>
+        <v>46079.44846875</v>
       </c>
       <c r="C55" s="8">
-        <v>46100.46822152778</v>
+        <v>46100.301554861115</v>
       </c>
       <c r="D55" s="8">
-        <v>46135.75940972222</v>
+        <v>46135.59274305556</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>205</v>
@@ -4755,13 +4755,13 @@
         <v>207</v>
       </c>
       <c r="B56" s="5">
-        <v>46078.74941568287</v>
+        <v>46078.582749016205</v>
       </c>
       <c r="C56" s="5">
-        <v>46100.46820005787</v>
+        <v>46100.301533391204</v>
       </c>
       <c r="D56" s="5">
-        <v>46122.193223229166</v>
+        <v>46122.0265565625</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>206</v>
@@ -4820,13 +4820,13 @@
         <v>211</v>
       </c>
       <c r="B57" s="8">
-        <v>46077.794070601856</v>
+        <v>46077.627403935185</v>
       </c>
       <c r="C57" s="8">
-        <v>46181.69656722222</v>
+        <v>46181.52990055556</v>
       </c>
       <c r="D57" s="8">
-        <v>46181.880506643516</v>
+        <v>46181.71383997685</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>212</v>
@@ -4869,13 +4869,13 @@
         <v>214</v>
       </c>
       <c r="B58" s="5">
-        <v>46077.79407089121</v>
+        <v>46077.627404224535</v>
       </c>
       <c r="C58" s="5">
-        <v>46099.60850569444</v>
+        <v>46099.44183902778</v>
       </c>
       <c r="D58" s="5">
-        <v>46099.60852430556</v>
+        <v>46099.441857638885</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>215</v>
@@ -4934,13 +4934,13 @@
         <v>219</v>
       </c>
       <c r="B59" s="8">
-        <v>46077.79406847223</v>
+        <v>46077.627401805556</v>
       </c>
       <c r="C59" s="8">
-        <v>46181.696550555556</v>
+        <v>46181.529883888885</v>
       </c>
       <c r="D59" s="8">
-        <v>46181.69656733796</v>
+        <v>46181.529900671296</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>57</v>
@@ -4999,13 +4999,13 @@
         <v>221</v>
       </c>
       <c r="B60" s="5">
-        <v>46077.79406880787</v>
+        <v>46077.6274021412</v>
       </c>
       <c r="C60" s="5">
-        <v>46099.608517685185</v>
+        <v>46099.44185101852</v>
       </c>
       <c r="D60" s="5">
-        <v>46108.14717359954</v>
+        <v>46107.98050693287</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>222</v>
@@ -5064,13 +5064,13 @@
         <v>224</v>
       </c>
       <c r="B61" s="8">
-        <v>46077.79406909722</v>
+        <v>46077.62740243056</v>
       </c>
       <c r="C61" s="8">
-        <v>46099.6085555787</v>
+        <v>46099.44188891204</v>
       </c>
       <c r="D61" s="8">
-        <v>46134.20545793981</v>
+        <v>46134.03879127315</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>225</v>
@@ -5129,13 +5129,13 @@
         <v>227</v>
       </c>
       <c r="B62" s="5">
-        <v>46078.64006494213</v>
+        <v>46078.47339827546</v>
       </c>
       <c r="C62" s="5">
-        <v>46099.856724178244</v>
+        <v>46099.69005751157</v>
       </c>
       <c r="D62" s="5">
-        <v>46099.856817928245</v>
+        <v>46099.69015126157</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>228</v>
@@ -5194,13 +5194,13 @@
         <v>230</v>
       </c>
       <c r="B63" s="8">
-        <v>46078.63913549768</v>
+        <v>46078.47246883102</v>
       </c>
       <c r="C63" s="8">
-        <v>46120.627901562504</v>
+        <v>46120.46123489583</v>
       </c>
       <c r="D63" s="8">
-        <v>46120.62792370371</v>
+        <v>46120.46125703704</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>231</v>
@@ -5259,13 +5259,13 @@
         <v>232</v>
       </c>
       <c r="B64" s="5">
-        <v>46077.794069386575</v>
+        <v>46077.62740271991</v>
       </c>
       <c r="C64" s="5">
-        <v>46181.69465158565</v>
+        <v>46181.52798491898</v>
       </c>
       <c r="D64" s="5">
-        <v>46197.58530666667</v>
+        <v>46197.41864</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>233</v>
@@ -5308,13 +5308,13 @@
         <v>235</v>
       </c>
       <c r="B65" s="8">
-        <v>46077.79406965278</v>
+        <v>46077.62740298611</v>
       </c>
       <c r="C65" s="8">
-        <v>46140.56150293982</v>
+        <v>46140.394836273146</v>
       </c>
       <c r="D65" s="8">
-        <v>46181.69470346065</v>
+        <v>46181.528036793985</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>236</v>
@@ -5373,13 +5373,13 @@
         <v>240</v>
       </c>
       <c r="B66" s="5">
-        <v>46077.79406990741</v>
+        <v>46077.62740324074</v>
       </c>
       <c r="C66" s="5">
-        <v>46181.69321660879</v>
+        <v>46181.52654994213</v>
       </c>
       <c r="D66" s="5">
-        <v>46181.69470399305</v>
+        <v>46181.52803732639</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>241</v>
@@ -5438,13 +5438,13 @@
         <v>244</v>
       </c>
       <c r="B67" s="8">
-        <v>46077.79407016204</v>
+        <v>46077.62740349537</v>
       </c>
       <c r="C67" s="8">
-        <v>46113.56087353009</v>
+        <v>46113.39420686342</v>
       </c>
       <c r="D67" s="8">
-        <v>46140.561511990745</v>
+        <v>46140.394845324074</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>245</v>
@@ -5503,13 +5503,13 @@
         <v>247</v>
       </c>
       <c r="B68" s="5">
-        <v>46077.79407042824</v>
+        <v>46077.62740376157</v>
       </c>
       <c r="C68" s="5">
-        <v>46181.69323842593</v>
+        <v>46181.526571759256</v>
       </c>
       <c r="D68" s="5">
-        <v>46181.694704525464</v>
+        <v>46181.52803785879</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>248</v>
@@ -5568,13 +5568,13 @@
         <v>250</v>
       </c>
       <c r="B69" s="8">
-        <v>46078.640146562495</v>
+        <v>46078.47347989584</v>
       </c>
       <c r="C69" s="8">
-        <v>46181.69324881944</v>
+        <v>46181.52658215278</v>
       </c>
       <c r="D69" s="8">
-        <v>46181.694705092596</v>
+        <v>46181.528038425924</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>229</v>
@@ -5633,13 +5633,13 @@
         <v>252</v>
       </c>
       <c r="B70" s="5">
-        <v>46077.79407070602</v>
+        <v>46077.62740403935</v>
       </c>
       <c r="C70" s="5">
-        <v>46181.69329174768</v>
+        <v>46181.526625081024</v>
       </c>
       <c r="D70" s="5">
-        <v>46181.694705671296</v>
+        <v>46181.528039004625</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>202</v>
@@ -5696,13 +5696,13 @@
         <v>255</v>
       </c>
       <c r="B71" s="8">
-        <v>46077.794071296295</v>
+        <v>46077.62740462963</v>
       </c>
       <c r="C71" s="8">
-        <v>46181.693661944446</v>
+        <v>46181.526995277774</v>
       </c>
       <c r="D71" s="8">
-        <v>46181.69470625</v>
+        <v>46181.52803958333</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>203</v>
@@ -5759,13 +5759,13 @@
         <v>257</v>
       </c>
       <c r="B72" s="5">
-        <v>46077.79406888889</v>
+        <v>46077.62740222222</v>
       </c>
       <c r="C72" s="5">
-        <v>46197.586652777776</v>
+        <v>46197.41998611111</v>
       </c>
       <c r="D72" s="5">
-        <v>46197.58666969907</v>
+        <v>46197.42000303241</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>258</v>
@@ -5812,13 +5812,13 @@
         <v>260</v>
       </c>
       <c r="B73" s="8">
-        <v>46077.79406920139</v>
+        <v>46077.62740253472</v>
       </c>
       <c r="C73" s="8">
-        <v>46197.58663336806</v>
+        <v>46197.41996670139</v>
       </c>
       <c r="D73" s="8">
-        <v>46197.586652858794</v>
+        <v>46197.41998619213</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5875,13 +5875,13 @@
         <v>266</v>
       </c>
       <c r="B74" s="5">
-        <v>46077.794069456024</v>
+        <v>46077.62740278935</v>
       </c>
       <c r="C74" s="5">
-        <v>46195.50555773148</v>
+        <v>46195.338891064814</v>
       </c>
       <c r="D74" s="5">
-        <v>46197.58665158565</v>
+        <v>46197.41998491898</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5938,13 +5938,13 @@
         <v>270</v>
       </c>
       <c r="B75" s="8">
-        <v>46077.79406971065</v>
+        <v>46077.62740304398</v>
       </c>
       <c r="C75" s="8">
-        <v>46195.50534894676</v>
+        <v>46195.3386822801</v>
       </c>
       <c r="D75" s="8">
-        <v>46195.50557208333</v>
+        <v>46195.33890541666</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>271</v>
@@ -6003,13 +6003,13 @@
         <v>275</v>
       </c>
       <c r="B76" s="5">
-        <v>46077.79407002315</v>
+        <v>46077.627403356484</v>
       </c>
       <c r="C76" s="5">
-        <v>46195.50540096065</v>
+        <v>46195.33873429398</v>
       </c>
       <c r="D76" s="5">
-        <v>46195.505416203705</v>
+        <v>46195.33874953704</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>276</v>
@@ -6066,11 +6066,11 @@
         <v>278</v>
       </c>
       <c r="B77" s="8">
-        <v>46077.794070289354</v>
+        <v>46077.62740362268</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46092.562138657406</v>
+        <v>46092.39547199074</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>279</v>
@@ -6113,11 +6113,11 @@
         <v>281</v>
       </c>
       <c r="B78" s="5">
-        <v>46077.794070578704</v>
+        <v>46077.62740391203</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46195.505419849535</v>
+        <v>46195.33875318287</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>282</v>
@@ -6176,11 +6176,11 @@
         <v>285</v>
       </c>
       <c r="B79" s="8">
-        <v>46077.794070856486</v>
+        <v>46077.627404189814</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46195.50541993056</v>
+        <v>46195.33875326389</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>286</v>
@@ -6239,11 +6239,11 @@
         <v>288</v>
       </c>
       <c r="B80" s="5">
-        <v>46092.542492141205</v>
+        <v>46092.37582547453</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46092.56213928241</v>
+        <v>46092.39547261574</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>289</v>
@@ -6292,11 +6292,11 @@
         <v>291</v>
       </c>
       <c r="B81" s="8">
-        <v>46092.542531493054</v>
+        <v>46092.37586482639</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46195.505421145834</v>
+        <v>46195.33875447916</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>292</v>
@@ -6355,11 +6355,11 @@
         <v>294</v>
       </c>
       <c r="B82" s="5">
-        <v>46092.542669120376</v>
+        <v>46092.376002453704</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46185.18163831018</v>
+        <v>46185.01497164352</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>295</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-02 15:13 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -1525,13 +1525,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46077.627401377315</v>
+        <v>46077.79406804398</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.55685046296</v>
+        <v>46092.723517129634</v>
       </c>
       <c r="D4" s="5">
-        <v>46109.53423996527</v>
+        <v>46109.700906631944</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1574,13 +1574,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46077.6274017824</v>
+        <v>46077.794068449075</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.55681896991</v>
+        <v>46092.723485636576</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.71098548611</v>
+        <v>46133.877652152776</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1637,13 +1637,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46077.62740207176</v>
+        <v>46077.794068738425</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.55681956018</v>
+        <v>46092.72348622685</v>
       </c>
       <c r="D6" s="5">
-        <v>46092.55685136574</v>
+        <v>46092.723518032406</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1700,13 +1700,13 @@
         <v>38</v>
       </c>
       <c r="B7" s="8">
-        <v>46077.62740237269</v>
+        <v>46077.79406903935</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.55682003472</v>
+        <v>46092.72348670139</v>
       </c>
       <c r="D7" s="8">
-        <v>46092.55685130787</v>
+        <v>46092.72351797453</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>39</v>
@@ -1763,13 +1763,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46077.62740265046</v>
+        <v>46077.794069317126</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.55682050926</v>
+        <v>46092.72348717593</v>
       </c>
       <c r="D8" s="5">
-        <v>46093.584122500004</v>
+        <v>46093.75078916667</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -1826,13 +1826,13 @@
         <v>43</v>
       </c>
       <c r="B9" s="8">
-        <v>46077.62740295139</v>
+        <v>46077.79406961806</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.556821307866</v>
+        <v>46092.72348797454</v>
       </c>
       <c r="D9" s="8">
-        <v>46092.556851932866</v>
+        <v>46092.72351859954</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>44</v>
@@ -1889,13 +1889,13 @@
         <v>45</v>
       </c>
       <c r="B10" s="5">
-        <v>46077.62740328704</v>
+        <v>46077.7940699537</v>
       </c>
       <c r="C10" s="5">
-        <v>46196.61776415509</v>
+        <v>46196.78443082176</v>
       </c>
       <c r="D10" s="5">
-        <v>46196.61777831019</v>
+        <v>46196.78444497685</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -1942,13 +1942,13 @@
         <v>48</v>
       </c>
       <c r="B11" s="8">
-        <v>46077.62740357639</v>
+        <v>46077.79407024306</v>
       </c>
       <c r="C11" s="8">
-        <v>46093.69463644676</v>
+        <v>46093.86130311343</v>
       </c>
       <c r="D11" s="8">
-        <v>46093.69465446759</v>
+        <v>46093.86132113426</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>49</v>
@@ -2007,13 +2007,13 @@
         <v>53</v>
       </c>
       <c r="B12" s="5">
-        <v>46077.62740385417</v>
+        <v>46077.79407052083</v>
       </c>
       <c r="C12" s="5">
-        <v>46196.61774609954</v>
+        <v>46196.7844127662</v>
       </c>
       <c r="D12" s="5">
-        <v>46196.61776166667</v>
+        <v>46196.78442833333</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -2072,13 +2072,13 @@
         <v>59</v>
       </c>
       <c r="B13" s="8">
-        <v>46077.62740414352</v>
+        <v>46077.79407081018</v>
       </c>
       <c r="C13" s="8">
-        <v>46093.58531388889</v>
+        <v>46093.75198055556</v>
       </c>
       <c r="D13" s="8">
-        <v>46108.615266134264</v>
+        <v>46108.78193280092</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>60</v>
@@ -2121,13 +2121,13 @@
         <v>62</v>
       </c>
       <c r="B14" s="5">
-        <v>46077.627401273145</v>
+        <v>46077.794067939816</v>
       </c>
       <c r="C14" s="5">
-        <v>46093.58438813657</v>
+        <v>46093.751054803244</v>
       </c>
       <c r="D14" s="5">
-        <v>46093.58440603009</v>
+        <v>46093.75107269676</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>63</v>
@@ -2186,13 +2186,13 @@
         <v>67</v>
       </c>
       <c r="B15" s="8">
-        <v>46077.62740166667</v>
+        <v>46077.79406833333</v>
       </c>
       <c r="C15" s="8">
-        <v>46093.58441967593</v>
+        <v>46093.75108634259</v>
       </c>
       <c r="D15" s="8">
-        <v>46093.584435173616</v>
+        <v>46093.75110184027</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>68</v>
@@ -2251,13 +2251,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="5">
-        <v>46077.62740196759</v>
+        <v>46077.79406863426</v>
       </c>
       <c r="C16" s="5">
-        <v>46093.58446482639</v>
+        <v>46093.75113149306</v>
       </c>
       <c r="D16" s="5">
-        <v>46093.58448149306</v>
+        <v>46093.75114815972</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>71</v>
@@ -2316,13 +2316,13 @@
         <v>73</v>
       </c>
       <c r="B17" s="8">
-        <v>46077.627402303246</v>
+        <v>46077.7940689699</v>
       </c>
       <c r="C17" s="8">
-        <v>46093.584481655096</v>
+        <v>46093.75114832176</v>
       </c>
       <c r="D17" s="8">
-        <v>46093.584503252314</v>
+        <v>46093.75116991898</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>74</v>
@@ -2381,13 +2381,13 @@
         <v>76</v>
       </c>
       <c r="B18" s="5">
-        <v>46077.62740258102</v>
+        <v>46077.794069247684</v>
       </c>
       <c r="C18" s="5">
-        <v>46093.58529377315</v>
+        <v>46093.75196043981</v>
       </c>
       <c r="D18" s="5">
-        <v>46093.58531599537</v>
+        <v>46093.75198266204</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>77</v>
@@ -2446,13 +2446,13 @@
         <v>80</v>
       </c>
       <c r="B19" s="8">
-        <v>46077.627402881946</v>
+        <v>46077.79406954861</v>
       </c>
       <c r="C19" s="8">
-        <v>46093.7060909375</v>
+        <v>46093.87275760417</v>
       </c>
       <c r="D19" s="8">
-        <v>46132.66148358796</v>
+        <v>46132.82815025463</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>81</v>
@@ -2495,13 +2495,13 @@
         <v>83</v>
       </c>
       <c r="B20" s="5">
-        <v>46077.627403506944</v>
+        <v>46077.79407017361</v>
       </c>
       <c r="C20" s="5">
-        <v>46093.58544189815</v>
+        <v>46093.75210856482</v>
       </c>
       <c r="D20" s="5">
-        <v>46093.58546634259</v>
+        <v>46093.75213300926</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>84</v>
@@ -2560,13 +2560,13 @@
         <v>86</v>
       </c>
       <c r="B21" s="8">
-        <v>46077.62740315972</v>
+        <v>46077.794069826385</v>
       </c>
       <c r="C21" s="8">
-        <v>46093.585455266206</v>
+        <v>46093.75212193287</v>
       </c>
       <c r="D21" s="8">
-        <v>46093.58547449074</v>
+        <v>46093.75214115741</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>87</v>
@@ -2625,13 +2625,13 @@
         <v>89</v>
       </c>
       <c r="B22" s="5">
-        <v>46077.627404224535</v>
+        <v>46077.79407089121</v>
       </c>
       <c r="C22" s="5">
-        <v>46093.58563809028</v>
+        <v>46093.75230475694</v>
       </c>
       <c r="D22" s="5">
-        <v>46093.58565371528</v>
+        <v>46093.752320381944</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>90</v>
@@ -2690,13 +2690,13 @@
         <v>92</v>
       </c>
       <c r="B23" s="8">
-        <v>46077.627403900464</v>
+        <v>46077.79407056713</v>
       </c>
       <c r="C23" s="8">
-        <v>46093.706072175926</v>
+        <v>46093.87273884259</v>
       </c>
       <c r="D23" s="8">
-        <v>46093.70609091435</v>
+        <v>46093.87275758102</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>93</v>
@@ -2755,13 +2755,13 @@
         <v>95</v>
       </c>
       <c r="B24" s="5">
-        <v>46077.627401516205</v>
+        <v>46077.79406818287</v>
       </c>
       <c r="C24" s="5">
-        <v>46093.58568167824</v>
+        <v>46093.752348344904</v>
       </c>
       <c r="D24" s="5">
-        <v>46093.58569738426</v>
+        <v>46093.752364050924</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>96</v>
@@ -2820,13 +2820,13 @@
         <v>98</v>
       </c>
       <c r="B25" s="8">
-        <v>46078.4729491551</v>
+        <v>46078.639615821754</v>
       </c>
       <c r="C25" s="8">
-        <v>46093.58570607639</v>
+        <v>46093.75237274305</v>
       </c>
       <c r="D25" s="8">
-        <v>46093.58572271991</v>
+        <v>46093.75238938657</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>99</v>
@@ -2885,13 +2885,13 @@
         <v>101</v>
       </c>
       <c r="B26" s="5">
-        <v>46078.47300032407</v>
+        <v>46078.63966699074</v>
       </c>
       <c r="C26" s="5">
-        <v>46093.58588290509</v>
+        <v>46093.75254957176</v>
       </c>
       <c r="D26" s="5">
-        <v>46093.58590293981</v>
+        <v>46093.752569606484</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>102</v>
@@ -2950,13 +2950,13 @@
         <v>104</v>
       </c>
       <c r="B27" s="8">
-        <v>46077.62740185185</v>
+        <v>46077.79406851852</v>
       </c>
       <c r="C27" s="8">
-        <v>46175.413840775465</v>
+        <v>46175.58050744213</v>
       </c>
       <c r="D27" s="8">
-        <v>46196.65220835648</v>
+        <v>46196.81887502315</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>105</v>
@@ -3001,13 +3001,13 @@
         <v>108</v>
       </c>
       <c r="B28" s="5">
-        <v>46077.62740210648</v>
+        <v>46077.794068773146</v>
       </c>
       <c r="C28" s="5">
-        <v>46196.652190810186</v>
+        <v>46196.81885747685</v>
       </c>
       <c r="D28" s="5">
-        <v>46196.65219232639</v>
+        <v>46196.81885899305</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>109</v>
@@ -3066,13 +3066,13 @@
         <v>113</v>
       </c>
       <c r="B29" s="8">
-        <v>46077.62740236111</v>
+        <v>46077.794069027776</v>
       </c>
       <c r="C29" s="8">
-        <v>46094.559746493054</v>
+        <v>46094.72641315972</v>
       </c>
       <c r="D29" s="8">
-        <v>46094.55974833333</v>
+        <v>46094.726415</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>114</v>
@@ -3131,13 +3131,13 @@
         <v>118</v>
       </c>
       <c r="B30" s="5">
-        <v>46077.627402604165</v>
+        <v>46077.794069270836</v>
       </c>
       <c r="C30" s="5">
-        <v>46094.559799826384</v>
+        <v>46094.726466493055</v>
       </c>
       <c r="D30" s="5">
-        <v>46094.559801296295</v>
+        <v>46094.72646796296</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>119</v>
@@ -3196,13 +3196,13 @@
         <v>121</v>
       </c>
       <c r="B31" s="8">
-        <v>46077.62740287037</v>
+        <v>46077.794069537034</v>
       </c>
       <c r="C31" s="8">
-        <v>46174.472768541666</v>
+        <v>46174.63943520833</v>
       </c>
       <c r="D31" s="8">
-        <v>46181.528307939814</v>
+        <v>46181.69497460648</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>122</v>
@@ -3261,13 +3261,13 @@
         <v>124</v>
       </c>
       <c r="B32" s="5">
-        <v>46077.627403136576</v>
+        <v>46077.79406980324</v>
       </c>
       <c r="C32" s="5">
-        <v>46094.56096149306</v>
+        <v>46094.72762815972</v>
       </c>
       <c r="D32" s="5">
-        <v>46169.6622078588</v>
+        <v>46169.82887452546</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>125</v>
@@ -3326,13 +3326,13 @@
         <v>127</v>
       </c>
       <c r="B33" s="8">
-        <v>46077.62740341436</v>
+        <v>46077.794070081014</v>
       </c>
       <c r="C33" s="8">
-        <v>46174.47188952546</v>
+        <v>46174.638556192134</v>
       </c>
       <c r="D33" s="8">
-        <v>46174.47189153935</v>
+        <v>46174.63855820602</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>128</v>
@@ -3389,13 +3389,13 @@
         <v>130</v>
       </c>
       <c r="B34" s="5">
-        <v>46077.627403680555</v>
+        <v>46077.79407034723</v>
       </c>
       <c r="C34" s="5">
-        <v>46094.56312236111</v>
+        <v>46094.72978902778</v>
       </c>
       <c r="D34" s="5">
-        <v>46094.56313879629</v>
+        <v>46094.729805462965</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>131</v>
@@ -3454,13 +3454,13 @@
         <v>133</v>
       </c>
       <c r="B35" s="8">
-        <v>46077.62740395834</v>
+        <v>46077.794070625</v>
       </c>
       <c r="C35" s="8">
-        <v>46094.56209177083</v>
+        <v>46094.7287584375</v>
       </c>
       <c r="D35" s="8">
-        <v>46094.5620933912</v>
+        <v>46094.72876005787</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>134</v>
@@ -3519,13 +3519,13 @@
         <v>136</v>
       </c>
       <c r="B36" s="5">
-        <v>46077.627401342594</v>
+        <v>46077.79406800926</v>
       </c>
       <c r="C36" s="5">
-        <v>46094.56310604166</v>
+        <v>46094.729772708335</v>
       </c>
       <c r="D36" s="5">
-        <v>46094.56310759259</v>
+        <v>46094.729774259264</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>137</v>
@@ -3584,13 +3584,13 @@
         <v>139</v>
       </c>
       <c r="B37" s="8">
-        <v>46077.62740167824</v>
+        <v>46077.79406834491</v>
       </c>
       <c r="C37" s="8">
-        <v>46094.55852871528</v>
+        <v>46094.72519538194</v>
       </c>
       <c r="D37" s="8">
-        <v>46130.00231289351</v>
+        <v>46130.168979560185</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>140</v>
@@ -3649,13 +3649,13 @@
         <v>142</v>
       </c>
       <c r="B38" s="5">
-        <v>46077.62740193287</v>
+        <v>46077.79406859954</v>
       </c>
       <c r="C38" s="5">
-        <v>46094.55824585648</v>
+        <v>46094.72491252315</v>
       </c>
       <c r="D38" s="5">
-        <v>46094.55824805556</v>
+        <v>46094.72491472222</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>143</v>
@@ -3714,13 +3714,13 @@
         <v>145</v>
       </c>
       <c r="B39" s="8">
-        <v>46077.627402199076</v>
+        <v>46077.79406886574</v>
       </c>
       <c r="C39" s="8">
-        <v>46094.55846472223</v>
+        <v>46094.725131388885</v>
       </c>
       <c r="D39" s="8">
-        <v>46094.558466076385</v>
+        <v>46094.72513274306</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>146</v>
@@ -3779,13 +3779,13 @@
         <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46077.627402453705</v>
+        <v>46077.79406912037</v>
       </c>
       <c r="C40" s="5">
-        <v>46094.558513449076</v>
+        <v>46094.72518011574</v>
       </c>
       <c r="D40" s="5">
-        <v>46094.55851484954</v>
+        <v>46094.7251815162</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>149</v>
@@ -3844,13 +3844,13 @@
         <v>151</v>
       </c>
       <c r="B41" s="8">
-        <v>46077.62740268519</v>
+        <v>46077.79406935185</v>
       </c>
       <c r="C41" s="8">
-        <v>46094.571954722225</v>
+        <v>46094.73862138889</v>
       </c>
       <c r="D41" s="8">
-        <v>46100.721328287036</v>
+        <v>46100.88799495371</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>152</v>
@@ -3909,13 +3909,13 @@
         <v>156</v>
       </c>
       <c r="B42" s="5">
-        <v>46077.62740291667</v>
+        <v>46077.79406958334</v>
       </c>
       <c r="C42" s="5">
-        <v>46094.57047277778</v>
+        <v>46094.73713944445</v>
       </c>
       <c r="D42" s="5">
-        <v>46094.57155354167</v>
+        <v>46094.73822020833</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>97</v>
@@ -3974,13 +3974,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46077.627403148144</v>
+        <v>46077.794069814816</v>
       </c>
       <c r="C43" s="8">
-        <v>46094.57193980324</v>
+        <v>46094.73860646991</v>
       </c>
       <c r="D43" s="8">
-        <v>46094.57194121528</v>
+        <v>46094.73860788194</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -4039,13 +4039,13 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46078.473167627315</v>
+        <v>46078.63983429398</v>
       </c>
       <c r="C44" s="5">
-        <v>46099.68990657407</v>
+        <v>46099.856573240744</v>
       </c>
       <c r="D44" s="5">
-        <v>46099.68998267361</v>
+        <v>46099.856649340276</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4104,13 +4104,13 @@
         <v>164</v>
       </c>
       <c r="B45" s="8">
-        <v>46078.473232118056</v>
+        <v>46078.63989878472</v>
       </c>
       <c r="C45" s="8">
-        <v>46099.68980662037</v>
+        <v>46099.856473287036</v>
       </c>
       <c r="D45" s="8">
-        <v>46099.68980807871</v>
+        <v>46099.85647474537</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>165</v>
@@ -4159,13 +4159,13 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46078.473311319445</v>
+        <v>46078.63997798611</v>
       </c>
       <c r="C46" s="5">
-        <v>46099.68988975695</v>
+        <v>46099.85655642361</v>
       </c>
       <c r="D46" s="5">
-        <v>46099.689891284725</v>
+        <v>46099.85655795139</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4214,13 +4214,13 @@
         <v>170</v>
       </c>
       <c r="B47" s="8">
-        <v>46078.47114583333</v>
+        <v>46078.637812500005</v>
       </c>
       <c r="C47" s="8">
-        <v>46099.671767708336</v>
+        <v>46099.838434375</v>
       </c>
       <c r="D47" s="8">
-        <v>46121.03949925926</v>
+        <v>46121.20616592593</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>171</v>
@@ -4279,13 +4279,13 @@
         <v>175</v>
       </c>
       <c r="B48" s="5">
-        <v>46078.47124960648</v>
+        <v>46078.63791627315</v>
       </c>
       <c r="C48" s="5">
-        <v>46094.58716689815</v>
+        <v>46094.75383356481</v>
       </c>
       <c r="D48" s="5">
-        <v>46099.37121840278</v>
+        <v>46099.53788506944</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>103</v>
@@ -4340,13 +4340,13 @@
         <v>177</v>
       </c>
       <c r="B49" s="8">
-        <v>46078.471415949076</v>
+        <v>46078.63808261574</v>
       </c>
       <c r="C49" s="8">
-        <v>46099.67175158564</v>
+        <v>46099.838418252315</v>
       </c>
       <c r="D49" s="8">
-        <v>46099.67446230324</v>
+        <v>46099.84112896991</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>178</v>
@@ -4395,13 +4395,13 @@
         <v>181</v>
       </c>
       <c r="B50" s="5">
-        <v>46077.627403391205</v>
+        <v>46077.79407005787</v>
       </c>
       <c r="C50" s="5">
-        <v>46181.52820383102</v>
+        <v>46181.69487049768</v>
       </c>
       <c r="D50" s="5">
-        <v>46181.528219050924</v>
+        <v>46181.69488571759</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>182</v>
@@ -4448,13 +4448,13 @@
         <v>184</v>
       </c>
       <c r="B51" s="8">
-        <v>46077.62740362268</v>
+        <v>46077.794070289354</v>
       </c>
       <c r="C51" s="8">
-        <v>46093.59776341435</v>
+        <v>46093.76443008102</v>
       </c>
       <c r="D51" s="8">
-        <v>46093.59778137731</v>
+        <v>46093.76444804398</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>185</v>
@@ -4513,13 +4513,13 @@
         <v>189</v>
       </c>
       <c r="B52" s="5">
-        <v>46077.62740170139</v>
+        <v>46077.79406836806</v>
       </c>
       <c r="C52" s="5">
-        <v>46097.36665752315</v>
+        <v>46097.53332418982</v>
       </c>
       <c r="D52" s="5">
-        <v>46097.366677962964</v>
+        <v>46097.53334462963</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>190</v>
@@ -4578,13 +4578,13 @@
         <v>195</v>
       </c>
       <c r="B53" s="8">
-        <v>46092.31643899306</v>
+        <v>46092.48310565972</v>
       </c>
       <c r="C53" s="8">
-        <v>46097.36670182871</v>
+        <v>46097.533368495366</v>
       </c>
       <c r="D53" s="8">
-        <v>46097.36671966435</v>
+        <v>46097.53338633102</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>196</v>
@@ -4641,13 +4641,13 @@
         <v>198</v>
       </c>
       <c r="B54" s="5">
-        <v>46092.31653091435</v>
+        <v>46092.48319758102</v>
       </c>
       <c r="C54" s="5">
-        <v>46181.52670012732</v>
+        <v>46181.69336679398</v>
       </c>
       <c r="D54" s="5">
-        <v>46181.52824409722</v>
+        <v>46181.694910763894</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>199</v>
@@ -4706,13 +4706,13 @@
         <v>204</v>
       </c>
       <c r="B55" s="8">
-        <v>46079.44846875</v>
+        <v>46079.615135416665</v>
       </c>
       <c r="C55" s="8">
-        <v>46100.301554861115</v>
+        <v>46100.46822152778</v>
       </c>
       <c r="D55" s="8">
-        <v>46135.59274305556</v>
+        <v>46135.75940972222</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>205</v>
@@ -4755,13 +4755,13 @@
         <v>207</v>
       </c>
       <c r="B56" s="5">
-        <v>46078.582749016205</v>
+        <v>46078.74941568287</v>
       </c>
       <c r="C56" s="5">
-        <v>46100.301533391204</v>
+        <v>46100.46820005787</v>
       </c>
       <c r="D56" s="5">
-        <v>46122.0265565625</v>
+        <v>46122.193223229166</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>206</v>
@@ -4820,13 +4820,13 @@
         <v>211</v>
       </c>
       <c r="B57" s="8">
-        <v>46077.627403935185</v>
+        <v>46077.794070601856</v>
       </c>
       <c r="C57" s="8">
-        <v>46181.52990055556</v>
+        <v>46181.69656722222</v>
       </c>
       <c r="D57" s="8">
-        <v>46181.71383997685</v>
+        <v>46181.880506643516</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>212</v>
@@ -4869,13 +4869,13 @@
         <v>214</v>
       </c>
       <c r="B58" s="5">
-        <v>46077.627404224535</v>
+        <v>46077.79407089121</v>
       </c>
       <c r="C58" s="5">
-        <v>46099.44183902778</v>
+        <v>46099.60850569444</v>
       </c>
       <c r="D58" s="5">
-        <v>46099.441857638885</v>
+        <v>46099.60852430556</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>215</v>
@@ -4934,13 +4934,13 @@
         <v>219</v>
       </c>
       <c r="B59" s="8">
-        <v>46077.627401805556</v>
+        <v>46077.79406847223</v>
       </c>
       <c r="C59" s="8">
-        <v>46181.529883888885</v>
+        <v>46181.696550555556</v>
       </c>
       <c r="D59" s="8">
-        <v>46181.529900671296</v>
+        <v>46181.69656733796</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>57</v>
@@ -4999,13 +4999,13 @@
         <v>221</v>
       </c>
       <c r="B60" s="5">
-        <v>46077.6274021412</v>
+        <v>46077.79406880787</v>
       </c>
       <c r="C60" s="5">
-        <v>46099.44185101852</v>
+        <v>46099.608517685185</v>
       </c>
       <c r="D60" s="5">
-        <v>46107.98050693287</v>
+        <v>46108.14717359954</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>222</v>
@@ -5064,13 +5064,13 @@
         <v>224</v>
       </c>
       <c r="B61" s="8">
-        <v>46077.62740243056</v>
+        <v>46077.79406909722</v>
       </c>
       <c r="C61" s="8">
-        <v>46099.44188891204</v>
+        <v>46099.6085555787</v>
       </c>
       <c r="D61" s="8">
-        <v>46134.03879127315</v>
+        <v>46134.20545793981</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>225</v>
@@ -5129,13 +5129,13 @@
         <v>227</v>
       </c>
       <c r="B62" s="5">
-        <v>46078.47339827546</v>
+        <v>46078.64006494213</v>
       </c>
       <c r="C62" s="5">
-        <v>46099.69005751157</v>
+        <v>46099.856724178244</v>
       </c>
       <c r="D62" s="5">
-        <v>46099.69015126157</v>
+        <v>46099.856817928245</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>228</v>
@@ -5194,13 +5194,13 @@
         <v>230</v>
       </c>
       <c r="B63" s="8">
-        <v>46078.47246883102</v>
+        <v>46078.63913549768</v>
       </c>
       <c r="C63" s="8">
-        <v>46120.46123489583</v>
+        <v>46120.627901562504</v>
       </c>
       <c r="D63" s="8">
-        <v>46120.46125703704</v>
+        <v>46120.62792370371</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>231</v>
@@ -5259,13 +5259,13 @@
         <v>232</v>
       </c>
       <c r="B64" s="5">
-        <v>46077.62740271991</v>
+        <v>46077.794069386575</v>
       </c>
       <c r="C64" s="5">
-        <v>46181.52798491898</v>
+        <v>46181.69465158565</v>
       </c>
       <c r="D64" s="5">
-        <v>46197.41864</v>
+        <v>46197.58530666667</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>233</v>
@@ -5308,13 +5308,13 @@
         <v>235</v>
       </c>
       <c r="B65" s="8">
-        <v>46077.62740298611</v>
+        <v>46077.79406965278</v>
       </c>
       <c r="C65" s="8">
-        <v>46140.394836273146</v>
+        <v>46140.56150293982</v>
       </c>
       <c r="D65" s="8">
-        <v>46181.528036793985</v>
+        <v>46181.69470346065</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>236</v>
@@ -5373,13 +5373,13 @@
         <v>240</v>
       </c>
       <c r="B66" s="5">
-        <v>46077.62740324074</v>
+        <v>46077.79406990741</v>
       </c>
       <c r="C66" s="5">
-        <v>46181.52654994213</v>
+        <v>46181.69321660879</v>
       </c>
       <c r="D66" s="5">
-        <v>46181.52803732639</v>
+        <v>46181.69470399305</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>241</v>
@@ -5438,13 +5438,13 @@
         <v>244</v>
       </c>
       <c r="B67" s="8">
-        <v>46077.62740349537</v>
+        <v>46077.79407016204</v>
       </c>
       <c r="C67" s="8">
-        <v>46113.39420686342</v>
+        <v>46113.56087353009</v>
       </c>
       <c r="D67" s="8">
-        <v>46140.394845324074</v>
+        <v>46140.561511990745</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>245</v>
@@ -5503,13 +5503,13 @@
         <v>247</v>
       </c>
       <c r="B68" s="5">
-        <v>46077.62740376157</v>
+        <v>46077.79407042824</v>
       </c>
       <c r="C68" s="5">
-        <v>46181.526571759256</v>
+        <v>46181.69323842593</v>
       </c>
       <c r="D68" s="5">
-        <v>46181.52803785879</v>
+        <v>46181.694704525464</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>248</v>
@@ -5568,13 +5568,13 @@
         <v>250</v>
       </c>
       <c r="B69" s="8">
-        <v>46078.47347989584</v>
+        <v>46078.640146562495</v>
       </c>
       <c r="C69" s="8">
-        <v>46181.52658215278</v>
+        <v>46181.69324881944</v>
       </c>
       <c r="D69" s="8">
-        <v>46181.528038425924</v>
+        <v>46181.694705092596</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>229</v>
@@ -5633,13 +5633,13 @@
         <v>252</v>
       </c>
       <c r="B70" s="5">
-        <v>46077.62740403935</v>
+        <v>46077.79407070602</v>
       </c>
       <c r="C70" s="5">
-        <v>46181.526625081024</v>
+        <v>46181.69329174768</v>
       </c>
       <c r="D70" s="5">
-        <v>46181.528039004625</v>
+        <v>46181.694705671296</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>202</v>
@@ -5696,13 +5696,13 @@
         <v>255</v>
       </c>
       <c r="B71" s="8">
-        <v>46077.62740462963</v>
+        <v>46077.794071296295</v>
       </c>
       <c r="C71" s="8">
-        <v>46181.526995277774</v>
+        <v>46181.693661944446</v>
       </c>
       <c r="D71" s="8">
-        <v>46181.52803958333</v>
+        <v>46181.69470625</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>203</v>
@@ -5759,13 +5759,13 @@
         <v>257</v>
       </c>
       <c r="B72" s="5">
-        <v>46077.62740222222</v>
+        <v>46077.79406888889</v>
       </c>
       <c r="C72" s="5">
-        <v>46197.41998611111</v>
+        <v>46197.586652777776</v>
       </c>
       <c r="D72" s="5">
-        <v>46197.42000303241</v>
+        <v>46197.58666969907</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>258</v>
@@ -5812,13 +5812,13 @@
         <v>260</v>
       </c>
       <c r="B73" s="8">
-        <v>46077.62740253472</v>
+        <v>46077.79406920139</v>
       </c>
       <c r="C73" s="8">
-        <v>46197.41996670139</v>
+        <v>46197.58663336806</v>
       </c>
       <c r="D73" s="8">
-        <v>46197.41998619213</v>
+        <v>46197.586652858794</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5875,13 +5875,13 @@
         <v>266</v>
       </c>
       <c r="B74" s="5">
-        <v>46077.62740278935</v>
+        <v>46077.794069456024</v>
       </c>
       <c r="C74" s="5">
-        <v>46195.338891064814</v>
+        <v>46195.50555773148</v>
       </c>
       <c r="D74" s="5">
-        <v>46197.41998491898</v>
+        <v>46197.58665158565</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5938,13 +5938,13 @@
         <v>270</v>
       </c>
       <c r="B75" s="8">
-        <v>46077.62740304398</v>
+        <v>46077.79406971065</v>
       </c>
       <c r="C75" s="8">
-        <v>46195.3386822801</v>
+        <v>46195.50534894676</v>
       </c>
       <c r="D75" s="8">
-        <v>46195.33890541666</v>
+        <v>46195.50557208333</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>271</v>
@@ -6003,13 +6003,13 @@
         <v>275</v>
       </c>
       <c r="B76" s="5">
-        <v>46077.627403356484</v>
+        <v>46077.79407002315</v>
       </c>
       <c r="C76" s="5">
-        <v>46195.33873429398</v>
+        <v>46195.50540096065</v>
       </c>
       <c r="D76" s="5">
-        <v>46195.33874953704</v>
+        <v>46195.505416203705</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>276</v>
@@ -6066,11 +6066,11 @@
         <v>278</v>
       </c>
       <c r="B77" s="8">
-        <v>46077.62740362268</v>
+        <v>46077.794070289354</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46092.39547199074</v>
+        <v>46092.562138657406</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>279</v>
@@ -6113,11 +6113,11 @@
         <v>281</v>
       </c>
       <c r="B78" s="5">
-        <v>46077.62740391203</v>
+        <v>46077.794070578704</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46195.33875318287</v>
+        <v>46195.505419849535</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>282</v>
@@ -6176,11 +6176,11 @@
         <v>285</v>
       </c>
       <c r="B79" s="8">
-        <v>46077.627404189814</v>
+        <v>46077.794070856486</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46195.33875326389</v>
+        <v>46195.50541993056</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>286</v>
@@ -6239,11 +6239,11 @@
         <v>288</v>
       </c>
       <c r="B80" s="5">
-        <v>46092.37582547453</v>
+        <v>46092.542492141205</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46092.39547261574</v>
+        <v>46092.56213928241</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>289</v>
@@ -6292,11 +6292,11 @@
         <v>291</v>
       </c>
       <c r="B81" s="8">
-        <v>46092.37586482639</v>
+        <v>46092.542531493054</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46195.33875447916</v>
+        <v>46195.505421145834</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>292</v>
@@ -6355,11 +6355,11 @@
         <v>294</v>
       </c>
       <c r="B82" s="5">
-        <v>46092.376002453704</v>
+        <v>46092.542669120376</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46185.01497164352</v>
+        <v>46185.18163831018</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>295</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-08 12:26 Chile
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -1525,13 +1525,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46077.79406804398</v>
+        <v>46077.627401377315</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.723517129634</v>
+        <v>46092.55685046296</v>
       </c>
       <c r="D4" s="5">
-        <v>46109.700906631944</v>
+        <v>46109.53423996527</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1574,13 +1574,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46077.794068449075</v>
+        <v>46077.6274017824</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.723485636576</v>
+        <v>46092.55681896991</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.877652152776</v>
+        <v>46133.71098548611</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1637,13 +1637,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46077.794068738425</v>
+        <v>46077.62740207176</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.72348622685</v>
+        <v>46092.55681956018</v>
       </c>
       <c r="D6" s="5">
-        <v>46092.723518032406</v>
+        <v>46092.55685136574</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1700,13 +1700,13 @@
         <v>38</v>
       </c>
       <c r="B7" s="8">
-        <v>46077.79406903935</v>
+        <v>46077.62740237269</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.72348670139</v>
+        <v>46092.55682003472</v>
       </c>
       <c r="D7" s="8">
-        <v>46092.72351797453</v>
+        <v>46092.55685130787</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>39</v>
@@ -1763,13 +1763,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46077.794069317126</v>
+        <v>46077.62740265046</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.72348717593</v>
+        <v>46092.55682050926</v>
       </c>
       <c r="D8" s="5">
-        <v>46093.75078916667</v>
+        <v>46093.584122500004</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -1826,13 +1826,13 @@
         <v>43</v>
       </c>
       <c r="B9" s="8">
-        <v>46077.79406961806</v>
+        <v>46077.62740295139</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.72348797454</v>
+        <v>46092.556821307866</v>
       </c>
       <c r="D9" s="8">
-        <v>46092.72351859954</v>
+        <v>46092.556851932866</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>44</v>
@@ -1889,13 +1889,13 @@
         <v>45</v>
       </c>
       <c r="B10" s="5">
-        <v>46077.7940699537</v>
+        <v>46077.62740328704</v>
       </c>
       <c r="C10" s="5">
-        <v>46196.78443082176</v>
+        <v>46196.61776415509</v>
       </c>
       <c r="D10" s="5">
-        <v>46196.78444497685</v>
+        <v>46196.61777831019</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -1942,13 +1942,13 @@
         <v>48</v>
       </c>
       <c r="B11" s="8">
-        <v>46077.79407024306</v>
+        <v>46077.62740357639</v>
       </c>
       <c r="C11" s="8">
-        <v>46093.86130311343</v>
+        <v>46093.69463644676</v>
       </c>
       <c r="D11" s="8">
-        <v>46093.86132113426</v>
+        <v>46093.69465446759</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>49</v>
@@ -2007,13 +2007,13 @@
         <v>53</v>
       </c>
       <c r="B12" s="5">
-        <v>46077.79407052083</v>
+        <v>46077.62740385417</v>
       </c>
       <c r="C12" s="5">
-        <v>46196.7844127662</v>
+        <v>46196.61774609954</v>
       </c>
       <c r="D12" s="5">
-        <v>46196.78442833333</v>
+        <v>46196.61776166667</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -2072,13 +2072,13 @@
         <v>59</v>
       </c>
       <c r="B13" s="8">
-        <v>46077.79407081018</v>
+        <v>46077.62740414352</v>
       </c>
       <c r="C13" s="8">
-        <v>46093.75198055556</v>
+        <v>46093.58531388889</v>
       </c>
       <c r="D13" s="8">
-        <v>46108.78193280092</v>
+        <v>46108.615266134264</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>60</v>
@@ -2121,13 +2121,13 @@
         <v>62</v>
       </c>
       <c r="B14" s="5">
-        <v>46077.794067939816</v>
+        <v>46077.627401273145</v>
       </c>
       <c r="C14" s="5">
-        <v>46093.751054803244</v>
+        <v>46093.58438813657</v>
       </c>
       <c r="D14" s="5">
-        <v>46093.75107269676</v>
+        <v>46093.58440603009</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>63</v>
@@ -2186,13 +2186,13 @@
         <v>67</v>
       </c>
       <c r="B15" s="8">
-        <v>46077.79406833333</v>
+        <v>46077.62740166667</v>
       </c>
       <c r="C15" s="8">
-        <v>46093.75108634259</v>
+        <v>46093.58441967593</v>
       </c>
       <c r="D15" s="8">
-        <v>46093.75110184027</v>
+        <v>46093.584435173616</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>68</v>
@@ -2251,13 +2251,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="5">
-        <v>46077.79406863426</v>
+        <v>46077.62740196759</v>
       </c>
       <c r="C16" s="5">
-        <v>46093.75113149306</v>
+        <v>46093.58446482639</v>
       </c>
       <c r="D16" s="5">
-        <v>46093.75114815972</v>
+        <v>46093.58448149306</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>71</v>
@@ -2316,13 +2316,13 @@
         <v>73</v>
       </c>
       <c r="B17" s="8">
-        <v>46077.7940689699</v>
+        <v>46077.627402303246</v>
       </c>
       <c r="C17" s="8">
-        <v>46093.75114832176</v>
+        <v>46093.584481655096</v>
       </c>
       <c r="D17" s="8">
-        <v>46093.75116991898</v>
+        <v>46093.584503252314</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>74</v>
@@ -2381,13 +2381,13 @@
         <v>76</v>
       </c>
       <c r="B18" s="5">
-        <v>46077.794069247684</v>
+        <v>46077.62740258102</v>
       </c>
       <c r="C18" s="5">
-        <v>46093.75196043981</v>
+        <v>46093.58529377315</v>
       </c>
       <c r="D18" s="5">
-        <v>46093.75198266204</v>
+        <v>46093.58531599537</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>77</v>
@@ -2446,13 +2446,13 @@
         <v>80</v>
       </c>
       <c r="B19" s="8">
-        <v>46077.79406954861</v>
+        <v>46077.627402881946</v>
       </c>
       <c r="C19" s="8">
-        <v>46093.87275760417</v>
+        <v>46093.7060909375</v>
       </c>
       <c r="D19" s="8">
-        <v>46132.82815025463</v>
+        <v>46132.66148358796</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>81</v>
@@ -2495,13 +2495,13 @@
         <v>83</v>
       </c>
       <c r="B20" s="5">
-        <v>46077.79407017361</v>
+        <v>46077.627403506944</v>
       </c>
       <c r="C20" s="5">
-        <v>46093.75210856482</v>
+        <v>46093.58544189815</v>
       </c>
       <c r="D20" s="5">
-        <v>46093.75213300926</v>
+        <v>46093.58546634259</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>84</v>
@@ -2560,13 +2560,13 @@
         <v>86</v>
       </c>
       <c r="B21" s="8">
-        <v>46077.794069826385</v>
+        <v>46077.62740315972</v>
       </c>
       <c r="C21" s="8">
-        <v>46093.75212193287</v>
+        <v>46093.585455266206</v>
       </c>
       <c r="D21" s="8">
-        <v>46093.75214115741</v>
+        <v>46093.58547449074</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>87</v>
@@ -2625,13 +2625,13 @@
         <v>89</v>
       </c>
       <c r="B22" s="5">
-        <v>46077.79407089121</v>
+        <v>46077.627404224535</v>
       </c>
       <c r="C22" s="5">
-        <v>46093.75230475694</v>
+        <v>46093.58563809028</v>
       </c>
       <c r="D22" s="5">
-        <v>46093.752320381944</v>
+        <v>46093.58565371528</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>90</v>
@@ -2690,13 +2690,13 @@
         <v>92</v>
       </c>
       <c r="B23" s="8">
-        <v>46077.79407056713</v>
+        <v>46077.627403900464</v>
       </c>
       <c r="C23" s="8">
-        <v>46093.87273884259</v>
+        <v>46093.706072175926</v>
       </c>
       <c r="D23" s="8">
-        <v>46093.87275758102</v>
+        <v>46093.70609091435</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>93</v>
@@ -2755,13 +2755,13 @@
         <v>95</v>
       </c>
       <c r="B24" s="5">
-        <v>46077.79406818287</v>
+        <v>46077.627401516205</v>
       </c>
       <c r="C24" s="5">
-        <v>46093.752348344904</v>
+        <v>46093.58568167824</v>
       </c>
       <c r="D24" s="5">
-        <v>46093.752364050924</v>
+        <v>46093.58569738426</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>96</v>
@@ -2820,13 +2820,13 @@
         <v>98</v>
       </c>
       <c r="B25" s="8">
-        <v>46078.639615821754</v>
+        <v>46078.4729491551</v>
       </c>
       <c r="C25" s="8">
-        <v>46093.75237274305</v>
+        <v>46093.58570607639</v>
       </c>
       <c r="D25" s="8">
-        <v>46093.75238938657</v>
+        <v>46093.58572271991</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>99</v>
@@ -2885,13 +2885,13 @@
         <v>101</v>
       </c>
       <c r="B26" s="5">
-        <v>46078.63966699074</v>
+        <v>46078.47300032407</v>
       </c>
       <c r="C26" s="5">
-        <v>46093.75254957176</v>
+        <v>46093.58588290509</v>
       </c>
       <c r="D26" s="5">
-        <v>46093.752569606484</v>
+        <v>46093.58590293981</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>102</v>
@@ -2950,13 +2950,13 @@
         <v>104</v>
       </c>
       <c r="B27" s="8">
-        <v>46077.79406851852</v>
+        <v>46077.62740185185</v>
       </c>
       <c r="C27" s="8">
-        <v>46175.58050744213</v>
+        <v>46175.413840775465</v>
       </c>
       <c r="D27" s="8">
-        <v>46196.81887502315</v>
+        <v>46196.65220835648</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>105</v>
@@ -3001,13 +3001,13 @@
         <v>108</v>
       </c>
       <c r="B28" s="5">
-        <v>46077.794068773146</v>
+        <v>46077.62740210648</v>
       </c>
       <c r="C28" s="5">
-        <v>46196.81885747685</v>
+        <v>46196.652190810186</v>
       </c>
       <c r="D28" s="5">
-        <v>46196.81885899305</v>
+        <v>46196.65219232639</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>109</v>
@@ -3066,13 +3066,13 @@
         <v>113</v>
       </c>
       <c r="B29" s="8">
-        <v>46077.794069027776</v>
+        <v>46077.62740236111</v>
       </c>
       <c r="C29" s="8">
-        <v>46094.72641315972</v>
+        <v>46094.559746493054</v>
       </c>
       <c r="D29" s="8">
-        <v>46094.726415</v>
+        <v>46094.55974833333</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>114</v>
@@ -3131,13 +3131,13 @@
         <v>118</v>
       </c>
       <c r="B30" s="5">
-        <v>46077.794069270836</v>
+        <v>46077.627402604165</v>
       </c>
       <c r="C30" s="5">
-        <v>46094.726466493055</v>
+        <v>46094.559799826384</v>
       </c>
       <c r="D30" s="5">
-        <v>46094.72646796296</v>
+        <v>46094.559801296295</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>119</v>
@@ -3196,13 +3196,13 @@
         <v>121</v>
       </c>
       <c r="B31" s="8">
-        <v>46077.794069537034</v>
+        <v>46077.62740287037</v>
       </c>
       <c r="C31" s="8">
-        <v>46174.63943520833</v>
+        <v>46174.472768541666</v>
       </c>
       <c r="D31" s="8">
-        <v>46181.69497460648</v>
+        <v>46181.528307939814</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>122</v>
@@ -3261,13 +3261,13 @@
         <v>124</v>
       </c>
       <c r="B32" s="5">
-        <v>46077.79406980324</v>
+        <v>46077.627403136576</v>
       </c>
       <c r="C32" s="5">
-        <v>46094.72762815972</v>
+        <v>46094.56096149306</v>
       </c>
       <c r="D32" s="5">
-        <v>46169.82887452546</v>
+        <v>46169.6622078588</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>125</v>
@@ -3326,13 +3326,13 @@
         <v>127</v>
       </c>
       <c r="B33" s="8">
-        <v>46077.794070081014</v>
+        <v>46077.62740341436</v>
       </c>
       <c r="C33" s="8">
-        <v>46174.638556192134</v>
+        <v>46174.47188952546</v>
       </c>
       <c r="D33" s="8">
-        <v>46174.63855820602</v>
+        <v>46174.47189153935</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>128</v>
@@ -3389,13 +3389,13 @@
         <v>130</v>
       </c>
       <c r="B34" s="5">
-        <v>46077.79407034723</v>
+        <v>46077.627403680555</v>
       </c>
       <c r="C34" s="5">
-        <v>46094.72978902778</v>
+        <v>46094.56312236111</v>
       </c>
       <c r="D34" s="5">
-        <v>46094.729805462965</v>
+        <v>46094.56313879629</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>131</v>
@@ -3454,13 +3454,13 @@
         <v>133</v>
       </c>
       <c r="B35" s="8">
-        <v>46077.794070625</v>
+        <v>46077.62740395834</v>
       </c>
       <c r="C35" s="8">
-        <v>46094.7287584375</v>
+        <v>46094.56209177083</v>
       </c>
       <c r="D35" s="8">
-        <v>46094.72876005787</v>
+        <v>46094.5620933912</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>134</v>
@@ -3519,13 +3519,13 @@
         <v>136</v>
       </c>
       <c r="B36" s="5">
-        <v>46077.79406800926</v>
+        <v>46077.627401342594</v>
       </c>
       <c r="C36" s="5">
-        <v>46094.729772708335</v>
+        <v>46094.56310604166</v>
       </c>
       <c r="D36" s="5">
-        <v>46094.729774259264</v>
+        <v>46094.56310759259</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>137</v>
@@ -3584,13 +3584,13 @@
         <v>139</v>
       </c>
       <c r="B37" s="8">
-        <v>46077.79406834491</v>
+        <v>46077.62740167824</v>
       </c>
       <c r="C37" s="8">
-        <v>46094.72519538194</v>
+        <v>46094.55852871528</v>
       </c>
       <c r="D37" s="8">
-        <v>46130.168979560185</v>
+        <v>46130.00231289351</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>140</v>
@@ -3649,13 +3649,13 @@
         <v>142</v>
       </c>
       <c r="B38" s="5">
-        <v>46077.79406859954</v>
+        <v>46077.62740193287</v>
       </c>
       <c r="C38" s="5">
-        <v>46094.72491252315</v>
+        <v>46094.55824585648</v>
       </c>
       <c r="D38" s="5">
-        <v>46094.72491472222</v>
+        <v>46094.55824805556</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>143</v>
@@ -3714,13 +3714,13 @@
         <v>145</v>
       </c>
       <c r="B39" s="8">
-        <v>46077.79406886574</v>
+        <v>46077.627402199076</v>
       </c>
       <c r="C39" s="8">
-        <v>46094.725131388885</v>
+        <v>46094.55846472223</v>
       </c>
       <c r="D39" s="8">
-        <v>46094.72513274306</v>
+        <v>46094.558466076385</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>146</v>
@@ -3779,13 +3779,13 @@
         <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46077.79406912037</v>
+        <v>46077.627402453705</v>
       </c>
       <c r="C40" s="5">
-        <v>46094.72518011574</v>
+        <v>46094.558513449076</v>
       </c>
       <c r="D40" s="5">
-        <v>46094.7251815162</v>
+        <v>46094.55851484954</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>149</v>
@@ -3844,13 +3844,13 @@
         <v>151</v>
       </c>
       <c r="B41" s="8">
-        <v>46077.79406935185</v>
+        <v>46077.62740268519</v>
       </c>
       <c r="C41" s="8">
-        <v>46094.73862138889</v>
+        <v>46094.571954722225</v>
       </c>
       <c r="D41" s="8">
-        <v>46100.88799495371</v>
+        <v>46100.721328287036</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>152</v>
@@ -3909,13 +3909,13 @@
         <v>156</v>
       </c>
       <c r="B42" s="5">
-        <v>46077.79406958334</v>
+        <v>46077.62740291667</v>
       </c>
       <c r="C42" s="5">
-        <v>46094.73713944445</v>
+        <v>46094.57047277778</v>
       </c>
       <c r="D42" s="5">
-        <v>46094.73822020833</v>
+        <v>46094.57155354167</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>97</v>
@@ -3974,13 +3974,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46077.794069814816</v>
+        <v>46077.627403148144</v>
       </c>
       <c r="C43" s="8">
-        <v>46094.73860646991</v>
+        <v>46094.57193980324</v>
       </c>
       <c r="D43" s="8">
-        <v>46094.73860788194</v>
+        <v>46094.57194121528</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -4039,13 +4039,13 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46078.63983429398</v>
+        <v>46078.473167627315</v>
       </c>
       <c r="C44" s="5">
-        <v>46099.856573240744</v>
+        <v>46099.68990657407</v>
       </c>
       <c r="D44" s="5">
-        <v>46099.856649340276</v>
+        <v>46099.68998267361</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4104,13 +4104,13 @@
         <v>164</v>
       </c>
       <c r="B45" s="8">
-        <v>46078.63989878472</v>
+        <v>46078.473232118056</v>
       </c>
       <c r="C45" s="8">
-        <v>46099.856473287036</v>
+        <v>46099.68980662037</v>
       </c>
       <c r="D45" s="8">
-        <v>46099.85647474537</v>
+        <v>46099.68980807871</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>165</v>
@@ -4159,13 +4159,13 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46078.63997798611</v>
+        <v>46078.473311319445</v>
       </c>
       <c r="C46" s="5">
-        <v>46099.85655642361</v>
+        <v>46099.68988975695</v>
       </c>
       <c r="D46" s="5">
-        <v>46099.85655795139</v>
+        <v>46099.689891284725</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4214,13 +4214,13 @@
         <v>170</v>
       </c>
       <c r="B47" s="8">
-        <v>46078.637812500005</v>
+        <v>46078.47114583333</v>
       </c>
       <c r="C47" s="8">
-        <v>46099.838434375</v>
+        <v>46099.671767708336</v>
       </c>
       <c r="D47" s="8">
-        <v>46121.20616592593</v>
+        <v>46121.03949925926</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>171</v>
@@ -4279,13 +4279,13 @@
         <v>175</v>
       </c>
       <c r="B48" s="5">
-        <v>46078.63791627315</v>
+        <v>46078.47124960648</v>
       </c>
       <c r="C48" s="5">
-        <v>46094.75383356481</v>
+        <v>46094.58716689815</v>
       </c>
       <c r="D48" s="5">
-        <v>46099.53788506944</v>
+        <v>46099.37121840278</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>103</v>
@@ -4340,13 +4340,13 @@
         <v>177</v>
       </c>
       <c r="B49" s="8">
-        <v>46078.63808261574</v>
+        <v>46078.471415949076</v>
       </c>
       <c r="C49" s="8">
-        <v>46099.838418252315</v>
+        <v>46099.67175158564</v>
       </c>
       <c r="D49" s="8">
-        <v>46099.84112896991</v>
+        <v>46099.67446230324</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>178</v>
@@ -4395,13 +4395,13 @@
         <v>181</v>
       </c>
       <c r="B50" s="5">
-        <v>46077.79407005787</v>
+        <v>46077.627403391205</v>
       </c>
       <c r="C50" s="5">
-        <v>46181.69487049768</v>
+        <v>46181.52820383102</v>
       </c>
       <c r="D50" s="5">
-        <v>46181.69488571759</v>
+        <v>46181.528219050924</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>182</v>
@@ -4448,13 +4448,13 @@
         <v>184</v>
       </c>
       <c r="B51" s="8">
-        <v>46077.794070289354</v>
+        <v>46077.62740362268</v>
       </c>
       <c r="C51" s="8">
-        <v>46093.76443008102</v>
+        <v>46093.59776341435</v>
       </c>
       <c r="D51" s="8">
-        <v>46093.76444804398</v>
+        <v>46093.59778137731</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>185</v>
@@ -4513,13 +4513,13 @@
         <v>189</v>
       </c>
       <c r="B52" s="5">
-        <v>46077.79406836806</v>
+        <v>46077.62740170139</v>
       </c>
       <c r="C52" s="5">
-        <v>46097.53332418982</v>
+        <v>46097.36665752315</v>
       </c>
       <c r="D52" s="5">
-        <v>46097.53334462963</v>
+        <v>46097.366677962964</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>190</v>
@@ -4578,13 +4578,13 @@
         <v>195</v>
       </c>
       <c r="B53" s="8">
-        <v>46092.48310565972</v>
+        <v>46092.31643899306</v>
       </c>
       <c r="C53" s="8">
-        <v>46097.533368495366</v>
+        <v>46097.36670182871</v>
       </c>
       <c r="D53" s="8">
-        <v>46097.53338633102</v>
+        <v>46097.36671966435</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>196</v>
@@ -4641,13 +4641,13 @@
         <v>198</v>
       </c>
       <c r="B54" s="5">
-        <v>46092.48319758102</v>
+        <v>46092.31653091435</v>
       </c>
       <c r="C54" s="5">
-        <v>46181.69336679398</v>
+        <v>46181.52670012732</v>
       </c>
       <c r="D54" s="5">
-        <v>46181.694910763894</v>
+        <v>46181.52824409722</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>199</v>
@@ -4706,13 +4706,13 @@
         <v>204</v>
       </c>
       <c r="B55" s="8">
-        <v>46079.615135416665</v>
+        <v>46079.44846875</v>
       </c>
       <c r="C55" s="8">
-        <v>46100.46822152778</v>
+        <v>46100.301554861115</v>
       </c>
       <c r="D55" s="8">
-        <v>46135.75940972222</v>
+        <v>46135.59274305556</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>205</v>
@@ -4755,13 +4755,13 @@
         <v>207</v>
       </c>
       <c r="B56" s="5">
-        <v>46078.74941568287</v>
+        <v>46078.582749016205</v>
       </c>
       <c r="C56" s="5">
-        <v>46100.46820005787</v>
+        <v>46100.301533391204</v>
       </c>
       <c r="D56" s="5">
-        <v>46122.193223229166</v>
+        <v>46122.0265565625</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>206</v>
@@ -4820,13 +4820,13 @@
         <v>211</v>
       </c>
       <c r="B57" s="8">
-        <v>46077.794070601856</v>
+        <v>46077.627403935185</v>
       </c>
       <c r="C57" s="8">
-        <v>46181.69656722222</v>
+        <v>46181.52990055556</v>
       </c>
       <c r="D57" s="8">
-        <v>46181.880506643516</v>
+        <v>46181.71383997685</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>212</v>
@@ -4869,13 +4869,13 @@
         <v>214</v>
       </c>
       <c r="B58" s="5">
-        <v>46077.79407089121</v>
+        <v>46077.627404224535</v>
       </c>
       <c r="C58" s="5">
-        <v>46099.60850569444</v>
+        <v>46099.44183902778</v>
       </c>
       <c r="D58" s="5">
-        <v>46099.60852430556</v>
+        <v>46099.441857638885</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>215</v>
@@ -4934,13 +4934,13 @@
         <v>219</v>
       </c>
       <c r="B59" s="8">
-        <v>46077.79406847223</v>
+        <v>46077.627401805556</v>
       </c>
       <c r="C59" s="8">
-        <v>46181.696550555556</v>
+        <v>46181.529883888885</v>
       </c>
       <c r="D59" s="8">
-        <v>46181.69656733796</v>
+        <v>46181.529900671296</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>57</v>
@@ -4999,13 +4999,13 @@
         <v>221</v>
       </c>
       <c r="B60" s="5">
-        <v>46077.79406880787</v>
+        <v>46077.6274021412</v>
       </c>
       <c r="C60" s="5">
-        <v>46099.608517685185</v>
+        <v>46099.44185101852</v>
       </c>
       <c r="D60" s="5">
-        <v>46108.14717359954</v>
+        <v>46107.98050693287</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>222</v>
@@ -5064,13 +5064,13 @@
         <v>224</v>
       </c>
       <c r="B61" s="8">
-        <v>46077.79406909722</v>
+        <v>46077.62740243056</v>
       </c>
       <c r="C61" s="8">
-        <v>46099.6085555787</v>
+        <v>46099.44188891204</v>
       </c>
       <c r="D61" s="8">
-        <v>46134.20545793981</v>
+        <v>46134.03879127315</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>225</v>
@@ -5129,13 +5129,13 @@
         <v>227</v>
       </c>
       <c r="B62" s="5">
-        <v>46078.64006494213</v>
+        <v>46078.47339827546</v>
       </c>
       <c r="C62" s="5">
-        <v>46099.856724178244</v>
+        <v>46099.69005751157</v>
       </c>
       <c r="D62" s="5">
-        <v>46099.856817928245</v>
+        <v>46099.69015126157</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>228</v>
@@ -5194,13 +5194,13 @@
         <v>230</v>
       </c>
       <c r="B63" s="8">
-        <v>46078.63913549768</v>
+        <v>46078.47246883102</v>
       </c>
       <c r="C63" s="8">
-        <v>46120.627901562504</v>
+        <v>46120.46123489583</v>
       </c>
       <c r="D63" s="8">
-        <v>46120.62792370371</v>
+        <v>46120.46125703704</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>231</v>
@@ -5259,13 +5259,13 @@
         <v>232</v>
       </c>
       <c r="B64" s="5">
-        <v>46077.794069386575</v>
+        <v>46077.62740271991</v>
       </c>
       <c r="C64" s="5">
-        <v>46181.69465158565</v>
+        <v>46181.52798491898</v>
       </c>
       <c r="D64" s="5">
-        <v>46197.58530666667</v>
+        <v>46197.41864</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>233</v>
@@ -5308,13 +5308,13 @@
         <v>235</v>
       </c>
       <c r="B65" s="8">
-        <v>46077.79406965278</v>
+        <v>46077.62740298611</v>
       </c>
       <c r="C65" s="8">
-        <v>46140.56150293982</v>
+        <v>46140.394836273146</v>
       </c>
       <c r="D65" s="8">
-        <v>46181.69470346065</v>
+        <v>46181.528036793985</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>236</v>
@@ -5373,13 +5373,13 @@
         <v>240</v>
       </c>
       <c r="B66" s="5">
-        <v>46077.79406990741</v>
+        <v>46077.62740324074</v>
       </c>
       <c r="C66" s="5">
-        <v>46181.69321660879</v>
+        <v>46181.52654994213</v>
       </c>
       <c r="D66" s="5">
-        <v>46181.69470399305</v>
+        <v>46181.52803732639</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>241</v>
@@ -5438,13 +5438,13 @@
         <v>244</v>
       </c>
       <c r="B67" s="8">
-        <v>46077.79407016204</v>
+        <v>46077.62740349537</v>
       </c>
       <c r="C67" s="8">
-        <v>46113.56087353009</v>
+        <v>46113.39420686342</v>
       </c>
       <c r="D67" s="8">
-        <v>46140.561511990745</v>
+        <v>46140.394845324074</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>245</v>
@@ -5503,13 +5503,13 @@
         <v>247</v>
       </c>
       <c r="B68" s="5">
-        <v>46077.79407042824</v>
+        <v>46077.62740376157</v>
       </c>
       <c r="C68" s="5">
-        <v>46181.69323842593</v>
+        <v>46181.526571759256</v>
       </c>
       <c r="D68" s="5">
-        <v>46181.694704525464</v>
+        <v>46181.52803785879</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>248</v>
@@ -5568,13 +5568,13 @@
         <v>250</v>
       </c>
       <c r="B69" s="8">
-        <v>46078.640146562495</v>
+        <v>46078.47347989584</v>
       </c>
       <c r="C69" s="8">
-        <v>46181.69324881944</v>
+        <v>46181.52658215278</v>
       </c>
       <c r="D69" s="8">
-        <v>46181.694705092596</v>
+        <v>46181.528038425924</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>229</v>
@@ -5633,13 +5633,13 @@
         <v>252</v>
       </c>
       <c r="B70" s="5">
-        <v>46077.79407070602</v>
+        <v>46077.62740403935</v>
       </c>
       <c r="C70" s="5">
-        <v>46181.69329174768</v>
+        <v>46181.526625081024</v>
       </c>
       <c r="D70" s="5">
-        <v>46181.694705671296</v>
+        <v>46181.528039004625</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>202</v>
@@ -5696,13 +5696,13 @@
         <v>255</v>
       </c>
       <c r="B71" s="8">
-        <v>46077.794071296295</v>
+        <v>46077.62740462963</v>
       </c>
       <c r="C71" s="8">
-        <v>46181.693661944446</v>
+        <v>46181.526995277774</v>
       </c>
       <c r="D71" s="8">
-        <v>46181.69470625</v>
+        <v>46181.52803958333</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>203</v>
@@ -5759,13 +5759,13 @@
         <v>257</v>
       </c>
       <c r="B72" s="5">
-        <v>46077.79406888889</v>
+        <v>46077.62740222222</v>
       </c>
       <c r="C72" s="5">
-        <v>46197.586652777776</v>
+        <v>46197.41998611111</v>
       </c>
       <c r="D72" s="5">
-        <v>46197.58666969907</v>
+        <v>46197.42000303241</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>258</v>
@@ -5812,13 +5812,13 @@
         <v>260</v>
       </c>
       <c r="B73" s="8">
-        <v>46077.79406920139</v>
+        <v>46077.62740253472</v>
       </c>
       <c r="C73" s="8">
-        <v>46197.58663336806</v>
+        <v>46197.41996670139</v>
       </c>
       <c r="D73" s="8">
-        <v>46197.586652858794</v>
+        <v>46197.41998619213</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5875,13 +5875,13 @@
         <v>266</v>
       </c>
       <c r="B74" s="5">
-        <v>46077.794069456024</v>
+        <v>46077.62740278935</v>
       </c>
       <c r="C74" s="5">
-        <v>46195.50555773148</v>
+        <v>46195.338891064814</v>
       </c>
       <c r="D74" s="5">
-        <v>46197.58665158565</v>
+        <v>46197.41998491898</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5938,13 +5938,13 @@
         <v>270</v>
       </c>
       <c r="B75" s="8">
-        <v>46077.79406971065</v>
+        <v>46077.62740304398</v>
       </c>
       <c r="C75" s="8">
-        <v>46195.50534894676</v>
+        <v>46195.3386822801</v>
       </c>
       <c r="D75" s="8">
-        <v>46195.50557208333</v>
+        <v>46195.33890541666</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>271</v>
@@ -6003,13 +6003,13 @@
         <v>275</v>
       </c>
       <c r="B76" s="5">
-        <v>46077.79407002315</v>
+        <v>46077.627403356484</v>
       </c>
       <c r="C76" s="5">
-        <v>46195.50540096065</v>
+        <v>46195.33873429398</v>
       </c>
       <c r="D76" s="5">
-        <v>46195.505416203705</v>
+        <v>46195.33874953704</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>276</v>
@@ -6066,11 +6066,11 @@
         <v>278</v>
       </c>
       <c r="B77" s="8">
-        <v>46077.794070289354</v>
+        <v>46077.62740362268</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46092.562138657406</v>
+        <v>46092.39547199074</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>279</v>
@@ -6113,11 +6113,11 @@
         <v>281</v>
       </c>
       <c r="B78" s="5">
-        <v>46077.794070578704</v>
+        <v>46077.62740391203</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46195.505419849535</v>
+        <v>46195.33875318287</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>282</v>
@@ -6176,11 +6176,11 @@
         <v>285</v>
       </c>
       <c r="B79" s="8">
-        <v>46077.794070856486</v>
+        <v>46077.627404189814</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46195.50541993056</v>
+        <v>46195.33875326389</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>286</v>
@@ -6239,11 +6239,11 @@
         <v>288</v>
       </c>
       <c r="B80" s="5">
-        <v>46092.542492141205</v>
+        <v>46092.37582547453</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46092.56213928241</v>
+        <v>46092.39547261574</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>289</v>
@@ -6292,11 +6292,11 @@
         <v>291</v>
       </c>
       <c r="B81" s="8">
-        <v>46092.542531493054</v>
+        <v>46092.37586482639</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46195.505421145834</v>
+        <v>46195.33875447916</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>292</v>
@@ -6355,11 +6355,11 @@
         <v>294</v>
       </c>
       <c r="B82" s="5">
-        <v>46092.542669120376</v>
+        <v>46092.376002453704</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46185.18163831018</v>
+        <v>46185.01497164352</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>295</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-08 19:08 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -1525,13 +1525,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46077.627401377315</v>
+        <v>46077.79406804398</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.55685046296</v>
+        <v>46092.723517129634</v>
       </c>
       <c r="D4" s="5">
-        <v>46109.53423996527</v>
+        <v>46109.700906631944</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1574,13 +1574,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46077.6274017824</v>
+        <v>46077.794068449075</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.55681896991</v>
+        <v>46092.723485636576</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.71098548611</v>
+        <v>46133.877652152776</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1637,13 +1637,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46077.62740207176</v>
+        <v>46077.794068738425</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.55681956018</v>
+        <v>46092.72348622685</v>
       </c>
       <c r="D6" s="5">
-        <v>46092.55685136574</v>
+        <v>46092.723518032406</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1700,13 +1700,13 @@
         <v>38</v>
       </c>
       <c r="B7" s="8">
-        <v>46077.62740237269</v>
+        <v>46077.79406903935</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.55682003472</v>
+        <v>46092.72348670139</v>
       </c>
       <c r="D7" s="8">
-        <v>46092.55685130787</v>
+        <v>46092.72351797453</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>39</v>
@@ -1763,13 +1763,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46077.62740265046</v>
+        <v>46077.794069317126</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.55682050926</v>
+        <v>46092.72348717593</v>
       </c>
       <c r="D8" s="5">
-        <v>46093.584122500004</v>
+        <v>46093.75078916667</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -1826,13 +1826,13 @@
         <v>43</v>
       </c>
       <c r="B9" s="8">
-        <v>46077.62740295139</v>
+        <v>46077.79406961806</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.556821307866</v>
+        <v>46092.72348797454</v>
       </c>
       <c r="D9" s="8">
-        <v>46092.556851932866</v>
+        <v>46092.72351859954</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>44</v>
@@ -1889,13 +1889,13 @@
         <v>45</v>
       </c>
       <c r="B10" s="5">
-        <v>46077.62740328704</v>
+        <v>46077.7940699537</v>
       </c>
       <c r="C10" s="5">
-        <v>46196.61776415509</v>
+        <v>46196.78443082176</v>
       </c>
       <c r="D10" s="5">
-        <v>46196.61777831019</v>
+        <v>46196.78444497685</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -1942,13 +1942,13 @@
         <v>48</v>
       </c>
       <c r="B11" s="8">
-        <v>46077.62740357639</v>
+        <v>46077.79407024306</v>
       </c>
       <c r="C11" s="8">
-        <v>46093.69463644676</v>
+        <v>46093.86130311343</v>
       </c>
       <c r="D11" s="8">
-        <v>46093.69465446759</v>
+        <v>46093.86132113426</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>49</v>
@@ -2007,13 +2007,13 @@
         <v>53</v>
       </c>
       <c r="B12" s="5">
-        <v>46077.62740385417</v>
+        <v>46077.79407052083</v>
       </c>
       <c r="C12" s="5">
-        <v>46196.61774609954</v>
+        <v>46196.7844127662</v>
       </c>
       <c r="D12" s="5">
-        <v>46196.61776166667</v>
+        <v>46196.78442833333</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -2072,13 +2072,13 @@
         <v>59</v>
       </c>
       <c r="B13" s="8">
-        <v>46077.62740414352</v>
+        <v>46077.79407081018</v>
       </c>
       <c r="C13" s="8">
-        <v>46093.58531388889</v>
+        <v>46093.75198055556</v>
       </c>
       <c r="D13" s="8">
-        <v>46108.615266134264</v>
+        <v>46108.78193280092</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>60</v>
@@ -2121,13 +2121,13 @@
         <v>62</v>
       </c>
       <c r="B14" s="5">
-        <v>46077.627401273145</v>
+        <v>46077.794067939816</v>
       </c>
       <c r="C14" s="5">
-        <v>46093.58438813657</v>
+        <v>46093.751054803244</v>
       </c>
       <c r="D14" s="5">
-        <v>46093.58440603009</v>
+        <v>46093.75107269676</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>63</v>
@@ -2186,13 +2186,13 @@
         <v>67</v>
       </c>
       <c r="B15" s="8">
-        <v>46077.62740166667</v>
+        <v>46077.79406833333</v>
       </c>
       <c r="C15" s="8">
-        <v>46093.58441967593</v>
+        <v>46093.75108634259</v>
       </c>
       <c r="D15" s="8">
-        <v>46093.584435173616</v>
+        <v>46093.75110184027</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>68</v>
@@ -2251,13 +2251,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="5">
-        <v>46077.62740196759</v>
+        <v>46077.79406863426</v>
       </c>
       <c r="C16" s="5">
-        <v>46093.58446482639</v>
+        <v>46093.75113149306</v>
       </c>
       <c r="D16" s="5">
-        <v>46093.58448149306</v>
+        <v>46093.75114815972</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>71</v>
@@ -2316,13 +2316,13 @@
         <v>73</v>
       </c>
       <c r="B17" s="8">
-        <v>46077.627402303246</v>
+        <v>46077.7940689699</v>
       </c>
       <c r="C17" s="8">
-        <v>46093.584481655096</v>
+        <v>46093.75114832176</v>
       </c>
       <c r="D17" s="8">
-        <v>46093.584503252314</v>
+        <v>46093.75116991898</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>74</v>
@@ -2381,13 +2381,13 @@
         <v>76</v>
       </c>
       <c r="B18" s="5">
-        <v>46077.62740258102</v>
+        <v>46077.794069247684</v>
       </c>
       <c r="C18" s="5">
-        <v>46093.58529377315</v>
+        <v>46093.75196043981</v>
       </c>
       <c r="D18" s="5">
-        <v>46093.58531599537</v>
+        <v>46093.75198266204</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>77</v>
@@ -2446,13 +2446,13 @@
         <v>80</v>
       </c>
       <c r="B19" s="8">
-        <v>46077.627402881946</v>
+        <v>46077.79406954861</v>
       </c>
       <c r="C19" s="8">
-        <v>46093.7060909375</v>
+        <v>46093.87275760417</v>
       </c>
       <c r="D19" s="8">
-        <v>46132.66148358796</v>
+        <v>46132.82815025463</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>81</v>
@@ -2495,13 +2495,13 @@
         <v>83</v>
       </c>
       <c r="B20" s="5">
-        <v>46077.627403506944</v>
+        <v>46077.79407017361</v>
       </c>
       <c r="C20" s="5">
-        <v>46093.58544189815</v>
+        <v>46093.75210856482</v>
       </c>
       <c r="D20" s="5">
-        <v>46093.58546634259</v>
+        <v>46093.75213300926</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>84</v>
@@ -2560,13 +2560,13 @@
         <v>86</v>
       </c>
       <c r="B21" s="8">
-        <v>46077.62740315972</v>
+        <v>46077.794069826385</v>
       </c>
       <c r="C21" s="8">
-        <v>46093.585455266206</v>
+        <v>46093.75212193287</v>
       </c>
       <c r="D21" s="8">
-        <v>46093.58547449074</v>
+        <v>46093.75214115741</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>87</v>
@@ -2625,13 +2625,13 @@
         <v>89</v>
       </c>
       <c r="B22" s="5">
-        <v>46077.627404224535</v>
+        <v>46077.79407089121</v>
       </c>
       <c r="C22" s="5">
-        <v>46093.58563809028</v>
+        <v>46093.75230475694</v>
       </c>
       <c r="D22" s="5">
-        <v>46093.58565371528</v>
+        <v>46093.752320381944</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>90</v>
@@ -2690,13 +2690,13 @@
         <v>92</v>
       </c>
       <c r="B23" s="8">
-        <v>46077.627403900464</v>
+        <v>46077.79407056713</v>
       </c>
       <c r="C23" s="8">
-        <v>46093.706072175926</v>
+        <v>46093.87273884259</v>
       </c>
       <c r="D23" s="8">
-        <v>46093.70609091435</v>
+        <v>46093.87275758102</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>93</v>
@@ -2755,13 +2755,13 @@
         <v>95</v>
       </c>
       <c r="B24" s="5">
-        <v>46077.627401516205</v>
+        <v>46077.79406818287</v>
       </c>
       <c r="C24" s="5">
-        <v>46093.58568167824</v>
+        <v>46093.752348344904</v>
       </c>
       <c r="D24" s="5">
-        <v>46093.58569738426</v>
+        <v>46093.752364050924</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>96</v>
@@ -2820,13 +2820,13 @@
         <v>98</v>
       </c>
       <c r="B25" s="8">
-        <v>46078.4729491551</v>
+        <v>46078.639615821754</v>
       </c>
       <c r="C25" s="8">
-        <v>46093.58570607639</v>
+        <v>46093.75237274305</v>
       </c>
       <c r="D25" s="8">
-        <v>46093.58572271991</v>
+        <v>46093.75238938657</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>99</v>
@@ -2885,13 +2885,13 @@
         <v>101</v>
       </c>
       <c r="B26" s="5">
-        <v>46078.47300032407</v>
+        <v>46078.63966699074</v>
       </c>
       <c r="C26" s="5">
-        <v>46093.58588290509</v>
+        <v>46093.75254957176</v>
       </c>
       <c r="D26" s="5">
-        <v>46093.58590293981</v>
+        <v>46093.752569606484</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>102</v>
@@ -2950,13 +2950,13 @@
         <v>104</v>
       </c>
       <c r="B27" s="8">
-        <v>46077.62740185185</v>
+        <v>46077.79406851852</v>
       </c>
       <c r="C27" s="8">
-        <v>46175.413840775465</v>
+        <v>46175.58050744213</v>
       </c>
       <c r="D27" s="8">
-        <v>46196.65220835648</v>
+        <v>46196.81887502315</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>105</v>
@@ -3001,13 +3001,13 @@
         <v>108</v>
       </c>
       <c r="B28" s="5">
-        <v>46077.62740210648</v>
+        <v>46077.794068773146</v>
       </c>
       <c r="C28" s="5">
-        <v>46196.652190810186</v>
+        <v>46196.81885747685</v>
       </c>
       <c r="D28" s="5">
-        <v>46196.65219232639</v>
+        <v>46196.81885899305</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>109</v>
@@ -3066,13 +3066,13 @@
         <v>113</v>
       </c>
       <c r="B29" s="8">
-        <v>46077.62740236111</v>
+        <v>46077.794069027776</v>
       </c>
       <c r="C29" s="8">
-        <v>46094.559746493054</v>
+        <v>46094.72641315972</v>
       </c>
       <c r="D29" s="8">
-        <v>46094.55974833333</v>
+        <v>46094.726415</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>114</v>
@@ -3131,13 +3131,13 @@
         <v>118</v>
       </c>
       <c r="B30" s="5">
-        <v>46077.627402604165</v>
+        <v>46077.794069270836</v>
       </c>
       <c r="C30" s="5">
-        <v>46094.559799826384</v>
+        <v>46094.726466493055</v>
       </c>
       <c r="D30" s="5">
-        <v>46094.559801296295</v>
+        <v>46094.72646796296</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>119</v>
@@ -3196,13 +3196,13 @@
         <v>121</v>
       </c>
       <c r="B31" s="8">
-        <v>46077.62740287037</v>
+        <v>46077.794069537034</v>
       </c>
       <c r="C31" s="8">
-        <v>46174.472768541666</v>
+        <v>46174.63943520833</v>
       </c>
       <c r="D31" s="8">
-        <v>46181.528307939814</v>
+        <v>46181.69497460648</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>122</v>
@@ -3261,13 +3261,13 @@
         <v>124</v>
       </c>
       <c r="B32" s="5">
-        <v>46077.627403136576</v>
+        <v>46077.79406980324</v>
       </c>
       <c r="C32" s="5">
-        <v>46094.56096149306</v>
+        <v>46094.72762815972</v>
       </c>
       <c r="D32" s="5">
-        <v>46169.6622078588</v>
+        <v>46169.82887452546</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>125</v>
@@ -3326,13 +3326,13 @@
         <v>127</v>
       </c>
       <c r="B33" s="8">
-        <v>46077.62740341436</v>
+        <v>46077.794070081014</v>
       </c>
       <c r="C33" s="8">
-        <v>46174.47188952546</v>
+        <v>46174.638556192134</v>
       </c>
       <c r="D33" s="8">
-        <v>46174.47189153935</v>
+        <v>46174.63855820602</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>128</v>
@@ -3389,13 +3389,13 @@
         <v>130</v>
       </c>
       <c r="B34" s="5">
-        <v>46077.627403680555</v>
+        <v>46077.79407034723</v>
       </c>
       <c r="C34" s="5">
-        <v>46094.56312236111</v>
+        <v>46094.72978902778</v>
       </c>
       <c r="D34" s="5">
-        <v>46094.56313879629</v>
+        <v>46094.729805462965</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>131</v>
@@ -3454,13 +3454,13 @@
         <v>133</v>
       </c>
       <c r="B35" s="8">
-        <v>46077.62740395834</v>
+        <v>46077.794070625</v>
       </c>
       <c r="C35" s="8">
-        <v>46094.56209177083</v>
+        <v>46094.7287584375</v>
       </c>
       <c r="D35" s="8">
-        <v>46094.5620933912</v>
+        <v>46094.72876005787</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>134</v>
@@ -3519,13 +3519,13 @@
         <v>136</v>
       </c>
       <c r="B36" s="5">
-        <v>46077.627401342594</v>
+        <v>46077.79406800926</v>
       </c>
       <c r="C36" s="5">
-        <v>46094.56310604166</v>
+        <v>46094.729772708335</v>
       </c>
       <c r="D36" s="5">
-        <v>46094.56310759259</v>
+        <v>46094.729774259264</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>137</v>
@@ -3584,13 +3584,13 @@
         <v>139</v>
       </c>
       <c r="B37" s="8">
-        <v>46077.62740167824</v>
+        <v>46077.79406834491</v>
       </c>
       <c r="C37" s="8">
-        <v>46094.55852871528</v>
+        <v>46094.72519538194</v>
       </c>
       <c r="D37" s="8">
-        <v>46130.00231289351</v>
+        <v>46130.168979560185</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>140</v>
@@ -3649,13 +3649,13 @@
         <v>142</v>
       </c>
       <c r="B38" s="5">
-        <v>46077.62740193287</v>
+        <v>46077.79406859954</v>
       </c>
       <c r="C38" s="5">
-        <v>46094.55824585648</v>
+        <v>46094.72491252315</v>
       </c>
       <c r="D38" s="5">
-        <v>46094.55824805556</v>
+        <v>46094.72491472222</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>143</v>
@@ -3714,13 +3714,13 @@
         <v>145</v>
       </c>
       <c r="B39" s="8">
-        <v>46077.627402199076</v>
+        <v>46077.79406886574</v>
       </c>
       <c r="C39" s="8">
-        <v>46094.55846472223</v>
+        <v>46094.725131388885</v>
       </c>
       <c r="D39" s="8">
-        <v>46094.558466076385</v>
+        <v>46094.72513274306</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>146</v>
@@ -3779,13 +3779,13 @@
         <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46077.627402453705</v>
+        <v>46077.79406912037</v>
       </c>
       <c r="C40" s="5">
-        <v>46094.558513449076</v>
+        <v>46094.72518011574</v>
       </c>
       <c r="D40" s="5">
-        <v>46094.55851484954</v>
+        <v>46094.7251815162</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>149</v>
@@ -3844,13 +3844,13 @@
         <v>151</v>
       </c>
       <c r="B41" s="8">
-        <v>46077.62740268519</v>
+        <v>46077.79406935185</v>
       </c>
       <c r="C41" s="8">
-        <v>46094.571954722225</v>
+        <v>46094.73862138889</v>
       </c>
       <c r="D41" s="8">
-        <v>46100.721328287036</v>
+        <v>46100.88799495371</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>152</v>
@@ -3909,13 +3909,13 @@
         <v>156</v>
       </c>
       <c r="B42" s="5">
-        <v>46077.62740291667</v>
+        <v>46077.79406958334</v>
       </c>
       <c r="C42" s="5">
-        <v>46094.57047277778</v>
+        <v>46094.73713944445</v>
       </c>
       <c r="D42" s="5">
-        <v>46094.57155354167</v>
+        <v>46094.73822020833</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>97</v>
@@ -3974,13 +3974,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46077.627403148144</v>
+        <v>46077.794069814816</v>
       </c>
       <c r="C43" s="8">
-        <v>46094.57193980324</v>
+        <v>46094.73860646991</v>
       </c>
       <c r="D43" s="8">
-        <v>46094.57194121528</v>
+        <v>46094.73860788194</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -4039,13 +4039,13 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46078.473167627315</v>
+        <v>46078.63983429398</v>
       </c>
       <c r="C44" s="5">
-        <v>46099.68990657407</v>
+        <v>46099.856573240744</v>
       </c>
       <c r="D44" s="5">
-        <v>46099.68998267361</v>
+        <v>46099.856649340276</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4104,13 +4104,13 @@
         <v>164</v>
       </c>
       <c r="B45" s="8">
-        <v>46078.473232118056</v>
+        <v>46078.63989878472</v>
       </c>
       <c r="C45" s="8">
-        <v>46099.68980662037</v>
+        <v>46099.856473287036</v>
       </c>
       <c r="D45" s="8">
-        <v>46099.68980807871</v>
+        <v>46099.85647474537</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>165</v>
@@ -4159,13 +4159,13 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46078.473311319445</v>
+        <v>46078.63997798611</v>
       </c>
       <c r="C46" s="5">
-        <v>46099.68988975695</v>
+        <v>46099.85655642361</v>
       </c>
       <c r="D46" s="5">
-        <v>46099.689891284725</v>
+        <v>46099.85655795139</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4214,13 +4214,13 @@
         <v>170</v>
       </c>
       <c r="B47" s="8">
-        <v>46078.47114583333</v>
+        <v>46078.637812500005</v>
       </c>
       <c r="C47" s="8">
-        <v>46099.671767708336</v>
+        <v>46099.838434375</v>
       </c>
       <c r="D47" s="8">
-        <v>46121.03949925926</v>
+        <v>46121.20616592593</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>171</v>
@@ -4279,13 +4279,13 @@
         <v>175</v>
       </c>
       <c r="B48" s="5">
-        <v>46078.47124960648</v>
+        <v>46078.63791627315</v>
       </c>
       <c r="C48" s="5">
-        <v>46094.58716689815</v>
+        <v>46094.75383356481</v>
       </c>
       <c r="D48" s="5">
-        <v>46099.37121840278</v>
+        <v>46099.53788506944</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>103</v>
@@ -4340,13 +4340,13 @@
         <v>177</v>
       </c>
       <c r="B49" s="8">
-        <v>46078.471415949076</v>
+        <v>46078.63808261574</v>
       </c>
       <c r="C49" s="8">
-        <v>46099.67175158564</v>
+        <v>46099.838418252315</v>
       </c>
       <c r="D49" s="8">
-        <v>46099.67446230324</v>
+        <v>46099.84112896991</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>178</v>
@@ -4395,13 +4395,13 @@
         <v>181</v>
       </c>
       <c r="B50" s="5">
-        <v>46077.627403391205</v>
+        <v>46077.79407005787</v>
       </c>
       <c r="C50" s="5">
-        <v>46181.52820383102</v>
+        <v>46181.69487049768</v>
       </c>
       <c r="D50" s="5">
-        <v>46181.528219050924</v>
+        <v>46181.69488571759</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>182</v>
@@ -4448,13 +4448,13 @@
         <v>184</v>
       </c>
       <c r="B51" s="8">
-        <v>46077.62740362268</v>
+        <v>46077.794070289354</v>
       </c>
       <c r="C51" s="8">
-        <v>46093.59776341435</v>
+        <v>46093.76443008102</v>
       </c>
       <c r="D51" s="8">
-        <v>46093.59778137731</v>
+        <v>46093.76444804398</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>185</v>
@@ -4513,13 +4513,13 @@
         <v>189</v>
       </c>
       <c r="B52" s="5">
-        <v>46077.62740170139</v>
+        <v>46077.79406836806</v>
       </c>
       <c r="C52" s="5">
-        <v>46097.36665752315</v>
+        <v>46097.53332418982</v>
       </c>
       <c r="D52" s="5">
-        <v>46097.366677962964</v>
+        <v>46097.53334462963</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>190</v>
@@ -4578,13 +4578,13 @@
         <v>195</v>
       </c>
       <c r="B53" s="8">
-        <v>46092.31643899306</v>
+        <v>46092.48310565972</v>
       </c>
       <c r="C53" s="8">
-        <v>46097.36670182871</v>
+        <v>46097.533368495366</v>
       </c>
       <c r="D53" s="8">
-        <v>46097.36671966435</v>
+        <v>46097.53338633102</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>196</v>
@@ -4641,13 +4641,13 @@
         <v>198</v>
       </c>
       <c r="B54" s="5">
-        <v>46092.31653091435</v>
+        <v>46092.48319758102</v>
       </c>
       <c r="C54" s="5">
-        <v>46181.52670012732</v>
+        <v>46181.69336679398</v>
       </c>
       <c r="D54" s="5">
-        <v>46181.52824409722</v>
+        <v>46181.694910763894</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>199</v>
@@ -4706,13 +4706,13 @@
         <v>204</v>
       </c>
       <c r="B55" s="8">
-        <v>46079.44846875</v>
+        <v>46079.615135416665</v>
       </c>
       <c r="C55" s="8">
-        <v>46100.301554861115</v>
+        <v>46100.46822152778</v>
       </c>
       <c r="D55" s="8">
-        <v>46135.59274305556</v>
+        <v>46135.75940972222</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>205</v>
@@ -4755,13 +4755,13 @@
         <v>207</v>
       </c>
       <c r="B56" s="5">
-        <v>46078.582749016205</v>
+        <v>46078.74941568287</v>
       </c>
       <c r="C56" s="5">
-        <v>46100.301533391204</v>
+        <v>46100.46820005787</v>
       </c>
       <c r="D56" s="5">
-        <v>46122.0265565625</v>
+        <v>46122.193223229166</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>206</v>
@@ -4820,13 +4820,13 @@
         <v>211</v>
       </c>
       <c r="B57" s="8">
-        <v>46077.627403935185</v>
+        <v>46077.794070601856</v>
       </c>
       <c r="C57" s="8">
-        <v>46181.52990055556</v>
+        <v>46181.69656722222</v>
       </c>
       <c r="D57" s="8">
-        <v>46181.71383997685</v>
+        <v>46181.880506643516</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>212</v>
@@ -4869,13 +4869,13 @@
         <v>214</v>
       </c>
       <c r="B58" s="5">
-        <v>46077.627404224535</v>
+        <v>46077.79407089121</v>
       </c>
       <c r="C58" s="5">
-        <v>46099.44183902778</v>
+        <v>46099.60850569444</v>
       </c>
       <c r="D58" s="5">
-        <v>46099.441857638885</v>
+        <v>46099.60852430556</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>215</v>
@@ -4934,13 +4934,13 @@
         <v>219</v>
       </c>
       <c r="B59" s="8">
-        <v>46077.627401805556</v>
+        <v>46077.79406847223</v>
       </c>
       <c r="C59" s="8">
-        <v>46181.529883888885</v>
+        <v>46181.696550555556</v>
       </c>
       <c r="D59" s="8">
-        <v>46181.529900671296</v>
+        <v>46181.69656733796</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>57</v>
@@ -4999,13 +4999,13 @@
         <v>221</v>
       </c>
       <c r="B60" s="5">
-        <v>46077.6274021412</v>
+        <v>46077.79406880787</v>
       </c>
       <c r="C60" s="5">
-        <v>46099.44185101852</v>
+        <v>46099.608517685185</v>
       </c>
       <c r="D60" s="5">
-        <v>46107.98050693287</v>
+        <v>46108.14717359954</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>222</v>
@@ -5064,13 +5064,13 @@
         <v>224</v>
       </c>
       <c r="B61" s="8">
-        <v>46077.62740243056</v>
+        <v>46077.79406909722</v>
       </c>
       <c r="C61" s="8">
-        <v>46099.44188891204</v>
+        <v>46099.6085555787</v>
       </c>
       <c r="D61" s="8">
-        <v>46134.03879127315</v>
+        <v>46134.20545793981</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>225</v>
@@ -5129,13 +5129,13 @@
         <v>227</v>
       </c>
       <c r="B62" s="5">
-        <v>46078.47339827546</v>
+        <v>46078.64006494213</v>
       </c>
       <c r="C62" s="5">
-        <v>46099.69005751157</v>
+        <v>46099.856724178244</v>
       </c>
       <c r="D62" s="5">
-        <v>46099.69015126157</v>
+        <v>46099.856817928245</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>228</v>
@@ -5194,13 +5194,13 @@
         <v>230</v>
       </c>
       <c r="B63" s="8">
-        <v>46078.47246883102</v>
+        <v>46078.63913549768</v>
       </c>
       <c r="C63" s="8">
-        <v>46120.46123489583</v>
+        <v>46120.627901562504</v>
       </c>
       <c r="D63" s="8">
-        <v>46120.46125703704</v>
+        <v>46120.62792370371</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>231</v>
@@ -5259,13 +5259,13 @@
         <v>232</v>
       </c>
       <c r="B64" s="5">
-        <v>46077.62740271991</v>
+        <v>46077.794069386575</v>
       </c>
       <c r="C64" s="5">
-        <v>46181.52798491898</v>
+        <v>46181.69465158565</v>
       </c>
       <c r="D64" s="5">
-        <v>46197.41864</v>
+        <v>46197.58530666667</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>233</v>
@@ -5308,13 +5308,13 @@
         <v>235</v>
       </c>
       <c r="B65" s="8">
-        <v>46077.62740298611</v>
+        <v>46077.79406965278</v>
       </c>
       <c r="C65" s="8">
-        <v>46140.394836273146</v>
+        <v>46140.56150293982</v>
       </c>
       <c r="D65" s="8">
-        <v>46181.528036793985</v>
+        <v>46181.69470346065</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>236</v>
@@ -5373,13 +5373,13 @@
         <v>240</v>
       </c>
       <c r="B66" s="5">
-        <v>46077.62740324074</v>
+        <v>46077.79406990741</v>
       </c>
       <c r="C66" s="5">
-        <v>46181.52654994213</v>
+        <v>46181.69321660879</v>
       </c>
       <c r="D66" s="5">
-        <v>46181.52803732639</v>
+        <v>46181.69470399305</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>241</v>
@@ -5438,13 +5438,13 @@
         <v>244</v>
       </c>
       <c r="B67" s="8">
-        <v>46077.62740349537</v>
+        <v>46077.79407016204</v>
       </c>
       <c r="C67" s="8">
-        <v>46113.39420686342</v>
+        <v>46113.56087353009</v>
       </c>
       <c r="D67" s="8">
-        <v>46140.394845324074</v>
+        <v>46140.561511990745</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>245</v>
@@ -5503,13 +5503,13 @@
         <v>247</v>
       </c>
       <c r="B68" s="5">
-        <v>46077.62740376157</v>
+        <v>46077.79407042824</v>
       </c>
       <c r="C68" s="5">
-        <v>46181.526571759256</v>
+        <v>46181.69323842593</v>
       </c>
       <c r="D68" s="5">
-        <v>46181.52803785879</v>
+        <v>46181.694704525464</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>248</v>
@@ -5568,13 +5568,13 @@
         <v>250</v>
       </c>
       <c r="B69" s="8">
-        <v>46078.47347989584</v>
+        <v>46078.640146562495</v>
       </c>
       <c r="C69" s="8">
-        <v>46181.52658215278</v>
+        <v>46181.69324881944</v>
       </c>
       <c r="D69" s="8">
-        <v>46181.528038425924</v>
+        <v>46181.694705092596</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>229</v>
@@ -5633,13 +5633,13 @@
         <v>252</v>
       </c>
       <c r="B70" s="5">
-        <v>46077.62740403935</v>
+        <v>46077.79407070602</v>
       </c>
       <c r="C70" s="5">
-        <v>46181.526625081024</v>
+        <v>46181.69329174768</v>
       </c>
       <c r="D70" s="5">
-        <v>46181.528039004625</v>
+        <v>46181.694705671296</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>202</v>
@@ -5696,13 +5696,13 @@
         <v>255</v>
       </c>
       <c r="B71" s="8">
-        <v>46077.62740462963</v>
+        <v>46077.794071296295</v>
       </c>
       <c r="C71" s="8">
-        <v>46181.526995277774</v>
+        <v>46181.693661944446</v>
       </c>
       <c r="D71" s="8">
-        <v>46181.52803958333</v>
+        <v>46181.69470625</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>203</v>
@@ -5759,13 +5759,13 @@
         <v>257</v>
       </c>
       <c r="B72" s="5">
-        <v>46077.62740222222</v>
+        <v>46077.79406888889</v>
       </c>
       <c r="C72" s="5">
-        <v>46197.41998611111</v>
+        <v>46197.586652777776</v>
       </c>
       <c r="D72" s="5">
-        <v>46197.42000303241</v>
+        <v>46197.58666969907</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>258</v>
@@ -5812,13 +5812,13 @@
         <v>260</v>
       </c>
       <c r="B73" s="8">
-        <v>46077.62740253472</v>
+        <v>46077.79406920139</v>
       </c>
       <c r="C73" s="8">
-        <v>46197.41996670139</v>
+        <v>46197.58663336806</v>
       </c>
       <c r="D73" s="8">
-        <v>46197.41998619213</v>
+        <v>46197.586652858794</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5875,13 +5875,13 @@
         <v>266</v>
       </c>
       <c r="B74" s="5">
-        <v>46077.62740278935</v>
+        <v>46077.794069456024</v>
       </c>
       <c r="C74" s="5">
-        <v>46195.338891064814</v>
+        <v>46195.50555773148</v>
       </c>
       <c r="D74" s="5">
-        <v>46197.41998491898</v>
+        <v>46197.58665158565</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5938,13 +5938,13 @@
         <v>270</v>
       </c>
       <c r="B75" s="8">
-        <v>46077.62740304398</v>
+        <v>46077.79406971065</v>
       </c>
       <c r="C75" s="8">
-        <v>46195.3386822801</v>
+        <v>46195.50534894676</v>
       </c>
       <c r="D75" s="8">
-        <v>46195.33890541666</v>
+        <v>46195.50557208333</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>271</v>
@@ -6003,13 +6003,13 @@
         <v>275</v>
       </c>
       <c r="B76" s="5">
-        <v>46077.627403356484</v>
+        <v>46077.79407002315</v>
       </c>
       <c r="C76" s="5">
-        <v>46195.33873429398</v>
+        <v>46195.50540096065</v>
       </c>
       <c r="D76" s="5">
-        <v>46195.33874953704</v>
+        <v>46195.505416203705</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>276</v>
@@ -6066,11 +6066,11 @@
         <v>278</v>
       </c>
       <c r="B77" s="8">
-        <v>46077.62740362268</v>
+        <v>46077.794070289354</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46092.39547199074</v>
+        <v>46092.562138657406</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>279</v>
@@ -6113,11 +6113,11 @@
         <v>281</v>
       </c>
       <c r="B78" s="5">
-        <v>46077.62740391203</v>
+        <v>46077.794070578704</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46195.33875318287</v>
+        <v>46195.505419849535</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>282</v>
@@ -6176,11 +6176,11 @@
         <v>285</v>
       </c>
       <c r="B79" s="8">
-        <v>46077.627404189814</v>
+        <v>46077.794070856486</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46195.33875326389</v>
+        <v>46195.50541993056</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>286</v>
@@ -6239,11 +6239,11 @@
         <v>288</v>
       </c>
       <c r="B80" s="5">
-        <v>46092.37582547453</v>
+        <v>46092.542492141205</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46092.39547261574</v>
+        <v>46092.56213928241</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>289</v>
@@ -6292,11 +6292,11 @@
         <v>291</v>
       </c>
       <c r="B81" s="8">
-        <v>46092.37586482639</v>
+        <v>46092.542531493054</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46195.33875447916</v>
+        <v>46195.505421145834</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>292</v>
@@ -6355,11 +6355,11 @@
         <v>294</v>
       </c>
       <c r="B82" s="5">
-        <v>46092.376002453704</v>
+        <v>46092.542669120376</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46185.01497164352</v>
+        <v>46185.18163831018</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>295</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-15 21:14 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="295">
   <si>
     <t>50001415-ZITRON PERU METRO DE LIMA  E05</t>
   </si>
@@ -722,9 +722,6 @@
   </si>
   <si>
     <t>Revestimiento</t>
-  </si>
-  <si>
-    <t>benjamin.bustos@zitron.com</t>
   </si>
   <si>
     <t>Montaje:,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensores</t>
@@ -5323,11 +5320,9 @@
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="H65" s="9" t="s">
-        <v>237</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H65" s="9"/>
       <c r="I65" s="8">
         <v>46122</v>
       </c>
@@ -5350,7 +5345,7 @@
         <v>206</v>
       </c>
       <c r="P65" s="9" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="Q65" s="8">
         <v>46122</v>
@@ -5362,7 +5357,7 @@
         <v>1</v>
       </c>
       <c r="T65" s="12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="U65" s="11" t="s">
         <v>33</v>
@@ -5370,7 +5365,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B66" s="5">
         <v>46077.79406990741</v>
@@ -5382,17 +5377,15 @@
         <v>46181.69470399305</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="H66" s="6" t="s">
-        <v>237</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H66" s="6"/>
       <c r="I66" s="5">
         <v>46142</v>
       </c>
@@ -5412,10 +5405,10 @@
         <v>233</v>
       </c>
       <c r="O66" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="P66" s="6" t="s">
         <v>242</v>
-      </c>
-      <c r="P66" s="6" t="s">
-        <v>243</v>
       </c>
       <c r="Q66" s="5">
         <v>46142</v>
@@ -5427,7 +5420,7 @@
         <v>1</v>
       </c>
       <c r="T66" s="12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="U66" s="11" t="s">
         <v>33</v>
@@ -5435,7 +5428,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B67" s="8">
         <v>46077.79407016204</v>
@@ -5447,17 +5440,15 @@
         <v>46140.561511990745</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="H67" s="9" t="s">
-        <v>237</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H67" s="9"/>
       <c r="I67" s="8">
         <v>46147</v>
       </c>
@@ -5477,10 +5468,10 @@
         <v>233</v>
       </c>
       <c r="O67" s="9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="P67" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="Q67" s="8">
         <v>46147</v>
@@ -5500,7 +5491,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B68" s="5">
         <v>46077.79407042824</v>
@@ -5512,17 +5503,15 @@
         <v>46181.694704525464</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>237</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H68" s="6"/>
       <c r="I68" s="5">
         <v>46149</v>
       </c>
@@ -5542,10 +5531,10 @@
         <v>233</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="Q68" s="5">
         <v>46149</v>
@@ -5565,7 +5554,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B69" s="8">
         <v>46078.640146562495</v>
@@ -5583,11 +5572,9 @@
         <v>26</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="H69" s="9" t="s">
-        <v>237</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H69" s="9"/>
       <c r="I69" s="8">
         <v>46150</v>
       </c>
@@ -5607,10 +5594,10 @@
         <v>233</v>
       </c>
       <c r="O69" s="9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="P69" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="Q69" s="8">
         <v>46153</v>
@@ -5630,7 +5617,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B70" s="5">
         <v>46077.79407070602</v>
@@ -5648,11 +5635,9 @@
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>237</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H70" s="6"/>
       <c r="I70" s="6"/>
       <c r="J70" s="5">
         <v>46155</v>
@@ -5670,10 +5655,10 @@
         <v>233</v>
       </c>
       <c r="O70" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="P70" s="6" t="s">
         <v>253</v>
-      </c>
-      <c r="P70" s="6" t="s">
-        <v>254</v>
       </c>
       <c r="Q70" s="5">
         <v>46155</v>
@@ -5693,7 +5678,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B71" s="8">
         <v>46077.794071296295</v>
@@ -5711,11 +5696,9 @@
         <v>26</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="H71" s="9" t="s">
-        <v>237</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H71" s="9"/>
       <c r="I71" s="9"/>
       <c r="J71" s="8">
         <v>46157</v>
@@ -5736,7 +5719,7 @@
         <v>199</v>
       </c>
       <c r="P71" s="9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="Q71" s="8">
         <v>46157</v>
@@ -5756,7 +5739,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B72" s="5">
         <v>46077.79406888889</v>
@@ -5768,7 +5751,7 @@
         <v>46197.58666969907</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>25</v>
@@ -5792,7 +5775,7 @@
         <v>26</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>26</v>
@@ -5809,7 +5792,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B73" s="8">
         <v>46077.79406920139</v>
@@ -5821,16 +5804,16 @@
         <v>46197.586652858794</v>
       </c>
       <c r="E73" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="F73" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G73" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="F73" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G73" s="9" t="s">
+      <c r="H73" s="9" t="s">
         <v>262</v>
-      </c>
-      <c r="H73" s="9" t="s">
-        <v>263</v>
       </c>
       <c r="I73" s="9"/>
       <c r="J73" s="8">
@@ -5846,13 +5829,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O73" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="P73" s="9" t="s">
         <v>264</v>
-      </c>
-      <c r="P73" s="9" t="s">
-        <v>265</v>
       </c>
       <c r="Q73" s="8">
         <v>46160</v>
@@ -5872,7 +5855,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B74" s="5">
         <v>46077.794069456024</v>
@@ -5884,17 +5867,15 @@
         <v>46197.58665158565</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>237</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H74" s="6"/>
       <c r="I74" s="6"/>
       <c r="J74" s="5">
         <v>46161</v>
@@ -5909,13 +5890,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O74" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="P74" s="6" t="s">
         <v>268</v>
-      </c>
-      <c r="P74" s="6" t="s">
-        <v>269</v>
       </c>
       <c r="Q74" s="5">
         <v>46161</v>
@@ -5935,7 +5916,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B75" s="8">
         <v>46077.79406971065</v>
@@ -5947,16 +5928,16 @@
         <v>46195.50557208333</v>
       </c>
       <c r="E75" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="F75" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G75" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="F75" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G75" s="9" t="s">
+      <c r="H75" s="9" t="s">
         <v>272</v>
-      </c>
-      <c r="H75" s="9" t="s">
-        <v>273</v>
       </c>
       <c r="I75" s="8">
         <v>46162</v>
@@ -5974,13 +5955,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="Q75" s="8">
         <v>46162</v>
@@ -6000,7 +5981,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B76" s="5">
         <v>46077.79407002315</v>
@@ -6012,16 +5993,16 @@
         <v>46195.505416203705</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="H76" s="6" t="s">
         <v>272</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>273</v>
       </c>
       <c r="I76" s="6"/>
       <c r="J76" s="5">
@@ -6037,13 +6018,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="Q76" s="5">
         <v>46164</v>
@@ -6063,7 +6044,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B77" s="8">
         <v>46077.794070289354</v>
@@ -6073,7 +6054,7 @@
         <v>46092.562138657406</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>25</v>
@@ -6097,7 +6078,7 @@
         <v>26</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="P77" s="9" t="s">
         <v>26</v>
@@ -6110,7 +6091,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B78" s="5">
         <v>46077.794070578704</v>
@@ -6120,16 +6101,16 @@
         <v>46195.505419849535</v>
       </c>
       <c r="E78" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G78" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="F78" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G78" s="6" t="s">
+      <c r="H78" s="6" t="s">
         <v>283</v>
-      </c>
-      <c r="H78" s="6" t="s">
-        <v>284</v>
       </c>
       <c r="I78" s="5">
         <v>46167</v>
@@ -6147,13 +6128,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Q78" s="5">
         <v>46167</v>
@@ -6173,7 +6154,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B79" s="8">
         <v>46077.794070856486</v>
@@ -6183,16 +6164,16 @@
         <v>46195.50541993056</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="H79" s="9" t="s">
         <v>283</v>
-      </c>
-      <c r="H79" s="9" t="s">
-        <v>284</v>
       </c>
       <c r="I79" s="8">
         <v>46167</v>
@@ -6210,13 +6191,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Q79" s="8">
         <v>46167</v>
@@ -6236,7 +6217,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B80" s="5">
         <v>46092.542492141205</v>
@@ -6246,7 +6227,7 @@
         <v>46092.56213928241</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>25</v>
@@ -6270,7 +6251,7 @@
         <v>26</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>26</v>
@@ -6289,7 +6270,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B81" s="8">
         <v>46092.542531493054</v>
@@ -6299,7 +6280,7 @@
         <v>46195.505421145834</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
@@ -6326,13 +6307,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="9" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="Q81" s="8">
         <v>46167</v>
@@ -6352,7 +6333,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B82" s="5">
         <v>46092.542669120376</v>
@@ -6362,7 +6343,7 @@
         <v>46185.18163831018</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
@@ -6389,13 +6370,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="Q82" s="5">
         <v>46176</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-20 15:15 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="296">
   <si>
     <t>50001415-ZITRON PERU METRO DE LIMA  E05</t>
   </si>
@@ -722,6 +722,9 @@
   </si>
   <si>
     <t>Revestimiento</t>
+  </si>
+  <si>
+    <t>nespinoza@zitron.com</t>
   </si>
   <si>
     <t>Montaje:,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensores</t>
@@ -5311,7 +5314,7 @@
         <v>46140.56150293982</v>
       </c>
       <c r="D65" s="8">
-        <v>46181.69470346065</v>
+        <v>46223.55574784722</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>236</v>
@@ -5320,9 +5323,11 @@
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H65" s="9"/>
+        <v>237</v>
+      </c>
+      <c r="H65" s="9" t="s">
+        <v>237</v>
+      </c>
       <c r="I65" s="8">
         <v>46122</v>
       </c>
@@ -5345,7 +5350,7 @@
         <v>206</v>
       </c>
       <c r="P65" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="Q65" s="8">
         <v>46122</v>
@@ -5357,7 +5362,7 @@
         <v>1</v>
       </c>
       <c r="T65" s="12" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="U65" s="11" t="s">
         <v>33</v>
@@ -5365,7 +5370,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B66" s="5">
         <v>46077.79406990741</v>
@@ -5374,18 +5379,20 @@
         <v>46181.69321660879</v>
       </c>
       <c r="D66" s="5">
-        <v>46181.69470399305</v>
+        <v>46223.55598479167</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H66" s="6"/>
+        <v>237</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>237</v>
+      </c>
       <c r="I66" s="5">
         <v>46142</v>
       </c>
@@ -5405,10 +5412,10 @@
         <v>233</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="P66" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="Q66" s="5">
         <v>46142</v>
@@ -5420,7 +5427,7 @@
         <v>1</v>
       </c>
       <c r="T66" s="12" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="U66" s="11" t="s">
         <v>33</v>
@@ -5428,7 +5435,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B67" s="8">
         <v>46077.79407016204</v>
@@ -5440,7 +5447,7 @@
         <v>46140.561511990745</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>26</v>
@@ -5468,10 +5475,10 @@
         <v>233</v>
       </c>
       <c r="O67" s="9" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="P67" s="9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="Q67" s="8">
         <v>46147</v>
@@ -5491,7 +5498,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B68" s="5">
         <v>46077.79407042824</v>
@@ -5503,7 +5510,7 @@
         <v>46181.694704525464</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
@@ -5531,10 +5538,10 @@
         <v>233</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="Q68" s="5">
         <v>46149</v>
@@ -5554,7 +5561,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B69" s="8">
         <v>46078.640146562495</v>
@@ -5563,7 +5570,7 @@
         <v>46181.69324881944</v>
       </c>
       <c r="D69" s="8">
-        <v>46181.694705092596</v>
+        <v>46223.556461643515</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>229</v>
@@ -5572,9 +5579,11 @@
         <v>26</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H69" s="9"/>
+        <v>237</v>
+      </c>
+      <c r="H69" s="9" t="s">
+        <v>237</v>
+      </c>
       <c r="I69" s="8">
         <v>46150</v>
       </c>
@@ -5594,10 +5603,10 @@
         <v>233</v>
       </c>
       <c r="O69" s="9" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="P69" s="9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="Q69" s="8">
         <v>46153</v>
@@ -5617,7 +5626,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B70" s="5">
         <v>46077.79407070602</v>
@@ -5626,7 +5635,7 @@
         <v>46181.69329174768</v>
       </c>
       <c r="D70" s="5">
-        <v>46181.694705671296</v>
+        <v>46223.55656295139</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>202</v>
@@ -5635,9 +5644,11 @@
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H70" s="6"/>
+        <v>237</v>
+      </c>
+      <c r="H70" s="6" t="s">
+        <v>237</v>
+      </c>
       <c r="I70" s="6"/>
       <c r="J70" s="5">
         <v>46155</v>
@@ -5655,10 +5666,10 @@
         <v>233</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="P70" s="6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="Q70" s="5">
         <v>46155</v>
@@ -5678,7 +5689,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B71" s="8">
         <v>46077.794071296295</v>
@@ -5687,7 +5698,7 @@
         <v>46181.693661944446</v>
       </c>
       <c r="D71" s="8">
-        <v>46181.69470625</v>
+        <v>46223.5566908912</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>203</v>
@@ -5696,9 +5707,11 @@
         <v>26</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H71" s="9"/>
+        <v>237</v>
+      </c>
+      <c r="H71" s="9" t="s">
+        <v>237</v>
+      </c>
       <c r="I71" s="9"/>
       <c r="J71" s="8">
         <v>46157</v>
@@ -5719,7 +5732,7 @@
         <v>199</v>
       </c>
       <c r="P71" s="9" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="Q71" s="8">
         <v>46157</v>
@@ -5739,7 +5752,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B72" s="5">
         <v>46077.79406888889</v>
@@ -5751,7 +5764,7 @@
         <v>46197.58666969907</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>25</v>
@@ -5775,7 +5788,7 @@
         <v>26</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>26</v>
@@ -5792,7 +5805,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B73" s="8">
         <v>46077.79406920139</v>
@@ -5804,16 +5817,16 @@
         <v>46197.586652858794</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I73" s="9"/>
       <c r="J73" s="8">
@@ -5829,13 +5842,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="9" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="O73" s="9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="P73" s="9" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q73" s="8">
         <v>46160</v>
@@ -5855,7 +5868,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B74" s="5">
         <v>46077.794069456024</v>
@@ -5867,7 +5880,7 @@
         <v>46197.58665158565</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
@@ -5890,13 +5903,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="Q74" s="5">
         <v>46161</v>
@@ -5916,7 +5929,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B75" s="8">
         <v>46077.79406971065</v>
@@ -5928,16 +5941,16 @@
         <v>46195.50557208333</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I75" s="8">
         <v>46162</v>
@@ -5955,13 +5968,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q75" s="8">
         <v>46162</v>
@@ -5981,7 +5994,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B76" s="5">
         <v>46077.79407002315</v>
@@ -5993,16 +6006,16 @@
         <v>46195.505416203705</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I76" s="6"/>
       <c r="J76" s="5">
@@ -6018,13 +6031,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="Q76" s="5">
         <v>46164</v>
@@ -6044,7 +6057,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B77" s="8">
         <v>46077.794070289354</v>
@@ -6054,7 +6067,7 @@
         <v>46092.562138657406</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>25</v>
@@ -6078,7 +6091,7 @@
         <v>26</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="P77" s="9" t="s">
         <v>26</v>
@@ -6091,7 +6104,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B78" s="5">
         <v>46077.794070578704</v>
@@ -6101,16 +6114,16 @@
         <v>46195.505419849535</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I78" s="5">
         <v>46167</v>
@@ -6128,13 +6141,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="Q78" s="5">
         <v>46167</v>
@@ -6154,7 +6167,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B79" s="8">
         <v>46077.794070856486</v>
@@ -6164,16 +6177,16 @@
         <v>46195.50541993056</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="9" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H79" s="9" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I79" s="8">
         <v>46167</v>
@@ -6191,13 +6204,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="Q79" s="8">
         <v>46167</v>
@@ -6217,7 +6230,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B80" s="5">
         <v>46092.542492141205</v>
@@ -6227,7 +6240,7 @@
         <v>46092.56213928241</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>25</v>
@@ -6251,7 +6264,7 @@
         <v>26</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>26</v>
@@ -6270,7 +6283,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B81" s="8">
         <v>46092.542531493054</v>
@@ -6280,7 +6293,7 @@
         <v>46195.505421145834</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
@@ -6307,13 +6320,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="9" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="Q81" s="8">
         <v>46167</v>
@@ -6333,7 +6346,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B82" s="5">
         <v>46092.542669120376</v>
@@ -6343,7 +6356,7 @@
         <v>46185.18163831018</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
@@ -6370,13 +6383,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="Q82" s="5">
         <v>46176</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-20 19:58 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="296">
   <si>
     <t>50001415-ZITRON PERU METRO DE LIMA  E05</t>
   </si>
@@ -5444,7 +5444,7 @@
         <v>46113.56087353009</v>
       </c>
       <c r="D67" s="8">
-        <v>46140.561511990745</v>
+        <v>46223.818650381945</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>245</v>
@@ -5453,9 +5453,11 @@
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H67" s="9"/>
+        <v>237</v>
+      </c>
+      <c r="H67" s="9" t="s">
+        <v>237</v>
+      </c>
       <c r="I67" s="8">
         <v>46147</v>
       </c>
@@ -5507,7 +5509,7 @@
         <v>46181.69323842593</v>
       </c>
       <c r="D68" s="5">
-        <v>46181.694704525464</v>
+        <v>46223.81864615741</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>248</v>
@@ -5516,9 +5518,11 @@
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H68" s="6"/>
+        <v>237</v>
+      </c>
+      <c r="H68" s="6" t="s">
+        <v>237</v>
+      </c>
       <c r="I68" s="5">
         <v>46149</v>
       </c>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-20 21:25 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="296">
   <si>
     <t>50001415-ZITRON PERU METRO DE LIMA  E05</t>
   </si>
@@ -5881,7 +5881,7 @@
         <v>46195.50555773148</v>
       </c>
       <c r="D74" s="5">
-        <v>46197.58665158565</v>
+        <v>46223.83366560185</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>
@@ -5890,9 +5890,11 @@
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H74" s="6"/>
+        <v>237</v>
+      </c>
+      <c r="H74" s="6" t="s">
+        <v>237</v>
+      </c>
       <c r="I74" s="6"/>
       <c r="J74" s="5">
         <v>46161</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-22 21:23 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="297">
   <si>
     <t>50001415-ZITRON PERU METRO DE LIMA  E05</t>
   </si>
@@ -722,6 +722,9 @@
   </si>
   <si>
     <t>Revestimiento</t>
+  </si>
+  <si>
+    <t>NATALYA ESPINOZA</t>
   </si>
   <si>
     <t>nespinoza@zitron.com</t>
@@ -5326,7 +5329,7 @@
         <v>237</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I65" s="8">
         <v>46122</v>
@@ -5350,7 +5353,7 @@
         <v>206</v>
       </c>
       <c r="P65" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="Q65" s="8">
         <v>46122</v>
@@ -5362,7 +5365,7 @@
         <v>1</v>
       </c>
       <c r="T65" s="12" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="U65" s="11" t="s">
         <v>33</v>
@@ -5370,7 +5373,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B66" s="5">
         <v>46077.79406990741</v>
@@ -5382,7 +5385,7 @@
         <v>46223.55598479167</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
@@ -5391,7 +5394,7 @@
         <v>237</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I66" s="5">
         <v>46142</v>
@@ -5412,10 +5415,10 @@
         <v>233</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P66" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Q66" s="5">
         <v>46142</v>
@@ -5427,7 +5430,7 @@
         <v>1</v>
       </c>
       <c r="T66" s="12" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="U66" s="11" t="s">
         <v>33</v>
@@ -5435,7 +5438,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B67" s="8">
         <v>46077.79407016204</v>
@@ -5447,7 +5450,7 @@
         <v>46223.818650381945</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>26</v>
@@ -5456,7 +5459,7 @@
         <v>237</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I67" s="8">
         <v>46147</v>
@@ -5477,10 +5480,10 @@
         <v>233</v>
       </c>
       <c r="O67" s="9" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="P67" s="9" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Q67" s="8">
         <v>46147</v>
@@ -5500,7 +5503,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B68" s="5">
         <v>46077.79407042824</v>
@@ -5512,7 +5515,7 @@
         <v>46223.81864615741</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
@@ -5521,7 +5524,7 @@
         <v>237</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I68" s="5">
         <v>46149</v>
@@ -5542,10 +5545,10 @@
         <v>233</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Q68" s="5">
         <v>46149</v>
@@ -5565,7 +5568,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B69" s="8">
         <v>46078.640146562495</v>
@@ -5586,7 +5589,7 @@
         <v>237</v>
       </c>
       <c r="H69" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I69" s="8">
         <v>46150</v>
@@ -5607,10 +5610,10 @@
         <v>233</v>
       </c>
       <c r="O69" s="9" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="P69" s="9" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Q69" s="8">
         <v>46153</v>
@@ -5630,7 +5633,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B70" s="5">
         <v>46077.79407070602</v>
@@ -5651,7 +5654,7 @@
         <v>237</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I70" s="6"/>
       <c r="J70" s="5">
@@ -5670,10 +5673,10 @@
         <v>233</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="P70" s="6" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="Q70" s="5">
         <v>46155</v>
@@ -5693,7 +5696,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B71" s="8">
         <v>46077.794071296295</v>
@@ -5714,7 +5717,7 @@
         <v>237</v>
       </c>
       <c r="H71" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I71" s="9"/>
       <c r="J71" s="8">
@@ -5736,7 +5739,7 @@
         <v>199</v>
       </c>
       <c r="P71" s="9" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="Q71" s="8">
         <v>46157</v>
@@ -5756,7 +5759,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B72" s="5">
         <v>46077.79406888889</v>
@@ -5768,7 +5771,7 @@
         <v>46197.58666969907</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>25</v>
@@ -5792,7 +5795,7 @@
         <v>26</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>26</v>
@@ -5809,7 +5812,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B73" s="8">
         <v>46077.79406920139</v>
@@ -5821,16 +5824,16 @@
         <v>46197.586652858794</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="I73" s="9"/>
       <c r="J73" s="8">
@@ -5846,13 +5849,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="9" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="O73" s="9" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="P73" s="9" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Q73" s="8">
         <v>46160</v>
@@ -5872,7 +5875,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B74" s="5">
         <v>46077.794069456024</v>
@@ -5884,7 +5887,7 @@
         <v>46223.83366560185</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
@@ -5893,7 +5896,7 @@
         <v>237</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I74" s="6"/>
       <c r="J74" s="5">
@@ -5909,13 +5912,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q74" s="5">
         <v>46161</v>
@@ -5935,7 +5938,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B75" s="8">
         <v>46077.79406971065</v>
@@ -5947,16 +5950,16 @@
         <v>46195.50557208333</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="I75" s="8">
         <v>46162</v>
@@ -5974,13 +5977,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Q75" s="8">
         <v>46162</v>
@@ -6000,7 +6003,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B76" s="5">
         <v>46077.79407002315</v>
@@ -6012,16 +6015,16 @@
         <v>46195.505416203705</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="I76" s="6"/>
       <c r="J76" s="5">
@@ -6037,13 +6040,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="Q76" s="5">
         <v>46164</v>
@@ -6063,7 +6066,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B77" s="8">
         <v>46077.794070289354</v>
@@ -6073,7 +6076,7 @@
         <v>46092.562138657406</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>25</v>
@@ -6097,7 +6100,7 @@
         <v>26</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="P77" s="9" t="s">
         <v>26</v>
@@ -6110,7 +6113,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B78" s="5">
         <v>46077.794070578704</v>
@@ -6120,16 +6123,16 @@
         <v>46195.505419849535</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="I78" s="5">
         <v>46167</v>
@@ -6147,13 +6150,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="Q78" s="5">
         <v>46167</v>
@@ -6173,7 +6176,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B79" s="8">
         <v>46077.794070856486</v>
@@ -6183,16 +6186,16 @@
         <v>46195.50541993056</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="9" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="H79" s="9" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="I79" s="8">
         <v>46167</v>
@@ -6210,13 +6213,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="Q79" s="8">
         <v>46167</v>
@@ -6236,7 +6239,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B80" s="5">
         <v>46092.542492141205</v>
@@ -6246,7 +6249,7 @@
         <v>46092.56213928241</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>25</v>
@@ -6270,7 +6273,7 @@
         <v>26</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>26</v>
@@ -6289,7 +6292,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B81" s="8">
         <v>46092.542531493054</v>
@@ -6299,7 +6302,7 @@
         <v>46195.505421145834</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
@@ -6326,13 +6329,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="9" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="Q81" s="8">
         <v>46167</v>
@@ -6352,7 +6355,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B82" s="5">
         <v>46092.542669120376</v>
@@ -6362,7 +6365,7 @@
         <v>46185.18163831018</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
@@ -6389,13 +6392,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="Q82" s="5">
         <v>46176</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-27 15:49 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -1898,7 +1898,7 @@
         <v>46196.78443082176</v>
       </c>
       <c r="D10" s="5">
-        <v>46196.78444497685</v>
+        <v>46228.631497696755</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -2455,7 +2455,7 @@
         <v>46093.87275760417</v>
       </c>
       <c r="D19" s="8">
-        <v>46132.82815025463</v>
+        <v>46229.69259979167</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>81</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-08-03 13:27 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -5884,7 +5884,7 @@
         <v>46195.50555773148</v>
       </c>
       <c r="D74" s="5">
-        <v>46223.83366560185</v>
+        <v>46237.516126030096</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>268</v>
@@ -5932,8 +5932,8 @@
       <c r="T74" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U74" s="12" t="s">
-        <v>107</v>
+      <c r="U74" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>46195.50534894676</v>
       </c>
       <c r="D75" s="8">
-        <v>46195.50557208333</v>
+        <v>46237.516144293986</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>272</v>
@@ -5997,8 +5997,8 @@
       <c r="T75" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U75" s="12" t="s">
-        <v>107</v>
+      <c r="U75" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-08-06 19:18 UTC
</commit_message>
<xml_diff>
--- a/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
+++ b/data/50001415 - ZITRON PERU METRO LIMA E05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="289">
   <si>
     <t>50001415-ZITRON PERU METRO DE LIMA  E05</t>
   </si>
@@ -847,7 +847,7 @@
     <t>Despacho</t>
   </si>
   <si>
-    <t>Logistica:,Gestion,Costos,Instalación Componentes</t>
+    <t>Logistica:,Gestion,Costos</t>
   </si>
   <si>
     <t>1213425187675737</t>
@@ -878,30 +878,6 @@
   </si>
   <si>
     <t>Despacho,Analisis de costeo</t>
-  </si>
-  <si>
-    <t>1213600211816618</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puesta en marcha </t>
-  </si>
-  <si>
-    <t>Instalación Componentes,Pruebas instalacion componentes</t>
-  </si>
-  <si>
-    <t>1213600211816620</t>
-  </si>
-  <si>
-    <t>Instalación Componentes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pruebas instalacion componentes,Puesta en marcha </t>
-  </si>
-  <si>
-    <t>1213600211816622</t>
-  </si>
-  <si>
-    <t>Pruebas instalacion componentes</t>
   </si>
 </sst>
 </file>
@@ -1425,7 +1401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U82"/>
+  <dimension ref="A1:U79"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -6012,7 +5988,7 @@
         <v>46195.50540096065</v>
       </c>
       <c r="D76" s="5">
-        <v>46195.505416203705</v>
+        <v>46240.70847309028</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>277</v>
@@ -6071,9 +6047,11 @@
       <c r="B77" s="8">
         <v>46077.794070289354</v>
       </c>
-      <c r="C77" s="9"/>
+      <c r="C77" s="8">
+        <v>46240.706420208335</v>
+      </c>
       <c r="D77" s="8">
-        <v>46092.562138657406</v>
+        <v>46240.70643387732</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>280</v>
@@ -6107,9 +6085,13 @@
       </c>
       <c r="Q77" s="9"/>
       <c r="R77" s="9"/>
-      <c r="S77" s="9"/>
+      <c r="S77" s="9">
+        <v>1</v>
+      </c>
       <c r="T77" s="9"/>
-      <c r="U77" s="9"/>
+      <c r="U77" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
@@ -6118,9 +6100,11 @@
       <c r="B78" s="5">
         <v>46077.794070578704</v>
       </c>
-      <c r="C78" s="6"/>
+      <c r="C78" s="5">
+        <v>46240.70640105324</v>
+      </c>
       <c r="D78" s="5">
-        <v>46195.505419849535</v>
+        <v>46240.70642094908</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>283</v>
@@ -6165,13 +6149,13 @@
         <v>46175</v>
       </c>
       <c r="S78" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T78" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U78" s="12" t="s">
-        <v>107</v>
+      <c r="U78" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
@@ -6181,9 +6165,11 @@
       <c r="B79" s="8">
         <v>46077.794070856486</v>
       </c>
-      <c r="C79" s="9"/>
+      <c r="C79" s="8">
+        <v>46240.70640920139</v>
+      </c>
       <c r="D79" s="8">
-        <v>46195.50541993056</v>
+        <v>46240.70642696759</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>287</v>
@@ -6228,192 +6214,13 @@
         <v>46175</v>
       </c>
       <c r="S79" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T79" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U79" s="12" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A80" s="4" t="s">
-        <v>289</v>
-      </c>
-      <c r="B80" s="5">
-        <v>46092.542492141205</v>
-      </c>
-      <c r="C80" s="6"/>
-      <c r="D80" s="5">
-        <v>46092.56213928241</v>
-      </c>
-      <c r="E80" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="F80" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G80" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H80" s="6"/>
-      <c r="I80" s="6"/>
-      <c r="J80" s="6"/>
-      <c r="K80" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L80" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M80" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="N80" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="O80" s="6" t="s">
-        <v>291</v>
-      </c>
-      <c r="P80" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q80" s="6"/>
-      <c r="R80" s="6"/>
-      <c r="S80" s="6">
-        <v>0</v>
-      </c>
-      <c r="T80" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="U80" s="10" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="81" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A81" s="7" t="s">
-        <v>292</v>
-      </c>
-      <c r="B81" s="8">
-        <v>46092.542531493054</v>
-      </c>
-      <c r="C81" s="9"/>
-      <c r="D81" s="8">
-        <v>46195.505421145834</v>
-      </c>
-      <c r="E81" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="F81" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G81" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="H81" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="I81" s="8">
-        <v>46167</v>
-      </c>
-      <c r="J81" s="8">
-        <v>46175</v>
-      </c>
-      <c r="K81" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L81" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M81" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N81" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="O81" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="P81" s="9" t="s">
-        <v>294</v>
-      </c>
-      <c r="Q81" s="8">
-        <v>46167</v>
-      </c>
-      <c r="R81" s="8">
-        <v>46175</v>
-      </c>
-      <c r="S81" s="9">
-        <v>0</v>
-      </c>
-      <c r="T81" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="U81" s="12" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="82" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A82" s="4" t="s">
-        <v>295</v>
-      </c>
-      <c r="B82" s="5">
-        <v>46092.542669120376</v>
-      </c>
-      <c r="C82" s="6"/>
-      <c r="D82" s="5">
-        <v>46185.18163831018</v>
-      </c>
-      <c r="E82" s="6" t="s">
-        <v>296</v>
-      </c>
-      <c r="F82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G82" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="H82" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="I82" s="5">
-        <v>46176</v>
-      </c>
-      <c r="J82" s="5">
-        <v>46184</v>
-      </c>
-      <c r="K82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N82" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="O82" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="P82" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="Q82" s="5">
-        <v>46176</v>
-      </c>
-      <c r="R82" s="5">
-        <v>46184</v>
-      </c>
-      <c r="S82" s="6">
-        <v>0</v>
-      </c>
-      <c r="T82" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="U82" s="10" t="s">
-        <v>117</v>
+      <c r="U79" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>